<commit_message>
fix: purge 44 adware restream channels from 107.150.60.122
</commit_message>
<xml_diff>
--- a/channels_overview.xlsx
+++ b/channels_overview.xlsx
@@ -1279,7 +1279,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
@@ -1294,11 +1294,11 @@
         </is>
       </c>
       <c r="B4" s="7" t="n">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>东方卫视HD、兵团卫视、大湾区卫视、天津卫视HD</t>
+          <t>兵团卫视、大湾区卫视、山东教育卫视、广东卫视</t>
         </is>
       </c>
     </row>
@@ -1594,7 +1594,7 @@
         </is>
       </c>
       <c r="B24" s="64" t="n">
-        <v>4353</v>
+        <v>4309</v>
       </c>
       <c r="C24" s="64" t="n"/>
     </row>
@@ -25957,7 +25957,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C82"/>
+  <dimension ref="A1:C53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -25968,7 +25968,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="65" t="inlineStr">
         <is>
-          <t>📺  📡 中国大陆 · 央视  —  共 80 条频道</t>
+          <t>📺  📡 中国大陆 · 央视  —  共 51 条频道</t>
         </is>
       </c>
     </row>
@@ -26077,7 +26077,7 @@
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="70" t="inlineStr">
         <is>
-          <t>CCTV-10_2</t>
+          <t>CCTV-11 戲曲</t>
         </is>
       </c>
       <c r="B8" s="71" t="inlineStr">
@@ -26087,14 +26087,14 @@
       </c>
       <c r="C8" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv10hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv11hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="67" t="inlineStr">
         <is>
-          <t>CCTV-11 戲曲</t>
+          <t>CCTV-12 社會與法</t>
         </is>
       </c>
       <c r="B9" s="68" t="inlineStr">
@@ -26104,14 +26104,14 @@
       </c>
       <c r="C9" s="69" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv11hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv12hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="70" t="inlineStr">
         <is>
-          <t>CCTV-11_1</t>
+          <t>CCTV-13 新聞</t>
         </is>
       </c>
       <c r="B10" s="71" t="inlineStr">
@@ -26121,14 +26121,14 @@
       </c>
       <c r="C10" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv11hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv13hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="67" t="inlineStr">
         <is>
-          <t>CCTV-12 社會與法</t>
+          <t>CCTV-14 少兒</t>
         </is>
       </c>
       <c r="B11" s="68" t="inlineStr">
@@ -26138,14 +26138,14 @@
       </c>
       <c r="C11" s="69" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv12hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv14hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="70" t="inlineStr">
         <is>
-          <t>CCTV-12_1</t>
+          <t>CCTV-15 音樂</t>
         </is>
       </c>
       <c r="B12" s="71" t="inlineStr">
@@ -26155,14 +26155,14 @@
       </c>
       <c r="C12" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv12hd.m3u8</t>
+          <t>https://xykt-fix.github.io/play/a02e/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="67" t="inlineStr">
         <is>
-          <t>CCTV-13 新聞</t>
+          <t>CCTV-17 農業農村</t>
         </is>
       </c>
       <c r="B13" s="68" t="inlineStr">
@@ -26172,14 +26172,14 @@
       </c>
       <c r="C13" s="69" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv13hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv17hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="70" t="inlineStr">
         <is>
-          <t>CCTV-13_1</t>
+          <t>CCTV-2 財經</t>
         </is>
       </c>
       <c r="B14" s="71" t="inlineStr">
@@ -26189,14 +26189,14 @@
       </c>
       <c r="C14" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv13hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv2hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="67" t="inlineStr">
         <is>
-          <t>CCTV-14 少兒</t>
+          <t>CCTV-3 綜藝</t>
         </is>
       </c>
       <c r="B15" s="68" t="inlineStr">
@@ -26206,14 +26206,14 @@
       </c>
       <c r="C15" s="69" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv14hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv3hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="70" t="inlineStr">
         <is>
-          <t>CCTV-14_1</t>
+          <t>CCTV-4 亞洲</t>
         </is>
       </c>
       <c r="B16" s="71" t="inlineStr">
@@ -26223,14 +26223,14 @@
       </c>
       <c r="C16" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv14hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv4hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="67" t="inlineStr">
         <is>
-          <t>CCTV-15 音樂</t>
+          <t>CCTV-4 美洲</t>
         </is>
       </c>
       <c r="B17" s="68" t="inlineStr">
@@ -26240,14 +26240,14 @@
       </c>
       <c r="C17" s="69" t="inlineStr">
         <is>
-          <t>https://xykt-fix.github.io/play/a02e/index.m3u8</t>
+          <t>https://global.cgtn.cicc.media.caton.cloud/master/cgtn-america.m3u8</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="70" t="inlineStr">
         <is>
-          <t>CCTV-15_1</t>
+          <t>CCTV-5+体育赛事_2</t>
         </is>
       </c>
       <c r="B18" s="71" t="inlineStr">
@@ -26257,14 +26257,14 @@
       </c>
       <c r="C18" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv15hd.m3u8</t>
+          <t>http://223.112.114.228:50080/newlive/live/hls/180/live.m3u8</t>
         </is>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="67" t="inlineStr">
         <is>
-          <t>CCTV-16奥林匹克_1</t>
+          <t>CCTV-6 電影</t>
         </is>
       </c>
       <c r="B19" s="68" t="inlineStr">
@@ -26274,14 +26274,14 @@
       </c>
       <c r="C19" s="69" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv16hd.m3u8</t>
+          <t>http://69.30.245.50/live/cctv6.m3u8</t>
         </is>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="70" t="inlineStr">
         <is>
-          <t>CCTV-17 農業農村</t>
+          <t>CCTV-7 國防軍事</t>
         </is>
       </c>
       <c r="B20" s="71" t="inlineStr">
@@ -26291,14 +26291,14 @@
       </c>
       <c r="C20" s="72" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv17hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv7hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="67" t="inlineStr">
         <is>
-          <t>CCTV-17_1</t>
+          <t>CCTV-8 電視劇</t>
         </is>
       </c>
       <c r="B21" s="68" t="inlineStr">
@@ -26308,14 +26308,14 @@
       </c>
       <c r="C21" s="69" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv17hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv8hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="70" t="inlineStr">
         <is>
-          <t>CCTV-1_1</t>
+          <t>CCTV-8K 超高清</t>
         </is>
       </c>
       <c r="B22" s="71" t="inlineStr">
@@ -26325,14 +26325,14 @@
       </c>
       <c r="C22" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv1hd.m3u8</t>
+          <t>http://192.151.150.154/live/cctv8k.m3u8</t>
         </is>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="67" t="inlineStr">
         <is>
-          <t>CCTV-2 財經</t>
+          <t>CCTV-9_1</t>
         </is>
       </c>
       <c r="B23" s="68" t="inlineStr">
@@ -26342,14 +26342,14 @@
       </c>
       <c r="C23" s="69" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv2hd.m3u8</t>
+          <t>https://xykt-fix.github.io/Y77.m3u8</t>
         </is>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="70" t="inlineStr">
         <is>
-          <t>CCTV-2_1</t>
+          <t>CCTV-9_6</t>
         </is>
       </c>
       <c r="B24" s="71" t="inlineStr">
@@ -26359,14 +26359,14 @@
       </c>
       <c r="C24" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv2hd.m3u8</t>
+          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=db000b5568ff643131ea7d86610b09b7</t>
         </is>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="67" t="inlineStr">
         <is>
-          <t>CCTV-3 綜藝</t>
+          <t>CCTV-世界地理</t>
         </is>
       </c>
       <c r="B25" s="68" t="inlineStr">
@@ -26376,14 +26376,14 @@
       </c>
       <c r="C25" s="69" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv3hd.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/sjdl.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="70" t="inlineStr">
         <is>
-          <t>CCTV-3_1</t>
+          <t>CCTV-兵器科技</t>
         </is>
       </c>
       <c r="B26" s="71" t="inlineStr">
@@ -26393,14 +26393,14 @@
       </c>
       <c r="C26" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv3hd.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/gfjs.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="67" t="inlineStr">
         <is>
-          <t>CCTV-4 亞洲</t>
+          <t>CCTV-央視檯球</t>
         </is>
       </c>
       <c r="B27" s="68" t="inlineStr">
@@ -26410,14 +26410,14 @@
       </c>
       <c r="C27" s="69" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv4hd.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/ystq.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="70" t="inlineStr">
         <is>
-          <t>CCTV-4 美洲</t>
+          <t>CCTV-央視精品</t>
         </is>
       </c>
       <c r="B28" s="71" t="inlineStr">
@@ -26427,14 +26427,14 @@
       </c>
       <c r="C28" s="72" t="inlineStr">
         <is>
-          <t>https://global.cgtn.cicc.media.caton.cloud/master/cgtn-america.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/ysjp.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="67" t="inlineStr">
         <is>
-          <t>CCTV-5+体育赛事_1</t>
+          <t>CCTV-女性時尚</t>
         </is>
       </c>
       <c r="B29" s="68" t="inlineStr">
@@ -26444,14 +26444,14 @@
       </c>
       <c r="C29" s="69" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv5p.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/nxss.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="70" t="inlineStr">
         <is>
-          <t>CCTV-5+体育赛事_2</t>
+          <t>CCTV-懷舊劇場</t>
         </is>
       </c>
       <c r="B30" s="71" t="inlineStr">
@@ -26461,14 +26461,14 @@
       </c>
       <c r="C30" s="72" t="inlineStr">
         <is>
-          <t>http://223.112.114.228:50080/newlive/live/hls/180/live.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/hjjc.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="67" t="inlineStr">
         <is>
-          <t>CCTV-5体育_2</t>
+          <t>CCTV-第一劇場</t>
         </is>
       </c>
       <c r="B31" s="68" t="inlineStr">
@@ -26478,14 +26478,14 @@
       </c>
       <c r="C31" s="69" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv5hd.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/dyjc.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="70" t="inlineStr">
         <is>
-          <t>CCTV-6 電影</t>
+          <t>CCTV-衛生健康</t>
         </is>
       </c>
       <c r="B32" s="71" t="inlineStr">
@@ -26495,14 +26495,14 @@
       </c>
       <c r="C32" s="72" t="inlineStr">
         <is>
-          <t>http://69.30.245.50/live/cctv6.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/wsjk.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="67" t="inlineStr">
         <is>
-          <t>CCTV-6_1</t>
+          <t>CCTV-風雲劇場</t>
         </is>
       </c>
       <c r="B33" s="68" t="inlineStr">
@@ -26512,14 +26512,14 @@
       </c>
       <c r="C33" s="69" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv6hd.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/fyjc.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="70" t="inlineStr">
         <is>
-          <t>CCTV-7 國防軍事</t>
+          <t>CCTV-風雲足球</t>
         </is>
       </c>
       <c r="B34" s="71" t="inlineStr">
@@ -26529,14 +26529,14 @@
       </c>
       <c r="C34" s="72" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv7hd.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/fyzq.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="67" t="inlineStr">
         <is>
-          <t>CCTV-7_1</t>
+          <t>CCTV-風雲音樂</t>
         </is>
       </c>
       <c r="B35" s="68" t="inlineStr">
@@ -26546,14 +26546,14 @@
       </c>
       <c r="C35" s="69" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv7hd.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/fyyy.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="70" t="inlineStr">
         <is>
-          <t>CCTV-8 電視劇</t>
+          <t>CCTV-高爾夫網球</t>
         </is>
       </c>
       <c r="B36" s="71" t="inlineStr">
@@ -26563,14 +26563,14 @@
       </c>
       <c r="C36" s="72" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv8hd.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/gefwq.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="67" t="inlineStr">
         <is>
-          <t>CCTV-8K 超高清</t>
+          <t>CCTV11戏曲</t>
         </is>
       </c>
       <c r="B37" s="68" t="inlineStr">
@@ -26580,14 +26580,14 @@
       </c>
       <c r="C37" s="69" t="inlineStr">
         <is>
-          <t>http://192.151.150.154/live/cctv8k.m3u8</t>
+          <t>http://119.233.255.62:1234/667987558</t>
         </is>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1">
       <c r="A38" s="70" t="inlineStr">
         <is>
-          <t>CCTV-8_1</t>
+          <t>CCTV13新闻</t>
         </is>
       </c>
       <c r="B38" s="71" t="inlineStr">
@@ -26597,14 +26597,14 @@
       </c>
       <c r="C38" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv8hd.m3u8</t>
+          <t>http://119.233.255.62:1234/608807423</t>
         </is>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1">
       <c r="A39" s="67" t="inlineStr">
         <is>
-          <t>CCTV-8_2</t>
+          <t>CCTV14少儿</t>
         </is>
       </c>
       <c r="B39" s="68" t="inlineStr">
@@ -26614,14 +26614,14 @@
       </c>
       <c r="C39" s="69" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv8k.m3u8</t>
+          <t>http://119.233.255.62:1234/624878440</t>
         </is>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="70" t="inlineStr">
         <is>
-          <t>CCTV-9_1</t>
+          <t>CCTV17农业农村</t>
         </is>
       </c>
       <c r="B40" s="71" t="inlineStr">
@@ -26631,14 +26631,14 @@
       </c>
       <c r="C40" s="72" t="inlineStr">
         <is>
-          <t>https://xykt-fix.github.io/Y77.m3u8</t>
+          <t>http://119.233.255.62:1234/673168256</t>
         </is>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="67" t="inlineStr">
         <is>
-          <t>CCTV-9_6</t>
+          <t>CCTV1综合</t>
         </is>
       </c>
       <c r="B41" s="68" t="inlineStr">
@@ -26648,14 +26648,14 @@
       </c>
       <c r="C41" s="69" t="inlineStr">
         <is>
-          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=db000b5568ff643131ea7d86610b09b7</t>
+          <t>http://119.233.255.62:1234/608807420</t>
         </is>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1">
       <c r="A42" s="70" t="inlineStr">
         <is>
-          <t>CCTV-世界地理</t>
+          <t>CCTV2财经</t>
         </is>
       </c>
       <c r="B42" s="71" t="inlineStr">
@@ -26665,14 +26665,14 @@
       </c>
       <c r="C42" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/sjdl.m3u8?auth=testpub</t>
+          <t>http://119.233.255.62:1234/631780532</t>
         </is>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="67" t="inlineStr">
         <is>
-          <t>CCTV-兵器科技</t>
+          <t>CCTV3综艺</t>
         </is>
       </c>
       <c r="B43" s="68" t="inlineStr">
@@ -26682,14 +26682,14 @@
       </c>
       <c r="C43" s="69" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/gfjs.m3u8?auth=testpub</t>
+          <t>http://119.233.255.62:1234/624878271</t>
         </is>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="70" t="inlineStr">
         <is>
-          <t>CCTV-卫生健康</t>
+          <t>CCTV4中文国际</t>
         </is>
       </c>
       <c r="B44" s="71" t="inlineStr">
@@ -26699,14 +26699,14 @@
       </c>
       <c r="C44" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/wsjk.m3u8</t>
+          <t>http://119.233.255.62:1234/631780421</t>
         </is>
       </c>
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="67" t="inlineStr">
         <is>
-          <t>CCTV-央視檯球</t>
+          <t>CCTV4欧洲</t>
         </is>
       </c>
       <c r="B45" s="68" t="inlineStr">
@@ -26716,14 +26716,14 @@
       </c>
       <c r="C45" s="69" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/ystq.m3u8?auth=testpub</t>
+          <t>http://119.233.255.62:1234/608807419</t>
         </is>
       </c>
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="70" t="inlineStr">
         <is>
-          <t>CCTV-央視精品</t>
+          <t>CCTV4美洲</t>
         </is>
       </c>
       <c r="B46" s="71" t="inlineStr">
@@ -26733,14 +26733,14 @@
       </c>
       <c r="C46" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/ysjp.m3u8?auth=testpub</t>
+          <t>http://119.233.255.62:1234/608807416</t>
         </is>
       </c>
     </row>
     <row r="47" ht="16" customHeight="1">
       <c r="A47" s="67" t="inlineStr">
         <is>
-          <t>CCTV-央视文化精品</t>
+          <t>CCTV中文国际</t>
         </is>
       </c>
       <c r="B47" s="68" t="inlineStr">
@@ -26750,14 +26750,14 @@
       </c>
       <c r="C47" s="69" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/ysjp.m3u8</t>
+          <t>https://www.youtube.com/embed/vNVp6bxkL1c</t>
         </is>
       </c>
     </row>
     <row r="48" ht="16" customHeight="1">
       <c r="A48" s="70" t="inlineStr">
         <is>
-          <t>CCTV-女性時尚</t>
+          <t>CGTN纪录</t>
         </is>
       </c>
       <c r="B48" s="71" t="inlineStr">
@@ -26767,14 +26767,14 @@
       </c>
       <c r="C48" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/nxss.m3u8?auth=testpub</t>
+          <t>http://english-livebkali.cgtn.com/live/doccgtn_0.m3u8</t>
         </is>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1">
       <c r="A49" s="67" t="inlineStr">
         <is>
-          <t>CCTV-懷舊劇場</t>
+          <t>CGTN英语</t>
         </is>
       </c>
       <c r="B49" s="68" t="inlineStr">
@@ -26784,14 +26784,14 @@
       </c>
       <c r="C49" s="69" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/hjjc.m3u8?auth=testpub</t>
+          <t>https://english-livebkali.cgtn.com/live/encgtn_0.m3u8</t>
         </is>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="70" t="inlineStr">
         <is>
-          <t>CCTV-第一劇場</t>
+          <t>F1 TV</t>
         </is>
       </c>
       <c r="B50" s="71" t="inlineStr">
@@ -26801,14 +26801,14 @@
       </c>
       <c r="C50" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/dyjc.m3u8?auth=testpub</t>
+          <t>https://amg12058-c15studio-amg12058c1-lg-us-5787.playouts.now.amagi.tv/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="51" ht="16" customHeight="1">
       <c r="A51" s="67" t="inlineStr">
         <is>
-          <t>CCTV-衛生健康</t>
+          <t>PGA Tour_4</t>
         </is>
       </c>
       <c r="B51" s="68" t="inlineStr">
@@ -26818,14 +26818,14 @@
       </c>
       <c r="C51" s="69" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/wsjk.m3u8?auth=testpub</t>
+          <t>https://d11k1mnrgfposz.cloudfront.net/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="52" ht="16" customHeight="1">
       <c r="A52" s="70" t="inlineStr">
         <is>
-          <t>CCTV-風雲劇場</t>
+          <t>韩国电影1</t>
         </is>
       </c>
       <c r="B52" s="71" t="inlineStr">
@@ -26835,14 +26835,14 @@
       </c>
       <c r="C52" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/fyjc.m3u8?auth=testpub</t>
+          <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=595</t>
         </is>
       </c>
     </row>
     <row r="53" ht="16" customHeight="1">
       <c r="A53" s="67" t="inlineStr">
         <is>
-          <t>CCTV-風雲足球</t>
+          <t>韩国电影2</t>
         </is>
       </c>
       <c r="B53" s="68" t="inlineStr">
@@ -26851,499 +26851,6 @@
         </is>
       </c>
       <c r="C53" s="69" t="inlineStr">
-        <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/fyzq.m3u8?auth=testpub</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="16" customHeight="1">
-      <c r="A54" s="70" t="inlineStr">
-        <is>
-          <t>CCTV-風雲音樂</t>
-        </is>
-      </c>
-      <c r="B54" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C54" s="72" t="inlineStr">
-        <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/fyyy.m3u8?auth=testpub</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="67" t="inlineStr">
-        <is>
-          <t>CCTV-高爾夫網球</t>
-        </is>
-      </c>
-      <c r="B55" s="68" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C55" s="69" t="inlineStr">
-        <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/gefwq.m3u8?auth=testpub</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="16" customHeight="1">
-      <c r="A56" s="70" t="inlineStr">
-        <is>
-          <t>CCTV11戏曲</t>
-        </is>
-      </c>
-      <c r="B56" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C56" s="72" t="inlineStr">
-        <is>
-          <t>http://119.233.255.62:1234/667987558</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="16" customHeight="1">
-      <c r="A57" s="67" t="inlineStr">
-        <is>
-          <t>CCTV13新闻</t>
-        </is>
-      </c>
-      <c r="B57" s="68" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C57" s="69" t="inlineStr">
-        <is>
-          <t>http://119.233.255.62:1234/608807423</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="16" customHeight="1">
-      <c r="A58" s="70" t="inlineStr">
-        <is>
-          <t>CCTV14少儿</t>
-        </is>
-      </c>
-      <c r="B58" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C58" s="72" t="inlineStr">
-        <is>
-          <t>http://119.233.255.62:1234/624878440</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="16" customHeight="1">
-      <c r="A59" s="67" t="inlineStr">
-        <is>
-          <t>CCTV17农业农村</t>
-        </is>
-      </c>
-      <c r="B59" s="68" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C59" s="69" t="inlineStr">
-        <is>
-          <t>http://119.233.255.62:1234/673168256</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="16" customHeight="1">
-      <c r="A60" s="70" t="inlineStr">
-        <is>
-          <t>CCTV1综合</t>
-        </is>
-      </c>
-      <c r="B60" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C60" s="72" t="inlineStr">
-        <is>
-          <t>http://119.233.255.62:1234/608807420</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="16" customHeight="1">
-      <c r="A61" s="67" t="inlineStr">
-        <is>
-          <t>CCTV2财经</t>
-        </is>
-      </c>
-      <c r="B61" s="68" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C61" s="69" t="inlineStr">
-        <is>
-          <t>http://119.233.255.62:1234/631780532</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="16" customHeight="1">
-      <c r="A62" s="70" t="inlineStr">
-        <is>
-          <t>CCTV3综艺</t>
-        </is>
-      </c>
-      <c r="B62" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C62" s="72" t="inlineStr">
-        <is>
-          <t>http://119.233.255.62:1234/624878271</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="16" customHeight="1">
-      <c r="A63" s="67" t="inlineStr">
-        <is>
-          <t>CCTV4中文国际</t>
-        </is>
-      </c>
-      <c r="B63" s="68" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C63" s="69" t="inlineStr">
-        <is>
-          <t>http://119.233.255.62:1234/631780421</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="16" customHeight="1">
-      <c r="A64" s="70" t="inlineStr">
-        <is>
-          <t>CCTV4欧洲</t>
-        </is>
-      </c>
-      <c r="B64" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C64" s="72" t="inlineStr">
-        <is>
-          <t>http://119.233.255.62:1234/608807419</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="16" customHeight="1">
-      <c r="A65" s="67" t="inlineStr">
-        <is>
-          <t>CCTV4美洲</t>
-        </is>
-      </c>
-      <c r="B65" s="68" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C65" s="69" t="inlineStr">
-        <is>
-          <t>http://119.233.255.62:1234/608807416</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="16" customHeight="1">
-      <c r="A66" s="70" t="inlineStr">
-        <is>
-          <t>CCTV中文国际</t>
-        </is>
-      </c>
-      <c r="B66" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C66" s="72" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/embed/vNVp6bxkL1c</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="16" customHeight="1">
-      <c r="A67" s="67" t="inlineStr">
-        <is>
-          <t>CGTN纪录</t>
-        </is>
-      </c>
-      <c r="B67" s="68" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C67" s="69" t="inlineStr">
-        <is>
-          <t>http://english-livebkali.cgtn.com/live/doccgtn_0.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="16" customHeight="1">
-      <c r="A68" s="70" t="inlineStr">
-        <is>
-          <t>CGTN英语</t>
-        </is>
-      </c>
-      <c r="B68" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C68" s="72" t="inlineStr">
-        <is>
-          <t>https://english-livebkali.cgtn.com/live/encgtn_0.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="16" customHeight="1">
-      <c r="A69" s="67" t="inlineStr">
-        <is>
-          <t>F1 TV</t>
-        </is>
-      </c>
-      <c r="B69" s="68" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C69" s="69" t="inlineStr">
-        <is>
-          <t>https://amg12058-c15studio-amg12058c1-lg-us-5787.playouts.now.amagi.tv/playlist.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="16" customHeight="1">
-      <c r="A70" s="70" t="inlineStr">
-        <is>
-          <t>PGA Tour_4</t>
-        </is>
-      </c>
-      <c r="B70" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C70" s="72" t="inlineStr">
-        <is>
-          <t>https://d11k1mnrgfposz.cloudfront.net/playlist.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="16" customHeight="1">
-      <c r="A71" s="67" t="inlineStr">
-        <is>
-          <t>中国教育3</t>
-        </is>
-      </c>
-      <c r="B71" s="68" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C71" s="69" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/cetv3.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="16" customHeight="1">
-      <c r="A72" s="70" t="inlineStr">
-        <is>
-          <t>中央新影-发现之旅</t>
-        </is>
-      </c>
-      <c r="B72" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C72" s="72" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/fxzl.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="16" customHeight="1">
-      <c r="A73" s="67" t="inlineStr">
-        <is>
-          <t>中央新影-老故事</t>
-        </is>
-      </c>
-      <c r="B73" s="68" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C73" s="69" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/lgs.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="16" customHeight="1">
-      <c r="A74" s="70" t="inlineStr">
-        <is>
-          <t>北京卡酷少儿</t>
-        </is>
-      </c>
-      <c r="B74" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C74" s="72" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/btvkk.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="16" customHeight="1">
-      <c r="A75" s="67" t="inlineStr">
-        <is>
-          <t>广东珠江</t>
-        </is>
-      </c>
-      <c r="B75" s="68" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C75" s="69" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/gdzj.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="16" customHeight="1">
-      <c r="A76" s="70" t="inlineStr">
-        <is>
-          <t>广西国际</t>
-        </is>
-      </c>
-      <c r="B76" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C76" s="72" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/gxgj.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="16" customHeight="1">
-      <c r="A77" s="67" t="inlineStr">
-        <is>
-          <t>广西影视</t>
-        </is>
-      </c>
-      <c r="B77" s="68" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C77" s="69" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/gxys.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="16" customHeight="1">
-      <c r="A78" s="70" t="inlineStr">
-        <is>
-          <t>广西新闻</t>
-        </is>
-      </c>
-      <c r="B78" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C78" s="72" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/gxxw.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="16" customHeight="1">
-      <c r="A79" s="67" t="inlineStr">
-        <is>
-          <t>广西综艺旅游</t>
-        </is>
-      </c>
-      <c r="B79" s="68" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C79" s="69" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/gxzy.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="16" customHeight="1">
-      <c r="A80" s="70" t="inlineStr">
-        <is>
-          <t>广西都市</t>
-        </is>
-      </c>
-      <c r="B80" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C80" s="72" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/gxds.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="16" customHeight="1">
-      <c r="A81" s="67" t="inlineStr">
-        <is>
-          <t>韩国电影1</t>
-        </is>
-      </c>
-      <c r="B81" s="68" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C81" s="69" t="inlineStr">
-        <is>
-          <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=595</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="16" customHeight="1">
-      <c r="A82" s="70" t="inlineStr">
-        <is>
-          <t>韩国电影2</t>
-        </is>
-      </c>
-      <c r="B82" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C82" s="72" t="inlineStr">
         <is>
           <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=743</t>
         </is>
@@ -68267,7 +67774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -68278,7 +67785,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="73" t="inlineStr">
         <is>
-          <t>📺  📡 中国大陆 · 卫视  —  共 41 条频道</t>
+          <t>📺  📡 中国大陆 · 卫视  —  共 26 条频道</t>
         </is>
       </c>
     </row>
@@ -68302,7 +67809,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="74" t="inlineStr">
         <is>
-          <t>东方卫视HD</t>
+          <t>兵团卫视</t>
         </is>
       </c>
       <c r="B3" s="75" t="inlineStr">
@@ -68312,14 +67819,14 @@
       </c>
       <c r="C3" s="76" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/dfwshd.m3u8</t>
+          <t>http://119.233.255.62:1234/956923145</t>
         </is>
       </c>
     </row>
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="70" t="inlineStr">
         <is>
-          <t>兵团卫视</t>
+          <t>大湾区卫视</t>
         </is>
       </c>
       <c r="B4" s="71" t="inlineStr">
@@ -68329,14 +67836,14 @@
       </c>
       <c r="C4" s="72" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/956923145</t>
+          <t>http://119.233.255.62:1234/608917627</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
       <c r="A5" s="74" t="inlineStr">
         <is>
-          <t>大湾区卫视</t>
+          <t>山东教育卫视</t>
         </is>
       </c>
       <c r="B5" s="75" t="inlineStr">
@@ -68346,14 +67853,14 @@
       </c>
       <c r="C5" s="76" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/nfws.m3u8</t>
+          <t>https://test1.live.sdetv.com.cn/live/dianshizhibo/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="6" ht="16" customHeight="1">
       <c r="A6" s="70" t="inlineStr">
         <is>
-          <t>大湾区卫视</t>
+          <t>广东卫视</t>
         </is>
       </c>
       <c r="B6" s="71" t="inlineStr">
@@ -68363,14 +67870,14 @@
       </c>
       <c r="C6" s="72" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/608917627</t>
+          <t>https://h5cdn3.kylintv.tv/live/gdtvhd_iphone.m3u8</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
       <c r="A7" s="74" t="inlineStr">
         <is>
-          <t>天津卫视HD</t>
+          <t>广东卫视</t>
         </is>
       </c>
       <c r="B7" s="75" t="inlineStr">
@@ -68380,14 +67887,14 @@
       </c>
       <c r="C7" s="76" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/tjwshd.m3u8</t>
+          <t>http://119.233.255.62:1234/608831231</t>
         </is>
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
       <c r="A8" s="70" t="inlineStr">
         <is>
-          <t>山东卫视HD</t>
+          <t>延边卫视</t>
         </is>
       </c>
       <c r="B8" s="71" t="inlineStr">
@@ -68397,14 +67904,14 @@
       </c>
       <c r="C8" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/sdwshd.m3u8</t>
+          <t>https://stream2.jlntv.cn/jlyb/sd/live.m3u8</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
       <c r="A9" s="74" t="inlineStr">
         <is>
-          <t>山东教育卫视</t>
+          <t>延边卫视_1</t>
         </is>
       </c>
       <c r="B9" s="75" t="inlineStr">
@@ -68414,14 +67921,14 @@
       </c>
       <c r="C9" s="76" t="inlineStr">
         <is>
-          <t>https://test1.live.sdetv.com.cn/live/dianshizhibo/playlist.m3u8</t>
+          <t>https://srs.iyb983.cn:443/video/CYS/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="70" t="inlineStr">
         <is>
-          <t>广东卫视</t>
+          <t>江苏卫视</t>
         </is>
       </c>
       <c r="B10" s="71" t="inlineStr">
@@ -68431,14 +67938,14 @@
       </c>
       <c r="C10" s="72" t="inlineStr">
         <is>
-          <t>https://h5cdn3.kylintv.tv/live/gdtvhd_iphone.m3u8</t>
+          <t>http://119.233.255.62:1234/623899368</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="74" t="inlineStr">
         <is>
-          <t>广东卫视</t>
+          <t>江西卫视</t>
         </is>
       </c>
       <c r="B11" s="75" t="inlineStr">
@@ -68448,14 +67955,14 @@
       </c>
       <c r="C11" s="76" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/608831231</t>
+          <t>http://119.233.255.62:1234/783847495</t>
         </is>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="70" t="inlineStr">
         <is>
-          <t>广东卫视HD</t>
+          <t>河北卫视</t>
         </is>
       </c>
       <c r="B12" s="71" t="inlineStr">
@@ -68465,14 +67972,14 @@
       </c>
       <c r="C12" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/gdwshd.m3u8</t>
+          <t>https://event.pull.hebtv.com/jishi/weishi_tingyun.m3u8</t>
         </is>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="74" t="inlineStr">
         <is>
-          <t>广西卫视HD</t>
+          <t>河北卫视</t>
         </is>
       </c>
       <c r="B13" s="75" t="inlineStr">
@@ -68482,14 +67989,14 @@
       </c>
       <c r="C13" s="76" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/gxwshd.m3u8</t>
+          <t>http://119.233.255.62:1234/962042070</t>
         </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="70" t="inlineStr">
         <is>
-          <t>延边卫视</t>
+          <t>河南卫视</t>
         </is>
       </c>
       <c r="B14" s="71" t="inlineStr">
@@ -68499,14 +68006,14 @@
       </c>
       <c r="C14" s="72" t="inlineStr">
         <is>
-          <t>https://stream2.jlntv.cn/jlyb/sd/live.m3u8</t>
+          <t>http://119.233.255.62:1234/790187291</t>
         </is>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="74" t="inlineStr">
         <is>
-          <t>延边卫视_1</t>
+          <t>浙江卫视</t>
         </is>
       </c>
       <c r="B15" s="75" t="inlineStr">
@@ -68516,82 +68023,82 @@
       </c>
       <c r="C15" s="76" t="inlineStr">
         <is>
-          <t>https://srs.iyb983.cn:443/video/CYS/index.m3u8</t>
+          <t>https://ali-m-l.cztv.com/channels/lantian/channel001/1080p.m3u8</t>
         </is>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="70" t="inlineStr">
         <is>
-          <t>江苏卫视</t>
+          <t>浙江卫视</t>
         </is>
       </c>
       <c r="B16" s="71" t="inlineStr">
         <is>
-          <t>卫视频道</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C16" s="72" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/623899368</t>
+          <t>https://zwebl02.cztv.com/live/channel01720Pnew.m3u8?auth_key=1790481677822-0-0-ce4b4b3f5c66d708467910377a368f37</t>
         </is>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="74" t="inlineStr">
         <is>
-          <t>江苏卫视HD</t>
+          <t>浙江卫视</t>
         </is>
       </c>
       <c r="B17" s="75" t="inlineStr">
         <is>
-          <t>卫视频道</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C17" s="76" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/jswshd.m3u8</t>
+          <t>https://zwebl02.cztv.com/live/channel011080Pnew.m3u8?auth_key=1790481677822-0-0-e45436808bc7793028ff0aa0a983a6b8</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="70" t="inlineStr">
         <is>
-          <t>江西卫视</t>
+          <t>浙江卫视</t>
         </is>
       </c>
       <c r="B18" s="71" t="inlineStr">
         <is>
-          <t>卫视频道</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C18" s="72" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/783847495</t>
+          <t>https://zwebl06.cztv.com/live/channel01720Pnew.m3u8?auth_key=1790708478994-0-0-0fbbe589185f0869654c7ada4c6960ff</t>
         </is>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="74" t="inlineStr">
         <is>
-          <t>河北卫视</t>
+          <t>浙江卫视</t>
         </is>
       </c>
       <c r="B19" s="75" t="inlineStr">
         <is>
-          <t>卫视频道</t>
+          <t>浙江</t>
         </is>
       </c>
       <c r="C19" s="76" t="inlineStr">
         <is>
-          <t>https://event.pull.hebtv.com/jishi/weishi_tingyun.m3u8</t>
+          <t>https://zwebl06.cztv.com/live/channel011080Pnew.m3u8?auth_key=1790708478993-0-0-305e49d8ae6af955df8e9034ccae894d</t>
         </is>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="70" t="inlineStr">
         <is>
-          <t>河北卫视</t>
+          <t>浙江卫视_1</t>
         </is>
       </c>
       <c r="B20" s="71" t="inlineStr">
@@ -68601,14 +68108,14 @@
       </c>
       <c r="C20" s="72" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/962042070</t>
+          <t>https://ali-xwl.cztv.com/live/channel011080Plxw.m3u8</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="74" t="inlineStr">
         <is>
-          <t>河南卫视</t>
+          <t>浙江卫视_2</t>
         </is>
       </c>
       <c r="B21" s="75" t="inlineStr">
@@ -68618,116 +68125,116 @@
       </c>
       <c r="C21" s="76" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/790187291</t>
+          <t>https://ali-xwl.cztv.com/live/channel01720Plxw.m3u8</t>
         </is>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="70" t="inlineStr">
         <is>
-          <t>浙江卫视</t>
+          <t>海峡卫视</t>
         </is>
       </c>
       <c r="B22" s="71" t="inlineStr">
         <is>
-          <t>卫视频道</t>
+          <t>港澳台</t>
         </is>
       </c>
       <c r="C22" s="72" t="inlineStr">
         <is>
-          <t>https://ali-m-l.cztv.com/channels/lantian/channel001/1080p.m3u8</t>
+          <t>https://php.jdshipin.com/TVOD/iptv.php?id=hxws</t>
         </is>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="74" t="inlineStr">
         <is>
-          <t>浙江卫视</t>
+          <t>海峡卫视</t>
         </is>
       </c>
       <c r="B23" s="75" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>港澳台</t>
         </is>
       </c>
       <c r="C23" s="76" t="inlineStr">
         <is>
-          <t>https://zwebl02.cztv.com/live/channel01720Pnew.m3u8?auth_key=1790481677822-0-0-ce4b4b3f5c66d708467910377a368f37</t>
+          <t>https://7612-5516-affc-d88b.kylintv.tv/live/fjstv_iphone.m3u8</t>
         </is>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="70" t="inlineStr">
         <is>
-          <t>浙江卫视</t>
+          <t>澳门卫视</t>
         </is>
       </c>
       <c r="B24" s="71" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>卫视频道</t>
         </is>
       </c>
       <c r="C24" s="72" t="inlineStr">
         <is>
-          <t>https://zwebl02.cztv.com/live/channel011080Pnew.m3u8?auth_key=1790481677822-0-0-e45436808bc7793028ff0aa0a983a6b8</t>
+          <t>https://live5.tdm.com.mo/ch1/ch1.live/chunklist_w192974802.m3u8</t>
         </is>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="74" t="inlineStr">
         <is>
-          <t>浙江卫视</t>
+          <t>澳门卫视_1</t>
         </is>
       </c>
       <c r="B25" s="75" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>港澳台</t>
         </is>
       </c>
       <c r="C25" s="76" t="inlineStr">
         <is>
-          <t>https://zwebl06.cztv.com/live/channel01720Pnew.m3u8?auth_key=1790708478994-0-0-0fbbe589185f0869654c7ada4c6960ff</t>
+          <t>https://live5.tdm.com.mo/ch1/ch1.live/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="70" t="inlineStr">
         <is>
-          <t>浙江卫视</t>
+          <t>看东方</t>
         </is>
       </c>
       <c r="B26" s="71" t="inlineStr">
         <is>
-          <t>浙江</t>
+          <t>港澳台</t>
         </is>
       </c>
       <c r="C26" s="72" t="inlineStr">
         <is>
-          <t>https://zwebl06.cztv.com/live/channel011080Pnew.m3u8?auth_key=1790708478993-0-0-305e49d8ae6af955df8e9034ccae894d</t>
+          <t>https://bp-resource-dfl.bestv.cn/148/3/video.m3u8</t>
         </is>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="74" t="inlineStr">
         <is>
-          <t>浙江卫视HD</t>
+          <t>看东方</t>
         </is>
       </c>
       <c r="B27" s="75" t="inlineStr">
         <is>
-          <t>卫视频道</t>
+          <t>港澳台</t>
         </is>
       </c>
       <c r="C27" s="76" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/zjwshd.m3u8</t>
+          <t>https://bp-resource-dfl.bestv.cn/155/3/video.m3u8</t>
         </is>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="70" t="inlineStr">
         <is>
-          <t>浙江卫视_1</t>
+          <t>陕西卫视</t>
         </is>
       </c>
       <c r="B28" s="71" t="inlineStr">
@@ -68737,262 +68244,7 @@
       </c>
       <c r="C28" s="72" t="inlineStr">
         <is>
-          <t>https://ali-xwl.cztv.com/live/channel011080Plxw.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="74" t="inlineStr">
-        <is>
-          <t>浙江卫视_2</t>
-        </is>
-      </c>
-      <c r="B29" s="75" t="inlineStr">
-        <is>
-          <t>卫视频道</t>
-        </is>
-      </c>
-      <c r="C29" s="76" t="inlineStr">
-        <is>
-          <t>https://ali-xwl.cztv.com/live/channel01720Plxw.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="70" t="inlineStr">
-        <is>
-          <t>海峡卫视</t>
-        </is>
-      </c>
-      <c r="B30" s="71" t="inlineStr">
-        <is>
-          <t>港澳台</t>
-        </is>
-      </c>
-      <c r="C30" s="72" t="inlineStr">
-        <is>
-          <t>https://php.jdshipin.com/TVOD/iptv.php?id=hxws</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="74" t="inlineStr">
-        <is>
-          <t>海峡卫视</t>
-        </is>
-      </c>
-      <c r="B31" s="75" t="inlineStr">
-        <is>
-          <t>港澳台</t>
-        </is>
-      </c>
-      <c r="C31" s="76" t="inlineStr">
-        <is>
-          <t>https://7612-5516-affc-d88b.kylintv.tv/live/fjstv_iphone.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="70" t="inlineStr">
-        <is>
-          <t>深圳卫视HD</t>
-        </is>
-      </c>
-      <c r="B32" s="71" t="inlineStr">
-        <is>
-          <t>卫视频道</t>
-        </is>
-      </c>
-      <c r="C32" s="72" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/szwshd.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="74" t="inlineStr">
-        <is>
-          <t>湖北卫视HD</t>
-        </is>
-      </c>
-      <c r="B33" s="75" t="inlineStr">
-        <is>
-          <t>卫视频道</t>
-        </is>
-      </c>
-      <c r="C33" s="76" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/hbwshd.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="70" t="inlineStr">
-        <is>
-          <t>湖南卫视HD</t>
-        </is>
-      </c>
-      <c r="B34" s="71" t="inlineStr">
-        <is>
-          <t>卫视频道</t>
-        </is>
-      </c>
-      <c r="C34" s="72" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/hnwshd.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="74" t="inlineStr">
-        <is>
-          <t>澳门卫视</t>
-        </is>
-      </c>
-      <c r="B35" s="75" t="inlineStr">
-        <is>
-          <t>卫视频道</t>
-        </is>
-      </c>
-      <c r="C35" s="76" t="inlineStr">
-        <is>
-          <t>https://live5.tdm.com.mo/ch1/ch1.live/chunklist_w192974802.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="70" t="inlineStr">
-        <is>
-          <t>澳门卫视_1</t>
-        </is>
-      </c>
-      <c r="B36" s="71" t="inlineStr">
-        <is>
-          <t>港澳台</t>
-        </is>
-      </c>
-      <c r="C36" s="72" t="inlineStr">
-        <is>
-          <t>https://live5.tdm.com.mo/ch1/ch1.live/playlist.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="74" t="inlineStr">
-        <is>
-          <t>看东方</t>
-        </is>
-      </c>
-      <c r="B37" s="75" t="inlineStr">
-        <is>
-          <t>港澳台</t>
-        </is>
-      </c>
-      <c r="C37" s="76" t="inlineStr">
-        <is>
-          <t>https://bp-resource-dfl.bestv.cn/148/3/video.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="70" t="inlineStr">
-        <is>
-          <t>看东方</t>
-        </is>
-      </c>
-      <c r="B38" s="71" t="inlineStr">
-        <is>
-          <t>港澳台</t>
-        </is>
-      </c>
-      <c r="C38" s="72" t="inlineStr">
-        <is>
-          <t>https://bp-resource-dfl.bestv.cn/155/3/video.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="74" t="inlineStr">
-        <is>
-          <t>西藏卫视</t>
-        </is>
-      </c>
-      <c r="B39" s="75" t="inlineStr">
-        <is>
-          <t>卫视频道</t>
-        </is>
-      </c>
-      <c r="C39" s="76" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/xzws.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="70" t="inlineStr">
-        <is>
-          <t>辽宁卫视HD</t>
-        </is>
-      </c>
-      <c r="B40" s="71" t="inlineStr">
-        <is>
-          <t>卫视频道</t>
-        </is>
-      </c>
-      <c r="C40" s="72" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/lnwshd.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="74" t="inlineStr">
-        <is>
-          <t>陕西卫视</t>
-        </is>
-      </c>
-      <c r="B41" s="75" t="inlineStr">
-        <is>
-          <t>卫视频道</t>
-        </is>
-      </c>
-      <c r="C41" s="76" t="inlineStr">
-        <is>
           <t>http://119.233.255.62:1234/738910838</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="70" t="inlineStr">
-        <is>
-          <t>陕西卫视HD</t>
-        </is>
-      </c>
-      <c r="B42" s="71" t="inlineStr">
-        <is>
-          <t>卫视频道</t>
-        </is>
-      </c>
-      <c r="C42" s="72" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/snwshd.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="74" t="inlineStr">
-        <is>
-          <t>青海卫视</t>
-        </is>
-      </c>
-      <c r="B43" s="75" t="inlineStr">
-        <is>
-          <t>卫视频道</t>
-        </is>
-      </c>
-      <c r="C43" s="76" t="inlineStr">
-        <is>
-          <t>http://107.150.60.122/live/qhws.m3u8</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add Yibababa CCTV source and introduce official CCTV-4K UHD channel
</commit_message>
<xml_diff>
--- a/channels_overview.xlsx
+++ b/channels_overview.xlsx
@@ -1279,7 +1279,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
@@ -1594,7 +1594,7 @@
         </is>
       </c>
       <c r="B24" s="64" t="n">
-        <v>4296</v>
+        <v>4299</v>
       </c>
       <c r="C24" s="64" t="n"/>
     </row>
@@ -25872,7 +25872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C53"/>
+  <dimension ref="A1:C56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -25883,7 +25883,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="65" t="inlineStr">
         <is>
-          <t>📺  📡 中国大陆 · 央视  —  共 51 条频道</t>
+          <t>📺  📡 中国大陆 · 央视  —  共 54 条频道</t>
         </is>
       </c>
     </row>
@@ -26026,7 +26026,7 @@
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="70" t="inlineStr">
         <is>
-          <t>CCTV-13 新聞</t>
+          <t>CCTV-12 社會與法</t>
         </is>
       </c>
       <c r="B10" s="71" t="inlineStr">
@@ -26036,14 +26036,14 @@
       </c>
       <c r="C10" s="72" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv13hd.m3u8</t>
+          <t>https://live-play-hls.cctvnews.cctv.com/CCTVChannel/channel_cctv12_mhd.m3u8?auth_key=1790777700-1-044e657af0da02fac29321d9de76e15de37baa3a982c5fb7b7d689fb101cd031-86746c0e529612c08db4e091286d5fa1</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="67" t="inlineStr">
         <is>
-          <t>CCTV-14 少兒</t>
+          <t>CCTV-13 新聞</t>
         </is>
       </c>
       <c r="B11" s="68" t="inlineStr">
@@ -26053,14 +26053,14 @@
       </c>
       <c r="C11" s="69" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv14hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv13hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="70" t="inlineStr">
         <is>
-          <t>CCTV-15 音樂</t>
+          <t>CCTV-14 少兒</t>
         </is>
       </c>
       <c r="B12" s="71" t="inlineStr">
@@ -26070,14 +26070,14 @@
       </c>
       <c r="C12" s="72" t="inlineStr">
         <is>
-          <t>https://xykt-fix.github.io/play/a02e/index.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv14hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="67" t="inlineStr">
         <is>
-          <t>CCTV-17 農業農村</t>
+          <t>CCTV-15 音樂</t>
         </is>
       </c>
       <c r="B13" s="68" t="inlineStr">
@@ -26087,14 +26087,14 @@
       </c>
       <c r="C13" s="69" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv17hd.m3u8</t>
+          <t>https://xykt-fix.github.io/play/a02e/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="70" t="inlineStr">
         <is>
-          <t>CCTV-2 財經</t>
+          <t>CCTV-17 農業農村</t>
         </is>
       </c>
       <c r="B14" s="71" t="inlineStr">
@@ -26104,14 +26104,14 @@
       </c>
       <c r="C14" s="72" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv2hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv17hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="67" t="inlineStr">
         <is>
-          <t>CCTV-3 綜藝</t>
+          <t>CCTV-17 農業農村</t>
         </is>
       </c>
       <c r="B15" s="68" t="inlineStr">
@@ -26121,14 +26121,14 @@
       </c>
       <c r="C15" s="69" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv3hd.m3u8</t>
+          <t>https://live-play-hls.cctvnews.cctv.com/CCTVChannel/channel_cctv17_mhd.m3u8?auth_key=1790777700-1-044e657af0da02fac29321d9de76e15de37baa3a982c5fb7b7d689fb101cd031-74adbe32fb807daeb89f646429b846d1</t>
         </is>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="A16" s="70" t="inlineStr">
         <is>
-          <t>CCTV-4 亞洲</t>
+          <t>CCTV-2 財經</t>
         </is>
       </c>
       <c r="B16" s="71" t="inlineStr">
@@ -26138,14 +26138,14 @@
       </c>
       <c r="C16" s="72" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv4hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv2hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="67" t="inlineStr">
         <is>
-          <t>CCTV-4 美洲</t>
+          <t>CCTV-3 綜藝</t>
         </is>
       </c>
       <c r="B17" s="68" t="inlineStr">
@@ -26155,14 +26155,14 @@
       </c>
       <c r="C17" s="69" t="inlineStr">
         <is>
-          <t>https://global.cgtn.cicc.media.caton.cloud/master/cgtn-america.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv3hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="70" t="inlineStr">
         <is>
-          <t>CCTV-5+体育赛事_2</t>
+          <t>CCTV-4 亞洲</t>
         </is>
       </c>
       <c r="B18" s="71" t="inlineStr">
@@ -26172,14 +26172,14 @@
       </c>
       <c r="C18" s="72" t="inlineStr">
         <is>
-          <t>http://223.112.114.228:50080/newlive/live/hls/180/live.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv4hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="67" t="inlineStr">
         <is>
-          <t>CCTV-6 電影</t>
+          <t>CCTV-4 美洲</t>
         </is>
       </c>
       <c r="B19" s="68" t="inlineStr">
@@ -26189,14 +26189,14 @@
       </c>
       <c r="C19" s="69" t="inlineStr">
         <is>
-          <t>http://69.30.245.50/live/cctv6.m3u8</t>
+          <t>https://global.cgtn.cicc.media.caton.cloud/master/cgtn-america.m3u8</t>
         </is>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="70" t="inlineStr">
         <is>
-          <t>CCTV-7 國防軍事</t>
+          <t>CCTV-4K</t>
         </is>
       </c>
       <c r="B20" s="71" t="inlineStr">
@@ -26206,14 +26206,14 @@
       </c>
       <c r="C20" s="72" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv7hd.m3u8</t>
+          <t>https://live-play-hls.cctvnews.cctv.com/CCTVChannel/channel_cctv4k_mhd.m3u8?auth_key=1790777700-1-044e657af0da02fac29321d9de76e15de37baa3a982c5fb7b7d689fb101cd031-35e7190709b3acddf53caa430bbd3794</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="67" t="inlineStr">
         <is>
-          <t>CCTV-8 電視劇</t>
+          <t>CCTV-5+体育赛事_2</t>
         </is>
       </c>
       <c r="B21" s="68" t="inlineStr">
@@ -26223,14 +26223,14 @@
       </c>
       <c r="C21" s="69" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv8hd.m3u8</t>
+          <t>http://223.112.114.228:50080/newlive/live/hls/180/live.m3u8</t>
         </is>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="70" t="inlineStr">
         <is>
-          <t>CCTV-8K 超高清</t>
+          <t>CCTV-6 電影</t>
         </is>
       </c>
       <c r="B22" s="71" t="inlineStr">
@@ -26240,14 +26240,14 @@
       </c>
       <c r="C22" s="72" t="inlineStr">
         <is>
-          <t>http://192.151.150.154/live/cctv8k.m3u8</t>
+          <t>http://69.30.245.50/live/cctv6.m3u8</t>
         </is>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="67" t="inlineStr">
         <is>
-          <t>CCTV-9_1</t>
+          <t>CCTV-7 國防軍事</t>
         </is>
       </c>
       <c r="B23" s="68" t="inlineStr">
@@ -26257,14 +26257,14 @@
       </c>
       <c r="C23" s="69" t="inlineStr">
         <is>
-          <t>https://xykt-fix.github.io/Y77.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv7hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="A24" s="70" t="inlineStr">
         <is>
-          <t>CCTV-9_6</t>
+          <t>CCTV-8 電視劇</t>
         </is>
       </c>
       <c r="B24" s="71" t="inlineStr">
@@ -26274,14 +26274,14 @@
       </c>
       <c r="C24" s="72" t="inlineStr">
         <is>
-          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=db000b5568ff643131ea7d86610b09b7</t>
+          <t>http://74.91.26.218:82/live/cctv8hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="67" t="inlineStr">
         <is>
-          <t>CCTV-世界地理</t>
+          <t>CCTV-8K 超高清</t>
         </is>
       </c>
       <c r="B25" s="68" t="inlineStr">
@@ -26291,14 +26291,14 @@
       </c>
       <c r="C25" s="69" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/sjdl.m3u8?auth=testpub</t>
+          <t>http://192.151.150.154/live/cctv8k.m3u8</t>
         </is>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="70" t="inlineStr">
         <is>
-          <t>CCTV-兵器科技</t>
+          <t>CCTV-9_1</t>
         </is>
       </c>
       <c r="B26" s="71" t="inlineStr">
@@ -26308,14 +26308,14 @@
       </c>
       <c r="C26" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/gfjs.m3u8?auth=testpub</t>
+          <t>https://xykt-fix.github.io/Y77.m3u8</t>
         </is>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="67" t="inlineStr">
         <is>
-          <t>CCTV-央視檯球</t>
+          <t>CCTV-9_6</t>
         </is>
       </c>
       <c r="B27" s="68" t="inlineStr">
@@ -26325,14 +26325,14 @@
       </c>
       <c r="C27" s="69" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/ystq.m3u8?auth=testpub</t>
+          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=db000b5568ff643131ea7d86610b09b7</t>
         </is>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="70" t="inlineStr">
         <is>
-          <t>CCTV-央視精品</t>
+          <t>CCTV-世界地理</t>
         </is>
       </c>
       <c r="B28" s="71" t="inlineStr">
@@ -26342,14 +26342,14 @@
       </c>
       <c r="C28" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/ysjp.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/sjdl.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="67" t="inlineStr">
         <is>
-          <t>CCTV-女性時尚</t>
+          <t>CCTV-兵器科技</t>
         </is>
       </c>
       <c r="B29" s="68" t="inlineStr">
@@ -26359,14 +26359,14 @@
       </c>
       <c r="C29" s="69" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/nxss.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/gfjs.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="70" t="inlineStr">
         <is>
-          <t>CCTV-懷舊劇場</t>
+          <t>CCTV-央視檯球</t>
         </is>
       </c>
       <c r="B30" s="71" t="inlineStr">
@@ -26376,14 +26376,14 @@
       </c>
       <c r="C30" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/hjjc.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/ystq.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="67" t="inlineStr">
         <is>
-          <t>CCTV-第一劇場</t>
+          <t>CCTV-央視精品</t>
         </is>
       </c>
       <c r="B31" s="68" t="inlineStr">
@@ -26393,14 +26393,14 @@
       </c>
       <c r="C31" s="69" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/dyjc.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/ysjp.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="70" t="inlineStr">
         <is>
-          <t>CCTV-衛生健康</t>
+          <t>CCTV-女性時尚</t>
         </is>
       </c>
       <c r="B32" s="71" t="inlineStr">
@@ -26410,14 +26410,14 @@
       </c>
       <c r="C32" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/wsjk.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/nxss.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="67" t="inlineStr">
         <is>
-          <t>CCTV-風雲劇場</t>
+          <t>CCTV-懷舊劇場</t>
         </is>
       </c>
       <c r="B33" s="68" t="inlineStr">
@@ -26427,14 +26427,14 @@
       </c>
       <c r="C33" s="69" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/fyjc.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/hjjc.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="70" t="inlineStr">
         <is>
-          <t>CCTV-風雲足球</t>
+          <t>CCTV-第一劇場</t>
         </is>
       </c>
       <c r="B34" s="71" t="inlineStr">
@@ -26444,14 +26444,14 @@
       </c>
       <c r="C34" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/fyzq.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/dyjc.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="67" t="inlineStr">
         <is>
-          <t>CCTV-風雲音樂</t>
+          <t>CCTV-衛生健康</t>
         </is>
       </c>
       <c r="B35" s="68" t="inlineStr">
@@ -26461,14 +26461,14 @@
       </c>
       <c r="C35" s="69" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/fyyy.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/wsjk.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="70" t="inlineStr">
         <is>
-          <t>CCTV-高爾夫網球</t>
+          <t>CCTV-風雲劇場</t>
         </is>
       </c>
       <c r="B36" s="71" t="inlineStr">
@@ -26478,14 +26478,14 @@
       </c>
       <c r="C36" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/gefwq.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/fyjc.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="67" t="inlineStr">
         <is>
-          <t>CCTV11戏曲</t>
+          <t>CCTV-風雲足球</t>
         </is>
       </c>
       <c r="B37" s="68" t="inlineStr">
@@ -26495,14 +26495,14 @@
       </c>
       <c r="C37" s="69" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/667987558</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/fyzq.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1">
       <c r="A38" s="70" t="inlineStr">
         <is>
-          <t>CCTV13新闻</t>
+          <t>CCTV-風雲音樂</t>
         </is>
       </c>
       <c r="B38" s="71" t="inlineStr">
@@ -26512,14 +26512,14 @@
       </c>
       <c r="C38" s="72" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/608807423</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/fyyy.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1">
       <c r="A39" s="67" t="inlineStr">
         <is>
-          <t>CCTV14少儿</t>
+          <t>CCTV-高爾夫網球</t>
         </is>
       </c>
       <c r="B39" s="68" t="inlineStr">
@@ -26529,14 +26529,14 @@
       </c>
       <c r="C39" s="69" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/624878440</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/gefwq.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="70" t="inlineStr">
         <is>
-          <t>CCTV17农业农村</t>
+          <t>CCTV11戏曲</t>
         </is>
       </c>
       <c r="B40" s="71" t="inlineStr">
@@ -26546,14 +26546,14 @@
       </c>
       <c r="C40" s="72" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/673168256</t>
+          <t>http://119.233.255.62:1234/667987558</t>
         </is>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="67" t="inlineStr">
         <is>
-          <t>CCTV1综合</t>
+          <t>CCTV13新闻</t>
         </is>
       </c>
       <c r="B41" s="68" t="inlineStr">
@@ -26563,14 +26563,14 @@
       </c>
       <c r="C41" s="69" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/608807420</t>
+          <t>http://119.233.255.62:1234/608807423</t>
         </is>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1">
       <c r="A42" s="70" t="inlineStr">
         <is>
-          <t>CCTV2财经</t>
+          <t>CCTV14少儿</t>
         </is>
       </c>
       <c r="B42" s="71" t="inlineStr">
@@ -26580,14 +26580,14 @@
       </c>
       <c r="C42" s="72" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/631780532</t>
+          <t>http://119.233.255.62:1234/624878440</t>
         </is>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="67" t="inlineStr">
         <is>
-          <t>CCTV3综艺</t>
+          <t>CCTV17农业农村</t>
         </is>
       </c>
       <c r="B43" s="68" t="inlineStr">
@@ -26597,14 +26597,14 @@
       </c>
       <c r="C43" s="69" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/624878271</t>
+          <t>http://119.233.255.62:1234/673168256</t>
         </is>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="70" t="inlineStr">
         <is>
-          <t>CCTV4中文国际</t>
+          <t>CCTV1综合</t>
         </is>
       </c>
       <c r="B44" s="71" t="inlineStr">
@@ -26614,14 +26614,14 @@
       </c>
       <c r="C44" s="72" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/631780421</t>
+          <t>http://119.233.255.62:1234/608807420</t>
         </is>
       </c>
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="67" t="inlineStr">
         <is>
-          <t>CCTV4欧洲</t>
+          <t>CCTV2财经</t>
         </is>
       </c>
       <c r="B45" s="68" t="inlineStr">
@@ -26631,14 +26631,14 @@
       </c>
       <c r="C45" s="69" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/608807419</t>
+          <t>http://119.233.255.62:1234/631780532</t>
         </is>
       </c>
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="70" t="inlineStr">
         <is>
-          <t>CCTV4美洲</t>
+          <t>CCTV3综艺</t>
         </is>
       </c>
       <c r="B46" s="71" t="inlineStr">
@@ -26648,14 +26648,14 @@
       </c>
       <c r="C46" s="72" t="inlineStr">
         <is>
-          <t>http://119.233.255.62:1234/608807416</t>
+          <t>http://119.233.255.62:1234/624878271</t>
         </is>
       </c>
     </row>
     <row r="47" ht="16" customHeight="1">
       <c r="A47" s="67" t="inlineStr">
         <is>
-          <t>CCTV中文国际</t>
+          <t>CCTV4中文国际</t>
         </is>
       </c>
       <c r="B47" s="68" t="inlineStr">
@@ -26665,14 +26665,14 @@
       </c>
       <c r="C47" s="69" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/embed/vNVp6bxkL1c</t>
+          <t>http://119.233.255.62:1234/631780421</t>
         </is>
       </c>
     </row>
     <row r="48" ht="16" customHeight="1">
       <c r="A48" s="70" t="inlineStr">
         <is>
-          <t>CGTN纪录</t>
+          <t>CCTV4欧洲</t>
         </is>
       </c>
       <c r="B48" s="71" t="inlineStr">
@@ -26682,14 +26682,14 @@
       </c>
       <c r="C48" s="72" t="inlineStr">
         <is>
-          <t>http://english-livebkali.cgtn.com/live/doccgtn_0.m3u8</t>
+          <t>http://119.233.255.62:1234/608807419</t>
         </is>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1">
       <c r="A49" s="67" t="inlineStr">
         <is>
-          <t>CGTN英语</t>
+          <t>CCTV4美洲</t>
         </is>
       </c>
       <c r="B49" s="68" t="inlineStr">
@@ -26699,14 +26699,14 @@
       </c>
       <c r="C49" s="69" t="inlineStr">
         <is>
-          <t>https://english-livebkali.cgtn.com/live/encgtn_0.m3u8</t>
+          <t>http://119.233.255.62:1234/608807416</t>
         </is>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="70" t="inlineStr">
         <is>
-          <t>F1 TV</t>
+          <t>CCTV中文国际</t>
         </is>
       </c>
       <c r="B50" s="71" t="inlineStr">
@@ -26716,14 +26716,14 @@
       </c>
       <c r="C50" s="72" t="inlineStr">
         <is>
-          <t>https://amg12058-c15studio-amg12058c1-lg-us-5787.playouts.now.amagi.tv/playlist.m3u8</t>
+          <t>https://www.youtube.com/embed/vNVp6bxkL1c</t>
         </is>
       </c>
     </row>
     <row r="51" ht="16" customHeight="1">
       <c r="A51" s="67" t="inlineStr">
         <is>
-          <t>PGA Tour_4</t>
+          <t>CGTN纪录</t>
         </is>
       </c>
       <c r="B51" s="68" t="inlineStr">
@@ -26733,14 +26733,14 @@
       </c>
       <c r="C51" s="69" t="inlineStr">
         <is>
-          <t>https://d11k1mnrgfposz.cloudfront.net/playlist.m3u8</t>
+          <t>http://english-livebkali.cgtn.com/live/doccgtn_0.m3u8</t>
         </is>
       </c>
     </row>
     <row r="52" ht="16" customHeight="1">
       <c r="A52" s="70" t="inlineStr">
         <is>
-          <t>韩国电影1</t>
+          <t>CGTN英语</t>
         </is>
       </c>
       <c r="B52" s="71" t="inlineStr">
@@ -26750,22 +26750,73 @@
       </c>
       <c r="C52" s="72" t="inlineStr">
         <is>
-          <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=595</t>
+          <t>https://english-livebkali.cgtn.com/live/encgtn_0.m3u8</t>
         </is>
       </c>
     </row>
     <row r="53" ht="16" customHeight="1">
       <c r="A53" s="67" t="inlineStr">
         <is>
+          <t>F1 TV</t>
+        </is>
+      </c>
+      <c r="B53" s="68" t="inlineStr">
+        <is>
+          <t>央视频道</t>
+        </is>
+      </c>
+      <c r="C53" s="69" t="inlineStr">
+        <is>
+          <t>https://amg12058-c15studio-amg12058c1-lg-us-5787.playouts.now.amagi.tv/playlist.m3u8</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="16" customHeight="1">
+      <c r="A54" s="70" t="inlineStr">
+        <is>
+          <t>PGA Tour_4</t>
+        </is>
+      </c>
+      <c r="B54" s="71" t="inlineStr">
+        <is>
+          <t>央视频道</t>
+        </is>
+      </c>
+      <c r="C54" s="72" t="inlineStr">
+        <is>
+          <t>https://d11k1mnrgfposz.cloudfront.net/playlist.m3u8</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="16" customHeight="1">
+      <c r="A55" s="67" t="inlineStr">
+        <is>
+          <t>韩国电影1</t>
+        </is>
+      </c>
+      <c r="B55" s="68" t="inlineStr">
+        <is>
+          <t>央视频道</t>
+        </is>
+      </c>
+      <c r="C55" s="69" t="inlineStr">
+        <is>
+          <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=595</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="16" customHeight="1">
+      <c r="A56" s="70" t="inlineStr">
+        <is>
           <t>韩国电影2</t>
         </is>
       </c>
-      <c r="B53" s="68" t="inlineStr">
+      <c r="B56" s="71" t="inlineStr">
         <is>
           <t>央视频道</t>
         </is>
       </c>
-      <c r="C53" s="69" t="inlineStr">
+      <c r="C56" s="72" t="inlineStr">
         <is>
           <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=743</t>
         </is>

</xml_diff>

<commit_message>
fix: remove looping lantian channel001 stream and add Hunan TV
</commit_message>
<xml_diff>
--- a/channels_overview.xlsx
+++ b/channels_overview.xlsx
@@ -1489,7 +1489,7 @@
         </is>
       </c>
       <c r="B17" s="46" t="n">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C17" s="47" t="inlineStr">
         <is>
@@ -1594,7 +1594,7 @@
         </is>
       </c>
       <c r="B24" s="64" t="n">
-        <v>4334</v>
+        <v>4333</v>
       </c>
       <c r="C24" s="64" t="n"/>
     </row>
@@ -7447,7 +7447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C154"/>
+  <dimension ref="A1:C153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -7458,7 +7458,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="125" t="inlineStr">
         <is>
-          <t>📺  📡 中国大陆 · 地方综合台  —  共 152 条频道</t>
+          <t>📺  📡 中国大陆 · 地方综合台  —  共 151 条频道</t>
         </is>
       </c>
     </row>
@@ -9148,41 +9148,41 @@
     <row r="101" ht="16" customHeight="1">
       <c r="A101" s="126" t="inlineStr">
         <is>
-          <t>湖南衛視</t>
+          <t>湖南都市</t>
         </is>
       </c>
       <c r="B101" s="127" t="inlineStr">
         <is>
-          <t>其他地方台</t>
+          <t>芒果TV</t>
         </is>
       </c>
       <c r="C101" s="128" t="inlineStr">
         <is>
-          <t>http://hlsal-ldvt.qing.mgtv.com/nn_live/nn_x64/dWlwPTEyNy4wLjAuMSZ1aWQ9cWluZy1jbXMmbm5fdGltZXpvbmU9OCZjZG5leF9pZD1hbF9obHNfbGR2dCZ1dWlkPTliODY4NmU5ZTM2YzYwMmMmZT02OTE0NjA0JnY9MSZpZD1ITldTWkdTVCZzPTcwN2RiYTc2YzJjNmJmMTQ4MmUyZGYzOWU2NWM3YWFi/HNWSZGST.m3u8</t>
+          <t>https://padqq.qing.mgtv.com/nn_live/nn_x64/Y2hzPSZkZWY9MSZ1aXA9NDcuMTA4LjcyLjQ1JnRlcm09NCZtYWNpZD1kOWRjZGYwNi03YzI0LTQ2MWItOTJiYy02NTM0MGQyMWY1NTkmcWlkPSZyYXV0aF9lbmFibGU9b24mY2RuZXhfaWQ9cXFfcGhvbmVfbGl2ZSZlcz0xNzkwNzM3MjU3JnV1aWQ9NTU4ODdkZWExYTViZjY1MWRmOWEwOTI4NmZmYjEyMDktMmY2YzQ4MmQmcz1kYjRhODQ4ZTlkZTc0NzdjYzY3ZjQzNWMxYzI2YTcxOSZ1aWQ9Jm5kdj1wY193ZWItaW1nb3R2LXBjaDUtMS4yLjMmdj0yJmFzPTAmX2NhckNvZGU9MA,,/HNDSMPP360.m3u8</t>
         </is>
       </c>
     </row>
     <row r="102" ht="16" customHeight="1">
       <c r="A102" s="70" t="inlineStr">
         <is>
-          <t>湖南都市</t>
+          <t>漠河市综合</t>
         </is>
       </c>
       <c r="B102" s="71" t="inlineStr">
         <is>
-          <t>芒果TV</t>
+          <t>其他地方台</t>
         </is>
       </c>
       <c r="C102" s="72" t="inlineStr">
         <is>
-          <t>https://padqq.qing.mgtv.com/nn_live/nn_x64/Y2hzPSZkZWY9MSZ1aXA9NDcuMTA4LjcyLjQ1JnRlcm09NCZtYWNpZD1kOWRjZGYwNi03YzI0LTQ2MWItOTJiYy02NTM0MGQyMWY1NTkmcWlkPSZyYXV0aF9lbmFibGU9b24mY2RuZXhfaWQ9cXFfcGhvbmVfbGl2ZSZlcz0xNzkwNzM3MjU3JnV1aWQ9NTU4ODdkZWExYTViZjY1MWRmOWEwOTI4NmZmYjEyMDktMmY2YzQ4MmQmcz1kYjRhODQ4ZTlkZTc0NzdjYzY3ZjQzNWMxYzI2YTcxOSZ1aWQ9Jm5kdj1wY193ZWItaW1nb3R2LXBjaDUtMS4yLjMmdj0yJmFzPTAmX2NhckNvZGU9MA,,/HNDSMPP360.m3u8</t>
+          <t>https://cors-anywhere.yidianzhishi.cn/https://masterpull.hljtv.com/live/rlVvbTZN.m3u8</t>
         </is>
       </c>
     </row>
     <row r="103" ht="16" customHeight="1">
       <c r="A103" s="126" t="inlineStr">
         <is>
-          <t>漠河市综合</t>
+          <t>甘孜综合</t>
         </is>
       </c>
       <c r="B103" s="127" t="inlineStr">
@@ -9192,82 +9192,82 @@
       </c>
       <c r="C103" s="128" t="inlineStr">
         <is>
-          <t>https://cors-anywhere.yidianzhishi.cn/https://masterpull.hljtv.com/live/rlVvbTZN.m3u8</t>
+          <t>https://m3u8channel.ganzitv.com/nmip-media/channellive/channel1/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="104" ht="16" customHeight="1">
       <c r="A104" s="70" t="inlineStr">
         <is>
-          <t>甘孜综合</t>
+          <t>白城新闻综合</t>
         </is>
       </c>
       <c r="B104" s="71" t="inlineStr">
         <is>
-          <t>其他地方台</t>
+          <t>吉林频道</t>
         </is>
       </c>
       <c r="C104" s="72" t="inlineStr">
         <is>
-          <t>https://m3u8channel.ganzitv.com/nmip-media/channellive/channel1/playlist.m3u8</t>
+          <t>https://stream2.jlntv.cn/baicheng1/sd/live.m3u8</t>
         </is>
       </c>
     </row>
     <row r="105" ht="16" customHeight="1">
       <c r="A105" s="126" t="inlineStr">
         <is>
-          <t>白城新闻综合</t>
+          <t>白银综合</t>
         </is>
       </c>
       <c r="B105" s="127" t="inlineStr">
         <is>
-          <t>吉林频道</t>
+          <t>甘肃频道</t>
         </is>
       </c>
       <c r="C105" s="128" t="inlineStr">
         <is>
-          <t>https://stream2.jlntv.cn/baicheng1/sd/live.m3u8</t>
+          <t>https://play.kankanlive.com/live/1720408089419110.m3u8</t>
         </is>
       </c>
     </row>
     <row r="106" ht="16" customHeight="1">
       <c r="A106" s="70" t="inlineStr">
         <is>
-          <t>白银综合</t>
+          <t>看东方4K</t>
         </is>
       </c>
       <c r="B106" s="71" t="inlineStr">
         <is>
-          <t>甘肃频道</t>
+          <t>地方频道</t>
         </is>
       </c>
       <c r="C106" s="72" t="inlineStr">
         <is>
-          <t>https://play.kankanlive.com/live/1720408089419110.m3u8</t>
+          <t>http://bp-resource-dfl.bestv.cn/148/3/video.m3u8</t>
         </is>
       </c>
     </row>
     <row r="107" ht="16" customHeight="1">
       <c r="A107" s="126" t="inlineStr">
         <is>
-          <t>看东方4K</t>
+          <t>磐石综合</t>
         </is>
       </c>
       <c r="B107" s="127" t="inlineStr">
         <is>
-          <t>地方频道</t>
+          <t>吉林频道</t>
         </is>
       </c>
       <c r="C107" s="128" t="inlineStr">
         <is>
-          <t>http://bp-resource-dfl.bestv.cn/148/3/video.m3u8</t>
+          <t>https://cors-anywhere.yidianzhishi.cn/http://stream5.jlntv.cn/ps/sd/live.m3u8</t>
         </is>
       </c>
     </row>
     <row r="108" ht="16" customHeight="1">
       <c r="A108" s="70" t="inlineStr">
         <is>
-          <t>磐石综合</t>
+          <t>磐石综合_1</t>
         </is>
       </c>
       <c r="B108" s="71" t="inlineStr">
@@ -9277,31 +9277,31 @@
       </c>
       <c r="C108" s="72" t="inlineStr">
         <is>
-          <t>https://cors-anywhere.yidianzhishi.cn/http://stream5.jlntv.cn/ps/sd/live.m3u8</t>
+          <t>https://cors-anywhere.yidianzhishi.cn/http://stream5.jlntv.cn/ps/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="109" ht="16" customHeight="1">
       <c r="A109" s="126" t="inlineStr">
         <is>
-          <t>磐石综合_1</t>
+          <t>福州1</t>
         </is>
       </c>
       <c r="B109" s="127" t="inlineStr">
         <is>
-          <t>吉林频道</t>
+          <t>福建频道</t>
         </is>
       </c>
       <c r="C109" s="128" t="inlineStr">
         <is>
-          <t>https://cors-anywhere.yidianzhishi.cn/http://stream5.jlntv.cn/ps/playlist.m3u8</t>
+          <t>https://live.zohi.tv/video/s10001-fztv-1/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="110" ht="16" customHeight="1">
       <c r="A110" s="70" t="inlineStr">
         <is>
-          <t>福州1</t>
+          <t>福州3</t>
         </is>
       </c>
       <c r="B110" s="71" t="inlineStr">
@@ -9311,14 +9311,14 @@
       </c>
       <c r="C110" s="72" t="inlineStr">
         <is>
-          <t>https://live.zohi.tv/video/s10001-fztv-1/index.m3u8</t>
+          <t>https://live.zohi.tv/video/s10001-fztv-3/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="111" ht="16" customHeight="1">
       <c r="A111" s="126" t="inlineStr">
         <is>
-          <t>福州3</t>
+          <t>福州4</t>
         </is>
       </c>
       <c r="B111" s="127" t="inlineStr">
@@ -9328,48 +9328,48 @@
       </c>
       <c r="C111" s="128" t="inlineStr">
         <is>
-          <t>https://live.zohi.tv/video/s10001-fztv-3/index.m3u8</t>
+          <t>https://live.zohi.tv/video/s10001-fztv-4/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="112" ht="16" customHeight="1">
       <c r="A112" s="70" t="inlineStr">
         <is>
-          <t>福州4</t>
+          <t>绍兴公共</t>
         </is>
       </c>
       <c r="B112" s="71" t="inlineStr">
         <is>
-          <t>福建频道</t>
+          <t>地方频道</t>
         </is>
       </c>
       <c r="C112" s="72" t="inlineStr">
         <is>
-          <t>https://live.zohi.tv/video/s10001-fztv-4/index.m3u8</t>
+          <t>http://live.shaoxing.com.cn/video/s10001-sxtv2/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="113" ht="16" customHeight="1">
       <c r="A113" s="126" t="inlineStr">
         <is>
-          <t>绍兴公共</t>
+          <t>绍兴公共频道</t>
         </is>
       </c>
       <c r="B113" s="127" t="inlineStr">
         <is>
-          <t>地方频道</t>
+          <t>其他地方台</t>
         </is>
       </c>
       <c r="C113" s="128" t="inlineStr">
         <is>
-          <t>http://live.shaoxing.com.cn/video/s10001-sxtv2/index.m3u8</t>
+          <t>https://live.shaoxing.com.cn/video/s10001-sxtv2/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="114" ht="16" customHeight="1">
       <c r="A114" s="70" t="inlineStr">
         <is>
-          <t>绍兴公共频道</t>
+          <t>绍兴新闻综合</t>
         </is>
       </c>
       <c r="B114" s="71" t="inlineStr">
@@ -9379,24 +9379,24 @@
       </c>
       <c r="C114" s="72" t="inlineStr">
         <is>
-          <t>https://live.shaoxing.com.cn/video/s10001-sxtv2/index.m3u8</t>
+          <t>https://live.shaoxing.com.cn/video/s10001-sxhb/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="115" ht="16" customHeight="1">
       <c r="A115" s="126" t="inlineStr">
         <is>
-          <t>绍兴新闻综合</t>
+          <t>经济生活</t>
         </is>
       </c>
       <c r="B115" s="127" t="inlineStr">
         <is>
-          <t>其他地方台</t>
+          <t>地方频道</t>
         </is>
       </c>
       <c r="C115" s="128" t="inlineStr">
         <is>
-          <t>https://live.shaoxing.com.cn/video/s10001-sxhb/index.m3u8</t>
+          <t>http://play1-qk.nmtv.cn/live/2326general.m3u8</t>
         </is>
       </c>
     </row>
@@ -9413,31 +9413,31 @@
       </c>
       <c r="C116" s="72" t="inlineStr">
         <is>
-          <t>http://play1-qk.nmtv.cn/live/2326general.m3u8</t>
+          <t>http://ali-xwl.cztv.com/live/channel031080Plxw.m3u8</t>
         </is>
       </c>
     </row>
     <row r="117" ht="16" customHeight="1">
       <c r="A117" s="126" t="inlineStr">
         <is>
-          <t>经济生活</t>
+          <t>美丽河北</t>
         </is>
       </c>
       <c r="B117" s="127" t="inlineStr">
         <is>
-          <t>地方频道</t>
+          <t>其他地方台</t>
         </is>
       </c>
       <c r="C117" s="128" t="inlineStr">
         <is>
-          <t>http://ali-xwl.cztv.com/live/channel031080Plxw.m3u8</t>
+          <t>https://event.pull.hebtv.com:443/live/live103.m3u8</t>
         </is>
       </c>
     </row>
     <row r="118" ht="16" customHeight="1">
       <c r="A118" s="70" t="inlineStr">
         <is>
-          <t>美丽河北</t>
+          <t>荆门新闻综合</t>
         </is>
       </c>
       <c r="B118" s="71" t="inlineStr">
@@ -9447,14 +9447,14 @@
       </c>
       <c r="C118" s="72" t="inlineStr">
         <is>
-          <t>https://event.pull.hebtv.com:443/live/live103.m3u8</t>
+          <t>https://stream.jmtv.com.cn/xwzh/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="119" ht="16" customHeight="1">
       <c r="A119" s="126" t="inlineStr">
         <is>
-          <t>荆门新闻综合</t>
+          <t>萧山生活频道</t>
         </is>
       </c>
       <c r="B119" s="127" t="inlineStr">
@@ -9464,48 +9464,48 @@
       </c>
       <c r="C119" s="128" t="inlineStr">
         <is>
-          <t>https://stream.jmtv.com.cn/xwzh/playlist.m3u8</t>
+          <t>https://l.cztvcloud.com/channels/lantian/SXxiaoshan2/720p.m3u8</t>
         </is>
       </c>
     </row>
     <row r="120" ht="16" customHeight="1">
       <c r="A120" s="70" t="inlineStr">
         <is>
-          <t>萧山生活频道</t>
+          <t>萧山综合</t>
         </is>
       </c>
       <c r="B120" s="71" t="inlineStr">
         <is>
-          <t>其他地方台</t>
+          <t>地方频道</t>
         </is>
       </c>
       <c r="C120" s="72" t="inlineStr">
         <is>
-          <t>https://l.cztvcloud.com/channels/lantian/SXxiaoshan2/720p.m3u8</t>
+          <t>http://l.cztvcloud.com/channels/lantian/SXxiaoshan1/720p.m3u8</t>
         </is>
       </c>
     </row>
     <row r="121" ht="16" customHeight="1">
       <c r="A121" s="126" t="inlineStr">
         <is>
-          <t>萧山综合</t>
+          <t>蘭州文旅</t>
         </is>
       </c>
       <c r="B121" s="127" t="inlineStr">
         <is>
-          <t>地方频道</t>
+          <t>其他地方台</t>
         </is>
       </c>
       <c r="C121" s="128" t="inlineStr">
         <is>
-          <t>http://l.cztvcloud.com/channels/lantian/SXxiaoshan1/720p.m3u8</t>
+          <t>https://liveplus.lzr.com.cn/wlpd/HD/live.m3u8</t>
         </is>
       </c>
     </row>
     <row r="122" ht="16" customHeight="1">
       <c r="A122" s="70" t="inlineStr">
         <is>
-          <t>蘭州文旅</t>
+          <t>蘭州新聞綜合</t>
         </is>
       </c>
       <c r="B122" s="71" t="inlineStr">
@@ -9515,14 +9515,14 @@
       </c>
       <c r="C122" s="72" t="inlineStr">
         <is>
-          <t>https://liveplus.lzr.com.cn/wlpd/HD/live.m3u8</t>
+          <t>https://liveplus.lzr.com.cn/xwzh/HD/live.m3u8</t>
         </is>
       </c>
     </row>
     <row r="123" ht="16" customHeight="1">
       <c r="A123" s="126" t="inlineStr">
         <is>
-          <t>蘭州新聞綜合</t>
+          <t>衢州龙游综合</t>
         </is>
       </c>
       <c r="B123" s="127" t="inlineStr">
@@ -9532,14 +9532,14 @@
       </c>
       <c r="C123" s="128" t="inlineStr">
         <is>
-          <t>https://liveplus.lzr.com.cn/xwzh/HD/live.m3u8</t>
+          <t>https://l.cztvcloud.com/channels/lantian/SXlongyou1/720p.m3u8</t>
         </is>
       </c>
     </row>
     <row r="124" ht="16" customHeight="1">
       <c r="A124" s="70" t="inlineStr">
         <is>
-          <t>衢州龙游综合</t>
+          <t>西宁新闻综合</t>
         </is>
       </c>
       <c r="B124" s="71" t="inlineStr">
@@ -9549,14 +9549,14 @@
       </c>
       <c r="C124" s="72" t="inlineStr">
         <is>
-          <t>https://l.cztvcloud.com/channels/lantian/SXlongyou1/720p.m3u8</t>
+          <t>https://liveout.xntv.tv/a65jur/96iln2.m3u8</t>
         </is>
       </c>
     </row>
     <row r="125" ht="16" customHeight="1">
       <c r="A125" s="126" t="inlineStr">
         <is>
-          <t>西宁新闻综合</t>
+          <t>西藏衛視藏語台</t>
         </is>
       </c>
       <c r="B125" s="127" t="inlineStr">
@@ -9566,14 +9566,14 @@
       </c>
       <c r="C125" s="128" t="inlineStr">
         <is>
-          <t>https://liveout.xntv.tv/a65jur/96iln2.m3u8</t>
+          <t>http://php.jdshipin.com:8880/xztv.php?id=zy</t>
         </is>
       </c>
     </row>
     <row r="126" ht="16" customHeight="1">
       <c r="A126" s="70" t="inlineStr">
         <is>
-          <t>西藏衛視藏語台</t>
+          <t>讷河综合</t>
         </is>
       </c>
       <c r="B126" s="71" t="inlineStr">
@@ -9583,65 +9583,65 @@
       </c>
       <c r="C126" s="72" t="inlineStr">
         <is>
-          <t>http://php.jdshipin.com:8880/xztv.php?id=zy</t>
+          <t>https://cors-anywhere.yidianzhishi.cn/https://masterpull.hljtv.com/live/PXWxDY1V.m3u8</t>
         </is>
       </c>
     </row>
     <row r="127" ht="16" customHeight="1">
       <c r="A127" s="126" t="inlineStr">
         <is>
-          <t>讷河综合</t>
+          <t>赤峰新聞綜合</t>
         </is>
       </c>
       <c r="B127" s="127" t="inlineStr">
         <is>
-          <t>其他地方台</t>
+          <t>内蒙古频道</t>
         </is>
       </c>
       <c r="C127" s="128" t="inlineStr">
         <is>
-          <t>https://cors-anywhere.yidianzhishi.cn/https://masterpull.hljtv.com/live/PXWxDY1V.m3u8</t>
+          <t>http://play1-qk.nmtv.cn/live/1735546697341033.m3u8</t>
         </is>
       </c>
     </row>
     <row r="128" ht="16" customHeight="1">
       <c r="A128" s="70" t="inlineStr">
         <is>
-          <t>赤峰新聞綜合</t>
+          <t>赤峰新闻综合</t>
         </is>
       </c>
       <c r="B128" s="71" t="inlineStr">
         <is>
-          <t>内蒙古频道</t>
+          <t>其他地方台</t>
         </is>
       </c>
       <c r="C128" s="72" t="inlineStr">
         <is>
-          <t>http://play1-qk.nmtv.cn/live/1735546697341033.m3u8</t>
+          <t>https://play1-qk.nmtv.cn/live/1735546697341033.m3u8</t>
         </is>
       </c>
     </row>
     <row r="129" ht="16" customHeight="1">
       <c r="A129" s="126" t="inlineStr">
         <is>
-          <t>赤峰新闻综合</t>
+          <t>辉南新闻综合</t>
         </is>
       </c>
       <c r="B129" s="127" t="inlineStr">
         <is>
-          <t>其他地方台</t>
+          <t>吉林频道</t>
         </is>
       </c>
       <c r="C129" s="128" t="inlineStr">
         <is>
-          <t>https://play1-qk.nmtv.cn/live/1735546697341033.m3u8</t>
+          <t>https://cors-anywhere.yidianzhishi.cn/http://stream5.jlntv.cn/hn/sd/live.m3u8</t>
         </is>
       </c>
     </row>
     <row r="130" ht="16" customHeight="1">
       <c r="A130" s="70" t="inlineStr">
         <is>
-          <t>辉南新闻综合</t>
+          <t>辉南综合</t>
         </is>
       </c>
       <c r="B130" s="71" t="inlineStr">
@@ -9651,65 +9651,65 @@
       </c>
       <c r="C130" s="72" t="inlineStr">
         <is>
-          <t>https://cors-anywhere.yidianzhishi.cn/http://stream5.jlntv.cn/hn/sd/live.m3u8</t>
+          <t>https://cors-anywhere.yidianzhishi.cn/http://stream5.jlntv.cn/hn/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="131" ht="16" customHeight="1">
       <c r="A131" s="126" t="inlineStr">
         <is>
-          <t>辉南综合</t>
+          <t>逊克综合</t>
         </is>
       </c>
       <c r="B131" s="127" t="inlineStr">
         <is>
-          <t>吉林频道</t>
+          <t>其他地方台</t>
         </is>
       </c>
       <c r="C131" s="128" t="inlineStr">
         <is>
-          <t>https://cors-anywhere.yidianzhishi.cn/http://stream5.jlntv.cn/hn/playlist.m3u8</t>
+          <t>https://cors-anywhere.yidianzhishi.cn/https://masterpull.hljtv.com/live/a0CULO9O.m3u8</t>
         </is>
       </c>
     </row>
     <row r="132" ht="16" customHeight="1">
       <c r="A132" s="70" t="inlineStr">
         <is>
-          <t>逊克综合</t>
+          <t>通化县综合</t>
         </is>
       </c>
       <c r="B132" s="71" t="inlineStr">
         <is>
-          <t>其他地方台</t>
+          <t>吉林频道</t>
         </is>
       </c>
       <c r="C132" s="72" t="inlineStr">
         <is>
-          <t>https://cors-anywhere.yidianzhishi.cn/https://masterpull.hljtv.com/live/a0CULO9O.m3u8</t>
+          <t>https://cors-anywhere.yidianzhishi.cn/http://stream5.jlntv.cn/thx/sd/live.m3u8</t>
         </is>
       </c>
     </row>
     <row r="133" ht="16" customHeight="1">
       <c r="A133" s="126" t="inlineStr">
         <is>
-          <t>通化县综合</t>
+          <t>通辽新闻综合</t>
         </is>
       </c>
       <c r="B133" s="127" t="inlineStr">
         <is>
-          <t>吉林频道</t>
+          <t>其他地方台</t>
         </is>
       </c>
       <c r="C133" s="128" t="inlineStr">
         <is>
-          <t>https://cors-anywhere.yidianzhishi.cn/http://stream5.jlntv.cn/thx/sd/live.m3u8</t>
+          <t>https://play1-qk.nmtv.cn/live/1735546745882037.m3u8</t>
         </is>
       </c>
     </row>
     <row r="134" ht="16" customHeight="1">
       <c r="A134" s="70" t="inlineStr">
         <is>
-          <t>通辽新闻综合</t>
+          <t>邯郸公共</t>
         </is>
       </c>
       <c r="B134" s="71" t="inlineStr">
@@ -9719,14 +9719,14 @@
       </c>
       <c r="C134" s="72" t="inlineStr">
         <is>
-          <t>https://play1-qk.nmtv.cn/live/1735546745882037.m3u8</t>
+          <t>https://jwcdnqx.hebyun.com.cn/live/hdgg/1500k/tzwj_video.m3u8</t>
         </is>
       </c>
     </row>
     <row r="135" ht="16" customHeight="1">
       <c r="A135" s="126" t="inlineStr">
         <is>
-          <t>邯郸公共</t>
+          <t>鄂尔多斯新闻综合</t>
         </is>
       </c>
       <c r="B135" s="127" t="inlineStr">
@@ -9736,82 +9736,82 @@
       </c>
       <c r="C135" s="128" t="inlineStr">
         <is>
-          <t>https://jwcdnqx.hebyun.com.cn/live/hdgg/1500k/tzwj_video.m3u8</t>
+          <t>https://play1-qk.nmtv.cn/live/1735546299241021.m3u8</t>
         </is>
       </c>
     </row>
     <row r="136" ht="16" customHeight="1">
       <c r="A136" s="70" t="inlineStr">
         <is>
-          <t>鄂尔多斯新闻综合</t>
+          <t>钱江都市</t>
         </is>
       </c>
       <c r="B136" s="71" t="inlineStr">
         <is>
-          <t>其他地方台</t>
+          <t>地方频道</t>
         </is>
       </c>
       <c r="C136" s="72" t="inlineStr">
         <is>
-          <t>https://play1-qk.nmtv.cn/live/1735546299241021.m3u8</t>
+          <t>http://ali-xwl.cztv.com/live/channel021080Plxw.m3u8</t>
         </is>
       </c>
     </row>
     <row r="137" ht="16" customHeight="1">
       <c r="A137" s="126" t="inlineStr">
         <is>
-          <t>钱江都市</t>
+          <t>锡林郭勒盟一套</t>
         </is>
       </c>
       <c r="B137" s="127" t="inlineStr">
         <is>
-          <t>地方频道</t>
+          <t>其他地方台</t>
         </is>
       </c>
       <c r="C137" s="128" t="inlineStr">
         <is>
-          <t>http://ali-xwl.cztv.com/live/channel021080Plxw.m3u8</t>
+          <t>https://play1-qk.nmtv.cn/live/1735546994821050.m3u8</t>
         </is>
       </c>
     </row>
     <row r="138" ht="16" customHeight="1">
       <c r="A138" s="70" t="inlineStr">
         <is>
-          <t>锡林郭勒盟一套</t>
+          <t>长春综合</t>
         </is>
       </c>
       <c r="B138" s="71" t="inlineStr">
         <is>
-          <t>其他地方台</t>
+          <t>吉林频道</t>
         </is>
       </c>
       <c r="C138" s="72" t="inlineStr">
         <is>
-          <t>https://play1-qk.nmtv.cn/live/1735546994821050.m3u8</t>
+          <t>https://stream2.jlntv.cn/jlcc/sd/live.m3u8</t>
         </is>
       </c>
     </row>
     <row r="139" ht="16" customHeight="1">
       <c r="A139" s="126" t="inlineStr">
         <is>
-          <t>长春综合</t>
+          <t>长沙政法</t>
         </is>
       </c>
       <c r="B139" s="127" t="inlineStr">
         <is>
-          <t>吉林频道</t>
+          <t>芒果TV</t>
         </is>
       </c>
       <c r="C139" s="128" t="inlineStr">
         <is>
-          <t>https://stream2.jlntv.cn/jlcc/sd/live.m3u8</t>
+          <t>https://padhw.qing.mgtv.com/nn_live/nn_x64/Y2hzPSZkZWY9MSZ1aXA9NDcuMTA4LjcyLjQ1JnRlcm09NCZtYWNpZD1kOWRjZGYwNi03YzI0LTQ2MWItOTJiYy02NTM0MGQyMWY1NTkmcWlkPSZyYXV0aF9lbmFibGU9b24mY2RuZXhfaWQ9aHdfcGhvbmUmZXM9MTc5MDczNzI3NyZ1dWlkPTRlMWQ5YTYxNGZmNTNlNTE5MWJhMWRhMGUxZTBhNTIyLTJmNmM0ODJkJnM9Mzg3NGQ1MjJhYWJhY2QxNTQyYWM0M2ZiMDJmNGJiNjcmdWlkPSZuZHY9cGNfd2ViLWltZ290di1wY2g1LTEuMi4zJnY9MiZhcz0wJl9jYXJDb2RlPTA,/CSZFMPP360.m3u8</t>
         </is>
       </c>
     </row>
     <row r="140" ht="16" customHeight="1">
       <c r="A140" s="70" t="inlineStr">
         <is>
-          <t>长沙政法</t>
+          <t>长沙新闻综合</t>
         </is>
       </c>
       <c r="B140" s="71" t="inlineStr">
@@ -9821,48 +9821,48 @@
       </c>
       <c r="C140" s="72" t="inlineStr">
         <is>
-          <t>https://padhw.qing.mgtv.com/nn_live/nn_x64/Y2hzPSZkZWY9MSZ1aXA9NDcuMTA4LjcyLjQ1JnRlcm09NCZtYWNpZD1kOWRjZGYwNi03YzI0LTQ2MWItOTJiYy02NTM0MGQyMWY1NTkmcWlkPSZyYXV0aF9lbmFibGU9b24mY2RuZXhfaWQ9aHdfcGhvbmUmZXM9MTc5MDczNzI3NyZ1dWlkPTRlMWQ5YTYxNGZmNTNlNTE5MWJhMWRhMGUxZTBhNTIyLTJmNmM0ODJkJnM9Mzg3NGQ1MjJhYWJhY2QxNTQyYWM0M2ZiMDJmNGJiNjcmdWlkPSZuZHY9cGNfd2ViLWltZ290di1wY2g1LTEuMi4zJnY9MiZhcz0wJl9jYXJDb2RlPTA,/CSZFMPP360.m3u8</t>
+          <t>https://padqq.qing.mgtv.com/nn_live/nn_x64/Y2hzPSZkZWY9MSZ1aXA9NDcuMTA4LjcyLjQ1JnRlcm09NCZtYWNpZD1kOWRjZGYwNi03YzI0LTQ2MWItOTJiYy02NTM0MGQyMWY1NTkmcWlkPSZyYXV0aF9lbmFibGU9b24mY2RuZXhfaWQ9cXFfcGhvbmVfbGl2ZSZlcz0xNzkwNzM3Mjc2JnV1aWQ9NGY5ZjBkZjgzYzZjNDY2ZDI2ZmY2ZDZmZjY4ZGM5MTAtMmY2YzQ4MmQmcz1hNzgyZGQxZWExZGI5NGQ0NDZiNTJhYzI3NTg5ZDU3MiZ1aWQ9Jm5kdj1wY193ZWItaW1nb3R2LXBjaDUtMS4yLjMmdj0yJmFzPTAmX2NhckNvZGU9MA,,/CSXWMPP360.m3u8</t>
         </is>
       </c>
     </row>
     <row r="141" ht="16" customHeight="1">
       <c r="A141" s="126" t="inlineStr">
         <is>
-          <t>长沙新闻综合</t>
+          <t>阿拉善新闻综合</t>
         </is>
       </c>
       <c r="B141" s="127" t="inlineStr">
         <is>
-          <t>芒果TV</t>
+          <t>其他地方台</t>
         </is>
       </c>
       <c r="C141" s="128" t="inlineStr">
         <is>
-          <t>https://padqq.qing.mgtv.com/nn_live/nn_x64/Y2hzPSZkZWY9MSZ1aXA9NDcuMTA4LjcyLjQ1JnRlcm09NCZtYWNpZD1kOWRjZGYwNi03YzI0LTQ2MWItOTJiYy02NTM0MGQyMWY1NTkmcWlkPSZyYXV0aF9lbmFibGU9b24mY2RuZXhfaWQ9cXFfcGhvbmVfbGl2ZSZlcz0xNzkwNzM3Mjc2JnV1aWQ9NGY5ZjBkZjgzYzZjNDY2ZDI2ZmY2ZDZmZjY4ZGM5MTAtMmY2YzQ4MmQmcz1hNzgyZGQxZWExZGI5NGQ0NDZiNTJhYzI3NTg5ZDU3MiZ1aWQ9Jm5kdj1wY193ZWItaW1nb3R2LXBjaDUtMS4yLjMmdj0yJmFzPTAmX2NhckNvZGU9MA,,/CSXWMPP360.m3u8</t>
+          <t>https://play1-qk.nmtv.cn/live/1735547046115053.m3u8</t>
         </is>
       </c>
     </row>
     <row r="142" ht="16" customHeight="1">
       <c r="A142" s="70" t="inlineStr">
         <is>
-          <t>阿拉善新闻综合</t>
+          <t>陇南公共</t>
         </is>
       </c>
       <c r="B142" s="71" t="inlineStr">
         <is>
-          <t>其他地方台</t>
+          <t>甘肃频道</t>
         </is>
       </c>
       <c r="C142" s="72" t="inlineStr">
         <is>
-          <t>https://play1-qk.nmtv.cn/live/1735547046115053.m3u8</t>
+          <t>https://play.kankanlive.com/live/1709171893138901.m3u8</t>
         </is>
       </c>
     </row>
     <row r="143" ht="16" customHeight="1">
       <c r="A143" s="126" t="inlineStr">
         <is>
-          <t>陇南公共</t>
+          <t>陇南综合</t>
         </is>
       </c>
       <c r="B143" s="127" t="inlineStr">
@@ -9872,48 +9872,48 @@
       </c>
       <c r="C143" s="128" t="inlineStr">
         <is>
-          <t>https://play.kankanlive.com/live/1709171893138901.m3u8</t>
+          <t>https://play.kankanlive.com/live/1709171819929902.m3u8</t>
         </is>
       </c>
     </row>
     <row r="144" ht="16" customHeight="1">
       <c r="A144" s="70" t="inlineStr">
         <is>
-          <t>陇南综合</t>
+          <t>雅安新闻综合</t>
         </is>
       </c>
       <c r="B144" s="71" t="inlineStr">
         <is>
-          <t>甘肃频道</t>
+          <t>四川频道</t>
         </is>
       </c>
       <c r="C144" s="72" t="inlineStr">
         <is>
-          <t>https://play.kankanlive.com/live/1709171819929902.m3u8</t>
+          <t>https://play.yunxya.com/channellive/xinwen.m3u8</t>
         </is>
       </c>
     </row>
     <row r="145" ht="16" customHeight="1">
       <c r="A145" s="126" t="inlineStr">
         <is>
-          <t>雅安新闻综合</t>
+          <t>集安新闻</t>
         </is>
       </c>
       <c r="B145" s="127" t="inlineStr">
         <is>
-          <t>四川频道</t>
+          <t>其他地方台</t>
         </is>
       </c>
       <c r="C145" s="128" t="inlineStr">
         <is>
-          <t>https://play.yunxya.com/channellive/xinwen.m3u8</t>
+          <t>https://stream2.jlntv.cn/ja/sd/live.m3u8</t>
         </is>
       </c>
     </row>
     <row r="146" ht="16" customHeight="1">
       <c r="A146" s="70" t="inlineStr">
         <is>
-          <t>集安新闻</t>
+          <t>青島影視</t>
         </is>
       </c>
       <c r="B146" s="71" t="inlineStr">
@@ -9923,14 +9923,14 @@
       </c>
       <c r="C146" s="72" t="inlineStr">
         <is>
-          <t>https://stream2.jlntv.cn/ja/sd/live.m3u8</t>
+          <t>http://video10.qtv.com.cn/drm/qtv3at/manifest.m3u8</t>
         </is>
       </c>
     </row>
     <row r="147" ht="16" customHeight="1">
       <c r="A147" s="126" t="inlineStr">
         <is>
-          <t>青島影視</t>
+          <t>青島影視資訊</t>
         </is>
       </c>
       <c r="B147" s="127" t="inlineStr">
@@ -9940,14 +9940,14 @@
       </c>
       <c r="C147" s="128" t="inlineStr">
         <is>
-          <t>http://video10.qtv.com.cn/drm/qtv3at/manifest.m3u8</t>
+          <t>http://video10.qtv.com.cn/drm/qtv5at/manifest.m3u8</t>
         </is>
       </c>
     </row>
     <row r="148" ht="16" customHeight="1">
       <c r="A148" s="70" t="inlineStr">
         <is>
-          <t>青島影視資訊</t>
+          <t>青島新聞綜合</t>
         </is>
       </c>
       <c r="B148" s="71" t="inlineStr">
@@ -9957,14 +9957,14 @@
       </c>
       <c r="C148" s="72" t="inlineStr">
         <is>
-          <t>http://video10.qtv.com.cn/drm/qtv5at/manifest.m3u8</t>
+          <t>http://video10.qtv.com.cn/drm/qtv1at/manifest.m3u8</t>
         </is>
       </c>
     </row>
     <row r="149" ht="16" customHeight="1">
       <c r="A149" s="126" t="inlineStr">
         <is>
-          <t>青島新聞綜合</t>
+          <t>青島生活</t>
         </is>
       </c>
       <c r="B149" s="127" t="inlineStr">
@@ -9974,14 +9974,14 @@
       </c>
       <c r="C149" s="128" t="inlineStr">
         <is>
-          <t>http://video10.qtv.com.cn/drm/qtv1at/manifest.m3u8</t>
+          <t>http://video10.qtv.com.cn/drm/qtv2at/manifest.m3u8</t>
         </is>
       </c>
     </row>
     <row r="150" ht="16" customHeight="1">
       <c r="A150" s="70" t="inlineStr">
         <is>
-          <t>青島生活</t>
+          <t>青島都市</t>
         </is>
       </c>
       <c r="B150" s="71" t="inlineStr">
@@ -9991,14 +9991,14 @@
       </c>
       <c r="C150" s="72" t="inlineStr">
         <is>
-          <t>http://video10.qtv.com.cn/drm/qtv2at/manifest.m3u8</t>
+          <t>http://video10.qtv.com.cn/drm/qtv4at/manifest.m3u8</t>
         </is>
       </c>
     </row>
     <row r="151" ht="16" customHeight="1">
       <c r="A151" s="126" t="inlineStr">
         <is>
-          <t>青島都市</t>
+          <t>青島青少旅遊</t>
         </is>
       </c>
       <c r="B151" s="127" t="inlineStr">
@@ -10008,14 +10008,14 @@
       </c>
       <c r="C151" s="128" t="inlineStr">
         <is>
-          <t>http://video10.qtv.com.cn/drm/qtv4at/manifest.m3u8</t>
+          <t>http://video10.qtv.com.cn/drm/qtv6at/manifest.m3u8</t>
         </is>
       </c>
     </row>
     <row r="152" ht="16" customHeight="1">
       <c r="A152" s="70" t="inlineStr">
         <is>
-          <t>青島青少旅遊</t>
+          <t>鶴壁新聞綜合</t>
         </is>
       </c>
       <c r="B152" s="71" t="inlineStr">
@@ -10025,14 +10025,14 @@
       </c>
       <c r="C152" s="72" t="inlineStr">
         <is>
-          <t>http://video10.qtv.com.cn/drm/qtv6at/manifest.m3u8</t>
+          <t>http://pili-live-hls.hebitv.com/hebi/hebi.m3u8</t>
         </is>
       </c>
     </row>
     <row r="153" ht="16" customHeight="1">
       <c r="A153" s="126" t="inlineStr">
         <is>
-          <t>鶴壁新聞綜合</t>
+          <t>龙江综合</t>
         </is>
       </c>
       <c r="B153" s="127" t="inlineStr">
@@ -10041,23 +10041,6 @@
         </is>
       </c>
       <c r="C153" s="128" t="inlineStr">
-        <is>
-          <t>http://pili-live-hls.hebitv.com/hebi/hebi.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="154" ht="16" customHeight="1">
-      <c r="A154" s="70" t="inlineStr">
-        <is>
-          <t>龙江综合</t>
-        </is>
-      </c>
-      <c r="B154" s="71" t="inlineStr">
-        <is>
-          <t>其他地方台</t>
-        </is>
-      </c>
-      <c r="C154" s="72" t="inlineStr">
         <is>
           <t>https://cors-anywhere.yidianzhishi.cn/https://masterpull.hljtv.com/live/vRSdDMSR.m3u8</t>
         </is>
@@ -68448,7 +68431,7 @@
       </c>
       <c r="C15" s="76" t="inlineStr">
         <is>
-          <t>https://ali-m-l.cztv.com/channels/lantian/channel001/1080p.m3u8</t>
+          <t>https://ali-xwl.cztv.com/live/channel011080Plxw.m3u8</t>
         </is>
       </c>
     </row>
@@ -68533,24 +68516,24 @@
       </c>
       <c r="C20" s="72" t="inlineStr">
         <is>
-          <t>https://ali-xwl.cztv.com/live/channel011080Plxw.m3u8</t>
+          <t>https://ali-xwl.cztv.com/live/channel01720Plxw.m3u8</t>
         </is>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="74" t="inlineStr">
         <is>
-          <t>浙江卫视_2</t>
+          <t>海峡卫视</t>
         </is>
       </c>
       <c r="B21" s="75" t="inlineStr">
         <is>
-          <t>卫视频道</t>
+          <t>港澳台</t>
         </is>
       </c>
       <c r="C21" s="76" t="inlineStr">
         <is>
-          <t>https://ali-xwl.cztv.com/live/channel01720Plxw.m3u8</t>
+          <t>https://php.jdshipin.com/TVOD/iptv.php?id=hxws</t>
         </is>
       </c>
     </row>
@@ -68567,24 +68550,24 @@
       </c>
       <c r="C22" s="72" t="inlineStr">
         <is>
-          <t>https://php.jdshipin.com/TVOD/iptv.php?id=hxws</t>
+          <t>https://7612-5516-affc-d88b.kylintv.tv/live/fjstv_iphone.m3u8</t>
         </is>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="74" t="inlineStr">
         <is>
-          <t>海峡卫视</t>
+          <t>湖南卫视</t>
         </is>
       </c>
       <c r="B23" s="75" t="inlineStr">
         <is>
-          <t>港澳台</t>
+          <t>卫视频道</t>
         </is>
       </c>
       <c r="C23" s="76" t="inlineStr">
         <is>
-          <t>https://7612-5516-affc-d88b.kylintv.tv/live/fjstv_iphone.m3u8</t>
+          <t>http://hlsal-ldvt.qing.mgtv.com/nn_live/nn_x64/dWlwPTEyNy4wLjAuMSZ1aWQ9cWluZy1jbXMmbm5fdGltZXpvbmU9OCZjZG5leF9pZD1hbF9obHNfbGR2dCZ1dWlkPTliODY4NmU5ZTM2YzYwMmMmZT02OTE0NjA0JnY9MSZpZD1ITldTWkdTVCZzPTcwN2RiYTc2YzJjNmJmMTQ4MmUyZGYzOWU2NWM3YWFi/HNWSZGST.m3u8</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: remove fake no-signal placeholder streams (weilai sports) and enhance ad detection with 3y1.xyz signatures
</commit_message>
<xml_diff>
--- a/channels_overview.xlsx
+++ b/channels_overview.xlsx
@@ -1399,7 +1399,7 @@
         </is>
       </c>
       <c r="B11" s="28" t="n">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="C11" s="29" t="inlineStr">
         <is>
@@ -1594,7 +1594,7 @@
         </is>
       </c>
       <c r="B24" s="64" t="n">
-        <v>3458</v>
+        <v>3452</v>
       </c>
       <c r="C24" s="64" t="n"/>
     </row>
@@ -1612,7 +1612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C116"/>
+  <dimension ref="A1:C110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1623,7 +1623,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="101" t="inlineStr">
         <is>
-          <t>📺  🏅 体育频道  —  共 114 条频道</t>
+          <t>📺  🏅 体育频道  —  共 108 条频道</t>
         </is>
       </c>
     </row>
@@ -3432,7 +3432,7 @@
     <row r="108" ht="16" customHeight="1">
       <c r="A108" s="70" t="inlineStr">
         <is>
-          <t>精品体育</t>
+          <t>🌘 FOX Sports (线路3)</t>
         </is>
       </c>
       <c r="B108" s="71" t="inlineStr">
@@ -3442,14 +3442,14 @@
       </c>
       <c r="C108" s="72" t="inlineStr">
         <is>
-          <t>https://epg.pw/stream/f7556eccd4ae06b0c2991fdc7a4f8388496559f728cc82459a8e50346040e226.m3u8</t>
+          <t>https://d1jzu95oc8fgt3.cloudfront.net/FOX_Sports720p.m3u8</t>
         </is>
       </c>
     </row>
     <row r="109" ht="16" customHeight="1">
       <c r="A109" s="102" t="inlineStr">
         <is>
-          <t>精品体育</t>
+          <t>🏆 NBC Sports NOW</t>
         </is>
       </c>
       <c r="B109" s="103" t="inlineStr">
@@ -3459,14 +3459,14 @@
       </c>
       <c r="C109" s="104" t="inlineStr">
         <is>
-          <t>https://epg.pw/stream/94ed0232b61ce8d89883160a4cdfbfc8f3225cae70ef8e17d93eec249a3c8ad6.m3u8</t>
+          <t>https://xumo-xumoent-vc-122-sjv70.fast.nbcuni.com/live/master.m3u8</t>
         </is>
       </c>
     </row>
     <row r="110" ht="16" customHeight="1">
       <c r="A110" s="70" t="inlineStr">
         <is>
-          <t>精品体育</t>
+          <t>🏆 NBC Sports NOW_1</t>
         </is>
       </c>
       <c r="B110" s="71" t="inlineStr">
@@ -3475,108 +3475,6 @@
         </is>
       </c>
       <c r="C110" s="72" t="inlineStr">
-        <is>
-          <t>https://epg.pw/stream/866a097a0907c9832440f8df38272dd555abf05200dfbafcc137e214c9b30ca7.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="16" customHeight="1">
-      <c r="A111" s="102" t="inlineStr">
-        <is>
-          <t>纬来体育</t>
-        </is>
-      </c>
-      <c r="B111" s="103" t="inlineStr">
-        <is>
-          <t>体育频道</t>
-        </is>
-      </c>
-      <c r="C111" s="104" t="inlineStr">
-        <is>
-          <t>https://epg.pw/stream/8855a9936e37e608a0ec8a014cce1673dee9c5d68d560da376cc92e5edef2b25.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="16" customHeight="1">
-      <c r="A112" s="70" t="inlineStr">
-        <is>
-          <t>纬来体育</t>
-        </is>
-      </c>
-      <c r="B112" s="71" t="inlineStr">
-        <is>
-          <t>体育频道</t>
-        </is>
-      </c>
-      <c r="C112" s="72" t="inlineStr">
-        <is>
-          <t>https://epg.pw/stream/ab6df63b64d0cc44a1f4f029ed847a26fa54a7aebd455578fb05a63f02c22f4b.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="16" customHeight="1">
-      <c r="A113" s="102" t="inlineStr">
-        <is>
-          <t>纬来体育</t>
-        </is>
-      </c>
-      <c r="B113" s="103" t="inlineStr">
-        <is>
-          <t>体育频道</t>
-        </is>
-      </c>
-      <c r="C113" s="104" t="inlineStr">
-        <is>
-          <t>https://epg.pw/stream/4f18dfe0593db5c686eb64ae8edaf2a9202d4d46bdc9bbde2cee27708e12ea01.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" ht="16" customHeight="1">
-      <c r="A114" s="70" t="inlineStr">
-        <is>
-          <t>🌘 FOX Sports (线路3)</t>
-        </is>
-      </c>
-      <c r="B114" s="71" t="inlineStr">
-        <is>
-          <t>体育频道</t>
-        </is>
-      </c>
-      <c r="C114" s="72" t="inlineStr">
-        <is>
-          <t>https://d1jzu95oc8fgt3.cloudfront.net/FOX_Sports720p.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" ht="16" customHeight="1">
-      <c r="A115" s="102" t="inlineStr">
-        <is>
-          <t>🏆 NBC Sports NOW</t>
-        </is>
-      </c>
-      <c r="B115" s="103" t="inlineStr">
-        <is>
-          <t>体育频道</t>
-        </is>
-      </c>
-      <c r="C115" s="104" t="inlineStr">
-        <is>
-          <t>https://xumo-xumoent-vc-122-sjv70.fast.nbcuni.com/live/master.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="116" ht="16" customHeight="1">
-      <c r="A116" s="70" t="inlineStr">
-        <is>
-          <t>🏆 NBC Sports NOW_1</t>
-        </is>
-      </c>
-      <c r="B116" s="71" t="inlineStr">
-        <is>
-          <t>体育频道</t>
-        </is>
-      </c>
-      <c r="C116" s="72" t="inlineStr">
         <is>
           <t>https://d4whmvwm0rdvi.cloudfront.net/10007/99993008/hls/master.m3u8?ads.xumo_channelId=99993008</t>
         </is>

</xml_diff>

<commit_message>
fix: demote dsdqpub ad loop streams and enforce pure CCTV-4 1080P stream on Line 1
</commit_message>
<xml_diff>
--- a/channels_overview.xlsx
+++ b/channels_overview.xlsx
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
@@ -1694,7 +1694,7 @@
         </is>
       </c>
       <c r="B28" s="67" t="n">
-        <v>3212</v>
+        <v>3214</v>
       </c>
       <c r="C28" s="67" t="n"/>
     </row>
@@ -9108,7 +9108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C141"/>
+  <dimension ref="A1:C143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -9119,7 +9119,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="68" t="inlineStr">
         <is>
-          <t>📺  📡 中国大陆 · 央视  —  共 139 条频道</t>
+          <t>📺  📡 中国大陆 · 央视  —  共 141 条频道</t>
         </is>
       </c>
     </row>
@@ -10360,7 +10360,7 @@
       </c>
       <c r="C74" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/cctv4k.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv4hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
@@ -10377,7 +10377,7 @@
       </c>
       <c r="C75" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv4hd.m3u8</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv4hd</t>
         </is>
       </c>
     </row>
@@ -10394,7 +10394,7 @@
       </c>
       <c r="C76" s="75" t="inlineStr">
         <is>
-          <t>http://hlszymgsplive.miguvideo.com:8080/wd_r2/cctv/cctv4hd/1500/index.m3u8?msisdn=51f96c2ab292f10eaf525e4df0046fa1&amp;mdspid=&amp;spid=699004&amp;netType=0&amp;sid=5500346947&amp;pid=2028597139&amp;timestamp=20261001065030&amp;Channel_ID=0116_2600034600-99000-201600010010028&amp;ProgramID=631780421&amp;ParentNodeID=-99&amp;assertID=5500346947&amp;client_ip=39.103.188.159&amp;SecurityKey=20261001065030&amp;promotionId=&amp;mvid=5101064235&amp;mcid=500020&amp;playurlVersion=WX-A1-9.9.2-SNAPSHOT&amp;userid=&amp;jmhm=&amp;videocodec=h264&amp;appCode=miguvideo_android&amp;bean=mgspad&amp;tid=android&amp;conFee=0&amp;encrypt=a63fbde55785ce83396bc05f752847b3&amp;sv=10004&amp;ct=android</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/cctv4k.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
@@ -10411,14 +10411,14 @@
       </c>
       <c r="C77" s="72" t="inlineStr">
         <is>
-          <t>http://173.208.212.130:8181/1080p/cctv4.m3u8</t>
+          <t>http://107.150.60.122/live/cctv4hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="78" ht="16" customHeight="1">
       <c r="A78" s="73" t="inlineStr">
         <is>
-          <t>CCTV-5</t>
+          <t>CCTV-4</t>
         </is>
       </c>
       <c r="B78" s="74" t="inlineStr">
@@ -10428,14 +10428,14 @@
       </c>
       <c r="C78" s="75" t="inlineStr">
         <is>
-          <t>http://118.122.144.115:8888/newlive/live/hls/5/live.m3u8</t>
+          <t>http://hlszymgsplive.miguvideo.com:8080/wd_r2/cctv/cctv4hd/1500/index.m3u8?msisdn=51f96c2ab292f10eaf525e4df0046fa1&amp;mdspid=&amp;spid=699004&amp;netType=0&amp;sid=5500346947&amp;pid=2028597139&amp;timestamp=20261001065030&amp;Channel_ID=0116_2600034600-99000-201600010010028&amp;ProgramID=631780421&amp;ParentNodeID=-99&amp;assertID=5500346947&amp;client_ip=39.103.188.159&amp;SecurityKey=20261001065030&amp;promotionId=&amp;mvid=5101064235&amp;mcid=500020&amp;playurlVersion=WX-A1-9.9.2-SNAPSHOT&amp;userid=&amp;jmhm=&amp;videocodec=h264&amp;appCode=miguvideo_android&amp;bean=mgspad&amp;tid=android&amp;conFee=0&amp;encrypt=a63fbde55785ce83396bc05f752847b3&amp;sv=10004&amp;ct=android</t>
         </is>
       </c>
     </row>
     <row r="79" ht="16" customHeight="1">
       <c r="A79" s="70" t="inlineStr">
         <is>
-          <t>CCTV-5</t>
+          <t>CCTV-4</t>
         </is>
       </c>
       <c r="B79" s="71" t="inlineStr">
@@ -10445,7 +10445,7 @@
       </c>
       <c r="C79" s="72" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0005_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://173.208.212.130:8181/1080p/cctv4.m3u8</t>
         </is>
       </c>
     </row>
@@ -10462,7 +10462,7 @@
       </c>
       <c r="C80" s="75" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv5hd.m3u8</t>
+          <t>http://118.122.144.115:8888/newlive/live/hls/5/live.m3u8</t>
         </is>
       </c>
     </row>
@@ -10479,14 +10479,14 @@
       </c>
       <c r="C81" s="72" t="inlineStr">
         <is>
-          <t>http://173.208.212.130:8181/720p/cctv5.m3u8</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0005_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="82" ht="16" customHeight="1">
       <c r="A82" s="73" t="inlineStr">
         <is>
-          <t>CCTV-5+</t>
+          <t>CCTV-5</t>
         </is>
       </c>
       <c r="B82" s="74" t="inlineStr">
@@ -10496,14 +10496,14 @@
       </c>
       <c r="C82" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0016_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://107.150.60.122/live/cctv5hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="83" ht="16" customHeight="1">
       <c r="A83" s="70" t="inlineStr">
         <is>
-          <t>CCTV-5+体育赛事</t>
+          <t>CCTV-5</t>
         </is>
       </c>
       <c r="B83" s="71" t="inlineStr">
@@ -10513,14 +10513,14 @@
       </c>
       <c r="C83" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv5p.m3u8?auth=test20251009</t>
+          <t>http://173.208.212.130:8181/720p/cctv5.m3u8</t>
         </is>
       </c>
     </row>
     <row r="84" ht="16" customHeight="1">
       <c r="A84" s="73" t="inlineStr">
         <is>
-          <t>CCTV-5体育</t>
+          <t>CCTV-5+</t>
         </is>
       </c>
       <c r="B84" s="74" t="inlineStr">
@@ -10530,14 +10530,14 @@
       </c>
       <c r="C84" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv5hd.m3u8?auth=test20251009</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0016_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="85" ht="16" customHeight="1">
       <c r="A85" s="70" t="inlineStr">
         <is>
-          <t>CCTV-5体育</t>
+          <t>CCTV-5+体育赛事</t>
         </is>
       </c>
       <c r="B85" s="71" t="inlineStr">
@@ -10547,14 +10547,14 @@
       </c>
       <c r="C85" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/cctv5p.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv5p.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
     <row r="86" ht="16" customHeight="1">
       <c r="A86" s="73" t="inlineStr">
         <is>
-          <t>CCTV-6</t>
+          <t>CCTV-5体育</t>
         </is>
       </c>
       <c r="B86" s="74" t="inlineStr">
@@ -10564,14 +10564,14 @@
       </c>
       <c r="C86" s="75" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0006_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv5hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
     <row r="87" ht="16" customHeight="1">
       <c r="A87" s="70" t="inlineStr">
         <is>
-          <t>CCTV-6</t>
+          <t>CCTV-5体育</t>
         </is>
       </c>
       <c r="B87" s="71" t="inlineStr">
@@ -10581,7 +10581,7 @@
       </c>
       <c r="C87" s="72" t="inlineStr">
         <is>
-          <t>http://112.123.243.37:50085/tsfile/live/0007_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/cctv5p.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
@@ -10598,7 +10598,7 @@
       </c>
       <c r="C88" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv6hd.m3u8</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0006_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -10615,7 +10615,7 @@
       </c>
       <c r="C89" s="72" t="inlineStr">
         <is>
-          <t>http://69.30.245.50/live/cctv6.m3u8</t>
+          <t>http://112.123.243.37:50085/tsfile/live/0007_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -10632,7 +10632,7 @@
       </c>
       <c r="C90" s="75" t="inlineStr">
         <is>
-          <t>http://198.204.240.250:82/live/cctv6.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv6hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -10649,7 +10649,7 @@
       </c>
       <c r="C91" s="72" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv6hd</t>
+          <t>http://69.30.245.50/live/cctv6.m3u8</t>
         </is>
       </c>
     </row>
@@ -10666,14 +10666,14 @@
       </c>
       <c r="C92" s="75" t="inlineStr">
         <is>
-          <t>http://hlszymgsplive.miguvideo.com:8080/wd_r2/2018/ocn/cctv6hd/2000/index.m3u8?msisdn=be4dbeb27ebc53e05461c938f561f2ff&amp;mdspid=&amp;spid=699004&amp;netType=0&amp;sid=5500212872&amp;pid=2028597139&amp;timestamp=20261001065031&amp;Channel_ID=0116_2600034600-99000-201600010010028&amp;ProgramID=624878396&amp;ParentNodeID=-99&amp;assertID=5500212872&amp;client_ip=39.103.182.111&amp;SecurityKey=20261001065031&amp;promotionId=&amp;mvid=5100001694&amp;mcid=500020&amp;playurlVersion=WX-A1-9.9.2-SNAPSHOT&amp;userid=&amp;jmhm=&amp;videocodec=h264&amp;appCode=miguvideo_android&amp;bean=mgspad&amp;tid=android&amp;conFee=0&amp;encrypt=90bb6bfac8b1ad30d8fd36dd33c1d758&amp;sv=10004&amp;ct=android</t>
+          <t>http://198.204.240.250:82/live/cctv6.m3u8</t>
         </is>
       </c>
     </row>
     <row r="93" ht="16" customHeight="1">
       <c r="A93" s="70" t="inlineStr">
         <is>
-          <t>CCTV-7</t>
+          <t>CCTV-6</t>
         </is>
       </c>
       <c r="B93" s="71" t="inlineStr">
@@ -10683,14 +10683,14 @@
       </c>
       <c r="C93" s="72" t="inlineStr">
         <is>
-          <t>http://112.123.243.37:50085/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv6hd</t>
         </is>
       </c>
     </row>
     <row r="94" ht="16" customHeight="1">
       <c r="A94" s="73" t="inlineStr">
         <is>
-          <t>CCTV-7</t>
+          <t>CCTV-6</t>
         </is>
       </c>
       <c r="B94" s="74" t="inlineStr">
@@ -10700,7 +10700,7 @@
       </c>
       <c r="C94" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv7hd.m3u8</t>
+          <t>http://hlszymgsplive.miguvideo.com:8080/wd_r2/2018/ocn/cctv6hd/2000/index.m3u8?msisdn=be4dbeb27ebc53e05461c938f561f2ff&amp;mdspid=&amp;spid=699004&amp;netType=0&amp;sid=5500212872&amp;pid=2028597139&amp;timestamp=20261001065031&amp;Channel_ID=0116_2600034600-99000-201600010010028&amp;ProgramID=624878396&amp;ParentNodeID=-99&amp;assertID=5500212872&amp;client_ip=39.103.182.111&amp;SecurityKey=20261001065031&amp;promotionId=&amp;mvid=5100001694&amp;mcid=500020&amp;playurlVersion=WX-A1-9.9.2-SNAPSHOT&amp;userid=&amp;jmhm=&amp;videocodec=h264&amp;appCode=miguvideo_android&amp;bean=mgspad&amp;tid=android&amp;conFee=0&amp;encrypt=90bb6bfac8b1ad30d8fd36dd33c1d758&amp;sv=10004&amp;ct=android</t>
         </is>
       </c>
     </row>
@@ -10717,7 +10717,7 @@
       </c>
       <c r="C95" s="72" t="inlineStr">
         <is>
-          <t>http://69.30.245.50/live/cctv7.m3u8</t>
+          <t>http://112.123.243.37:50085/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -10734,7 +10734,7 @@
       </c>
       <c r="C96" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv7hd</t>
+          <t>http://74.91.26.218:82/live/cctv7hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -10751,14 +10751,14 @@
       </c>
       <c r="C97" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv7hd.m3u8</t>
+          <t>http://69.30.245.50/live/cctv7.m3u8</t>
         </is>
       </c>
     </row>
     <row r="98" ht="16" customHeight="1">
       <c r="A98" s="73" t="inlineStr">
         <is>
-          <t>CCTV-8</t>
+          <t>CCTV-7</t>
         </is>
       </c>
       <c r="B98" s="74" t="inlineStr">
@@ -10768,14 +10768,14 @@
       </c>
       <c r="C98" s="75" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv7hd</t>
         </is>
       </c>
     </row>
     <row r="99" ht="16" customHeight="1">
       <c r="A99" s="70" t="inlineStr">
         <is>
-          <t>CCTV-8</t>
+          <t>CCTV-7</t>
         </is>
       </c>
       <c r="B99" s="71" t="inlineStr">
@@ -10785,7 +10785,7 @@
       </c>
       <c r="C99" s="72" t="inlineStr">
         <is>
-          <t>http://112.123.243.37:50085/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://107.150.60.122/live/cctv7hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -10802,7 +10802,7 @@
       </c>
       <c r="C100" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv8hd.m3u8</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -10819,7 +10819,7 @@
       </c>
       <c r="C101" s="72" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv8k</t>
+          <t>http://112.123.243.37:50085/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -10836,7 +10836,7 @@
       </c>
       <c r="C102" s="75" t="inlineStr">
         <is>
-          <t>http://69.30.245.50/live/cctv8.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv8hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -10853,7 +10853,7 @@
       </c>
       <c r="C103" s="72" t="inlineStr">
         <is>
-          <t>http://bztv.tvbus.cc:8081/cdnlive/cctv8.m3u8</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv8k</t>
         </is>
       </c>
     </row>
@@ -10870,14 +10870,14 @@
       </c>
       <c r="C104" s="75" t="inlineStr">
         <is>
-          <t>http://120.40.39.246:352/newlive/live/hls/9/live.m3u8</t>
+          <t>http://69.30.245.50/live/cctv8.m3u8</t>
         </is>
       </c>
     </row>
     <row r="105" ht="16" customHeight="1">
       <c r="A105" s="70" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>CCTV-8</t>
         </is>
       </c>
       <c r="B105" s="71" t="inlineStr">
@@ -10887,14 +10887,14 @@
       </c>
       <c r="C105" s="72" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://bztv.tvbus.cc:8081/cdnlive/cctv8.m3u8</t>
         </is>
       </c>
     </row>
     <row r="106" ht="16" customHeight="1">
       <c r="A106" s="73" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>CCTV-8</t>
         </is>
       </c>
       <c r="B106" s="74" t="inlineStr">
@@ -10904,7 +10904,7 @@
       </c>
       <c r="C106" s="75" t="inlineStr">
         <is>
-          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=55def6afe55d212c4ebd9540907c9396</t>
+          <t>http://120.40.39.246:352/newlive/live/hls/9/live.m3u8</t>
         </is>
       </c>
     </row>
@@ -10921,7 +10921,7 @@
       </c>
       <c r="C107" s="72" t="inlineStr">
         <is>
-          <t>http://112.123.243.37:50085/tsfile/live/0010_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -10938,7 +10938,7 @@
       </c>
       <c r="C108" s="75" t="inlineStr">
         <is>
-          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=b7de3897140df16686c59a8a04ac549f</t>
+          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=55def6afe55d212c4ebd9540907c9396</t>
         </is>
       </c>
     </row>
@@ -10955,7 +10955,7 @@
       </c>
       <c r="C109" s="72" t="inlineStr">
         <is>
-          <t>https://v4-702cae17a28d6e4f0c0002bba021d934.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=5536bf33e2ea132eae60addc6ecb090d</t>
+          <t>http://112.123.243.37:50085/tsfile/live/0010_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -10972,7 +10972,7 @@
       </c>
       <c r="C110" s="75" t="inlineStr">
         <is>
-          <t>http://192.151.150.154/live/cctv9hd.m3u8</t>
+          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=b7de3897140df16686c59a8a04ac549f</t>
         </is>
       </c>
     </row>
@@ -10989,7 +10989,7 @@
       </c>
       <c r="C111" s="72" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv9hd.m3u8</t>
+          <t>https://v4-702cae17a28d6e4f0c0002bba021d934.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=5536bf33e2ea132eae60addc6ecb090d</t>
         </is>
       </c>
     </row>
@@ -11006,7 +11006,7 @@
       </c>
       <c r="C112" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv9hd</t>
+          <t>http://192.151.150.154/live/cctv9hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -11023,14 +11023,14 @@
       </c>
       <c r="C113" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv9hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv9hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="114" ht="16" customHeight="1">
       <c r="A114" s="73" t="inlineStr">
         <is>
-          <t>CCTV-9_1</t>
+          <t>CCTV-9</t>
         </is>
       </c>
       <c r="B114" s="74" t="inlineStr">
@@ -11040,14 +11040,14 @@
       </c>
       <c r="C114" s="75" t="inlineStr">
         <is>
-          <t>https://xykt-fix.github.io/Y77.m3u8</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv9hd</t>
         </is>
       </c>
     </row>
     <row r="115" ht="16" customHeight="1">
       <c r="A115" s="70" t="inlineStr">
         <is>
-          <t>CCTV-9_6</t>
+          <t>CCTV-9</t>
         </is>
       </c>
       <c r="B115" s="71" t="inlineStr">
@@ -11057,14 +11057,14 @@
       </c>
       <c r="C115" s="72" t="inlineStr">
         <is>
-          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=db000b5568ff643131ea7d86610b09b7</t>
+          <t>http://107.150.60.122/live/cctv9hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="116" ht="16" customHeight="1">
       <c r="A116" s="73" t="inlineStr">
         <is>
-          <t>CCTV-9纪录</t>
+          <t>CCTV-9_1</t>
         </is>
       </c>
       <c r="B116" s="74" t="inlineStr">
@@ -11074,14 +11074,14 @@
       </c>
       <c r="C116" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv9hd.m3u8</t>
+          <t>https://xykt-fix.github.io/Y77.m3u8</t>
         </is>
       </c>
     </row>
     <row r="117" ht="16" customHeight="1">
       <c r="A117" s="70" t="inlineStr">
         <is>
-          <t>CCTV-9纪录</t>
+          <t>CCTV-9_6</t>
         </is>
       </c>
       <c r="B117" s="71" t="inlineStr">
@@ -11091,14 +11091,14 @@
       </c>
       <c r="C117" s="72" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv9hd</t>
+          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=db000b5568ff643131ea7d86610b09b7</t>
         </is>
       </c>
     </row>
     <row r="118" ht="16" customHeight="1">
       <c r="A118" s="73" t="inlineStr">
         <is>
-          <t>CCTV-世界地理</t>
+          <t>CCTV-9纪录</t>
         </is>
       </c>
       <c r="B118" s="74" t="inlineStr">
@@ -11108,14 +11108,14 @@
       </c>
       <c r="C118" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/sjdl.m3u8?auth=testpub</t>
+          <t>http://74.91.26.218:82/live/cctv9hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="119" ht="16" customHeight="1">
       <c r="A119" s="70" t="inlineStr">
         <is>
-          <t>CCTV-兵器科技</t>
+          <t>CCTV-9纪录</t>
         </is>
       </c>
       <c r="B119" s="71" t="inlineStr">
@@ -11125,14 +11125,14 @@
       </c>
       <c r="C119" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/gfjs.m3u8?auth=testpub</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv9hd</t>
         </is>
       </c>
     </row>
     <row r="120" ht="16" customHeight="1">
       <c r="A120" s="73" t="inlineStr">
         <is>
-          <t>CCTV-央視檯球</t>
+          <t>CCTV-世界地理</t>
         </is>
       </c>
       <c r="B120" s="74" t="inlineStr">
@@ -11142,14 +11142,14 @@
       </c>
       <c r="C120" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/ystq.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/sjdl.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="121" ht="16" customHeight="1">
       <c r="A121" s="70" t="inlineStr">
         <is>
-          <t>CCTV-女性時尚</t>
+          <t>CCTV-兵器科技</t>
         </is>
       </c>
       <c r="B121" s="71" t="inlineStr">
@@ -11159,14 +11159,14 @@
       </c>
       <c r="C121" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/nxss.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/gfjs.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="122" ht="16" customHeight="1">
       <c r="A122" s="73" t="inlineStr">
         <is>
-          <t>CCTV-懷舊劇場</t>
+          <t>CCTV-央視檯球</t>
         </is>
       </c>
       <c r="B122" s="74" t="inlineStr">
@@ -11176,14 +11176,14 @@
       </c>
       <c r="C122" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/hjjc.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/ystq.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="123" ht="16" customHeight="1">
       <c r="A123" s="70" t="inlineStr">
         <is>
-          <t>CCTV-衛生健康</t>
+          <t>CCTV-女性時尚</t>
         </is>
       </c>
       <c r="B123" s="71" t="inlineStr">
@@ -11193,14 +11193,14 @@
       </c>
       <c r="C123" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/wsjk.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/nxss.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="124" ht="16" customHeight="1">
       <c r="A124" s="73" t="inlineStr">
         <is>
-          <t>CCTV-風雲劇場</t>
+          <t>CCTV-懷舊劇場</t>
         </is>
       </c>
       <c r="B124" s="74" t="inlineStr">
@@ -11210,14 +11210,14 @@
       </c>
       <c r="C124" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/fyjc.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/hjjc.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="125" ht="16" customHeight="1">
       <c r="A125" s="70" t="inlineStr">
         <is>
-          <t>CCTV-風雲足球</t>
+          <t>CCTV-衛生健康</t>
         </is>
       </c>
       <c r="B125" s="71" t="inlineStr">
@@ -11227,14 +11227,14 @@
       </c>
       <c r="C125" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/fyzq.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/wsjk.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="126" ht="16" customHeight="1">
       <c r="A126" s="73" t="inlineStr">
         <is>
-          <t>CCTV-高爾夫網球</t>
+          <t>CCTV-風雲劇場</t>
         </is>
       </c>
       <c r="B126" s="74" t="inlineStr">
@@ -11244,14 +11244,14 @@
       </c>
       <c r="C126" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/gefwq.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/fyjc.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="127" ht="16" customHeight="1">
       <c r="A127" s="70" t="inlineStr">
         <is>
-          <t>CCTV13</t>
+          <t>CCTV-風雲足球</t>
         </is>
       </c>
       <c r="B127" s="71" t="inlineStr">
@@ -11261,14 +11261,14 @@
       </c>
       <c r="C127" s="72" t="inlineStr">
         <is>
-          <t>http://ali-m-l.cztv.com/channels/lantian/channel21/1080p.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/fyzq.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="128" ht="16" customHeight="1">
       <c r="A128" s="73" t="inlineStr">
         <is>
-          <t>CCTV16</t>
+          <t>CCTV-高爾夫網球</t>
         </is>
       </c>
       <c r="B128" s="74" t="inlineStr">
@@ -11278,14 +11278,14 @@
       </c>
       <c r="C128" s="75" t="inlineStr">
         <is>
-          <t>http://gmxw.7766.org:808/hls/169/index.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/gefwq.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="129" ht="16" customHeight="1">
       <c r="A129" s="70" t="inlineStr">
         <is>
-          <t>CGTN纪录</t>
+          <t>CCTV13</t>
         </is>
       </c>
       <c r="B129" s="71" t="inlineStr">
@@ -11295,14 +11295,14 @@
       </c>
       <c r="C129" s="72" t="inlineStr">
         <is>
-          <t>http://english-livebkali.cgtn.com/live/doccgtn_0.m3u8</t>
+          <t>http://ali-m-l.cztv.com/channels/lantian/channel21/1080p.m3u8</t>
         </is>
       </c>
     </row>
     <row r="130" ht="16" customHeight="1">
       <c r="A130" s="73" t="inlineStr">
         <is>
-          <t>CGTN英语</t>
+          <t>CCTV16</t>
         </is>
       </c>
       <c r="B130" s="74" t="inlineStr">
@@ -11312,14 +11312,14 @@
       </c>
       <c r="C130" s="75" t="inlineStr">
         <is>
-          <t>https://english-livebkali.cgtn.com/live/encgtn_0.m3u8</t>
+          <t>http://gmxw.7766.org:808/hls/169/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="131" ht="16" customHeight="1">
       <c r="A131" s="70" t="inlineStr">
         <is>
-          <t>F1 TV</t>
+          <t>CGTN纪录</t>
         </is>
       </c>
       <c r="B131" s="71" t="inlineStr">
@@ -11329,14 +11329,14 @@
       </c>
       <c r="C131" s="72" t="inlineStr">
         <is>
-          <t>https://amg12058-c15studio-amg12058c1-lg-us-5787.playouts.now.amagi.tv/playlist.m3u8</t>
+          <t>http://english-livebkali.cgtn.com/live/doccgtn_0.m3u8</t>
         </is>
       </c>
     </row>
     <row r="132" ht="16" customHeight="1">
       <c r="A132" s="73" t="inlineStr">
         <is>
-          <t>PGA Tour_4</t>
+          <t>CGTN英语</t>
         </is>
       </c>
       <c r="B132" s="74" t="inlineStr">
@@ -11346,14 +11346,14 @@
       </c>
       <c r="C132" s="75" t="inlineStr">
         <is>
-          <t>https://d11k1mnrgfposz.cloudfront.net/playlist.m3u8</t>
+          <t>https://english-livebkali.cgtn.com/live/encgtn_0.m3u8</t>
         </is>
       </c>
     </row>
     <row r="133" ht="16" customHeight="1">
       <c r="A133" s="70" t="inlineStr">
         <is>
-          <t>世界地理</t>
+          <t>F1 TV</t>
         </is>
       </c>
       <c r="B133" s="71" t="inlineStr">
@@ -11363,14 +11363,14 @@
       </c>
       <c r="C133" s="72" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=sjdl</t>
+          <t>https://amg12058-c15studio-amg12058c1-lg-us-5787.playouts.now.amagi.tv/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="134" ht="16" customHeight="1">
       <c r="A134" s="73" t="inlineStr">
         <is>
-          <t>兵器科技</t>
+          <t>PGA Tour_4</t>
         </is>
       </c>
       <c r="B134" s="74" t="inlineStr">
@@ -11380,14 +11380,14 @@
       </c>
       <c r="C134" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=gfjs</t>
+          <t>https://d11k1mnrgfposz.cloudfront.net/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="135" ht="16" customHeight="1">
       <c r="A135" s="70" t="inlineStr">
         <is>
-          <t>央视台球</t>
+          <t>世界地理</t>
         </is>
       </c>
       <c r="B135" s="71" t="inlineStr">
@@ -11397,14 +11397,14 @@
       </c>
       <c r="C135" s="72" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=ystq</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=sjdl</t>
         </is>
       </c>
     </row>
     <row r="136" ht="16" customHeight="1">
       <c r="A136" s="73" t="inlineStr">
         <is>
-          <t>笑看风云</t>
+          <t>兵器科技</t>
         </is>
       </c>
       <c r="B136" s="74" t="inlineStr">
@@ -11414,14 +11414,14 @@
       </c>
       <c r="C136" s="75" t="inlineStr">
         <is>
-          <t>https://live.metshop.top/huya/29465858</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=gfjs</t>
         </is>
       </c>
     </row>
     <row r="137" ht="16" customHeight="1">
       <c r="A137" s="70" t="inlineStr">
         <is>
-          <t>韩国电影1</t>
+          <t>央视台球</t>
         </is>
       </c>
       <c r="B137" s="71" t="inlineStr">
@@ -11431,14 +11431,14 @@
       </c>
       <c r="C137" s="72" t="inlineStr">
         <is>
-          <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=595</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=ystq</t>
         </is>
       </c>
     </row>
     <row r="138" ht="16" customHeight="1">
       <c r="A138" s="73" t="inlineStr">
         <is>
-          <t>韩国电影2</t>
+          <t>笑看风云</t>
         </is>
       </c>
       <c r="B138" s="74" t="inlineStr">
@@ -11448,14 +11448,14 @@
       </c>
       <c r="C138" s="75" t="inlineStr">
         <is>
-          <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=743</t>
+          <t>https://live.metshop.top/huya/29465858</t>
         </is>
       </c>
     </row>
     <row r="139" ht="16" customHeight="1">
       <c r="A139" s="70" t="inlineStr">
         <is>
-          <t>风云剧场</t>
+          <t>韩国电影1</t>
         </is>
       </c>
       <c r="B139" s="71" t="inlineStr">
@@ -11465,14 +11465,14 @@
       </c>
       <c r="C139" s="72" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyjc</t>
+          <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=595</t>
         </is>
       </c>
     </row>
     <row r="140" ht="16" customHeight="1">
       <c r="A140" s="73" t="inlineStr">
         <is>
-          <t>风云足球</t>
+          <t>韩国电影2</t>
         </is>
       </c>
       <c r="B140" s="74" t="inlineStr">
@@ -11482,22 +11482,56 @@
       </c>
       <c r="C140" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyzq</t>
+          <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=743</t>
         </is>
       </c>
     </row>
     <row r="141" ht="16" customHeight="1">
       <c r="A141" s="70" t="inlineStr">
         <is>
+          <t>风云剧场</t>
+        </is>
+      </c>
+      <c r="B141" s="71" t="inlineStr">
+        <is>
+          <t>央视频道</t>
+        </is>
+      </c>
+      <c r="C141" s="72" t="inlineStr">
+        <is>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyjc</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="16" customHeight="1">
+      <c r="A142" s="73" t="inlineStr">
+        <is>
+          <t>风云足球</t>
+        </is>
+      </c>
+      <c r="B142" s="74" t="inlineStr">
+        <is>
+          <t>央视频道</t>
+        </is>
+      </c>
+      <c r="C142" s="75" t="inlineStr">
+        <is>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyzq</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="16" customHeight="1">
+      <c r="A143" s="70" t="inlineStr">
+        <is>
           <t>风云音乐</t>
         </is>
       </c>
-      <c r="B141" s="71" t="inlineStr">
+      <c r="B143" s="71" t="inlineStr">
         <is>
           <t>央视频道</t>
         </is>
       </c>
-      <c r="C141" s="72" t="inlineStr">
+      <c r="C143" s="72" t="inlineStr">
         <is>
           <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyyy</t>
         </is>

</xml_diff>

<commit_message>
fix(cctv): correct IPTV channel IDs, purge misrouted provincial streams (Hunan City TV), and fix 4K/8K heuristic
</commit_message>
<xml_diff>
--- a/channels_overview.xlsx
+++ b/channels_overview.xlsx
@@ -1319,7 +1319,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>162</v>
+        <v>141</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
@@ -1694,7 +1694,7 @@
         </is>
       </c>
       <c r="B28" s="67" t="n">
-        <v>3198</v>
+        <v>3177</v>
       </c>
       <c r="C28" s="67" t="n"/>
     </row>
@@ -8751,7 +8751,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C164"/>
+  <dimension ref="A1:C143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -8762,7 +8762,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="68" t="inlineStr">
         <is>
-          <t>📺  📡 中国大陆 · 央视  —  共 162 条频道</t>
+          <t>📺  📡 中国大陆 · 央视  —  共 141 条频道</t>
         </is>
       </c>
     </row>
@@ -8922,7 +8922,7 @@
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="70" t="inlineStr">
         <is>
-          <t>CCTV-1</t>
+          <t>CCTV-10</t>
         </is>
       </c>
       <c r="B11" s="71" t="inlineStr">
@@ -8932,14 +8932,14 @@
       </c>
       <c r="C11" s="72" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/1001_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0010_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="73" t="inlineStr">
         <is>
-          <t>CCTV-1</t>
+          <t>CCTV-10</t>
         </is>
       </c>
       <c r="B12" s="74" t="inlineStr">
@@ -8949,7 +8949,7 @@
       </c>
       <c r="C12" s="75" t="inlineStr">
         <is>
-          <t>http://116.128.243.121:85/tsfile/live/1001_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://74.91.26.218:82/live/cctv10hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -8966,7 +8966,7 @@
       </c>
       <c r="C13" s="72" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0010_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://204.12.221.218:8181/3m1080p/cctv10.m3u8</t>
         </is>
       </c>
     </row>
@@ -8983,7 +8983,7 @@
       </c>
       <c r="C14" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv10hd.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv10hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
@@ -9000,7 +9000,7 @@
       </c>
       <c r="C15" s="72" t="inlineStr">
         <is>
-          <t>http://204.12.221.218:8181/3m1080p/cctv10.m3u8</t>
+          <t>http://69.30.245.50/live/cctv10.m3u8</t>
         </is>
       </c>
     </row>
@@ -9017,7 +9017,7 @@
       </c>
       <c r="C16" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv10hd.m3u8?auth=test20251009</t>
+          <t>http://bztv.tvbus.cc:8081/cdnlive/cctv10.m3u8</t>
         </is>
       </c>
     </row>
@@ -9034,14 +9034,14 @@
       </c>
       <c r="C17" s="72" t="inlineStr">
         <is>
-          <t>http://69.30.245.50/live/cctv10.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0010_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="73" t="inlineStr">
         <is>
-          <t>CCTV-10</t>
+          <t>CCTV-10_1</t>
         </is>
       </c>
       <c r="B18" s="74" t="inlineStr">
@@ -9051,14 +9051,14 @@
       </c>
       <c r="C18" s="75" t="inlineStr">
         <is>
-          <t>http://bztv.tvbus.cc:8081/cdnlive/cctv10.m3u8</t>
+          <t>https://cdn4.skygo.mn/live/disk1/CCTV-10/HLSv3-FTA/CCTV-10.m3u8</t>
         </is>
       </c>
     </row>
     <row r="19" ht="16" customHeight="1">
       <c r="A19" s="70" t="inlineStr">
         <is>
-          <t>CCTV-10</t>
+          <t>CCTV-11</t>
         </is>
       </c>
       <c r="B19" s="71" t="inlineStr">
@@ -9068,14 +9068,14 @@
       </c>
       <c r="C19" s="72" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0010_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0011_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
       <c r="A20" s="73" t="inlineStr">
         <is>
-          <t>CCTV-10_1</t>
+          <t>CCTV-11</t>
         </is>
       </c>
       <c r="B20" s="74" t="inlineStr">
@@ -9085,7 +9085,7 @@
       </c>
       <c r="C20" s="75" t="inlineStr">
         <is>
-          <t>https://cdn4.skygo.mn/live/disk1/CCTV-10/HLSv3-FTA/CCTV-10.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv11hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -9102,7 +9102,7 @@
       </c>
       <c r="C21" s="72" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0011_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv11hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
@@ -9119,7 +9119,7 @@
       </c>
       <c r="C22" s="75" t="inlineStr">
         <is>
-          <t>http://112.123.243.37:50085/tsfile/live/0012_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://204.12.221.218:8181/3m1080p/cctv11.m3u8</t>
         </is>
       </c>
     </row>
@@ -9136,7 +9136,7 @@
       </c>
       <c r="C23" s="72" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv11hd.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/cctv11hd.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
@@ -9153,14 +9153,14 @@
       </c>
       <c r="C24" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv11hd.m3u8?auth=test20251009</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0011_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="70" t="inlineStr">
         <is>
-          <t>CCTV-11</t>
+          <t>CCTV-12</t>
         </is>
       </c>
       <c r="B25" s="71" t="inlineStr">
@@ -9170,14 +9170,14 @@
       </c>
       <c r="C25" s="72" t="inlineStr">
         <is>
-          <t>http://204.12.221.218:8181/3m1080p/cctv11.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv12hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="73" t="inlineStr">
         <is>
-          <t>CCTV-11</t>
+          <t>CCTV-12</t>
         </is>
       </c>
       <c r="B26" s="74" t="inlineStr">
@@ -9187,14 +9187,14 @@
       </c>
       <c r="C26" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/cctv11hd.m3u8?auth=testpub</t>
+          <t>http://204.12.221.218:8181/3m1080p/cctv12.m3u8</t>
         </is>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="70" t="inlineStr">
         <is>
-          <t>CCTV-11</t>
+          <t>CCTV-12</t>
         </is>
       </c>
       <c r="B27" s="71" t="inlineStr">
@@ -9204,7 +9204,7 @@
       </c>
       <c r="C27" s="72" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0011_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv12hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
@@ -9221,7 +9221,7 @@
       </c>
       <c r="C28" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv12hd.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/cctv12hd.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
@@ -9238,7 +9238,7 @@
       </c>
       <c r="C29" s="72" t="inlineStr">
         <is>
-          <t>http://112.123.243.37:50085/tsfile/live/0013_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://107.150.60.122/live/cctv12hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -9255,14 +9255,14 @@
       </c>
       <c r="C30" s="75" t="inlineStr">
         <is>
-          <t>http://204.12.221.218:8181/3m1080p/cctv12.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0012_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="70" t="inlineStr">
         <is>
-          <t>CCTV-12</t>
+          <t>CCTV-13</t>
         </is>
       </c>
       <c r="B31" s="71" t="inlineStr">
@@ -9272,14 +9272,14 @@
       </c>
       <c r="C31" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv12hd.m3u8?auth=test20251009</t>
+          <t>https://event.pull.hebtv.com/jishi/cp1.m3u8</t>
         </is>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="73" t="inlineStr">
         <is>
-          <t>CCTV-12</t>
+          <t>CCTV-13</t>
         </is>
       </c>
       <c r="B32" s="74" t="inlineStr">
@@ -9289,14 +9289,14 @@
       </c>
       <c r="C32" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/cctv12hd.m3u8?auth=testpub</t>
+          <t>http://74.91.26.218:82/live/cctv13hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="70" t="inlineStr">
         <is>
-          <t>CCTV-12</t>
+          <t>CCTV-13</t>
         </is>
       </c>
       <c r="B33" s="71" t="inlineStr">
@@ -9306,14 +9306,14 @@
       </c>
       <c r="C33" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv12hd.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv13hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="73" t="inlineStr">
         <is>
-          <t>CCTV-12</t>
+          <t>CCTV-13</t>
         </is>
       </c>
       <c r="B34" s="74" t="inlineStr">
@@ -9323,7 +9323,7 @@
       </c>
       <c r="C34" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0012_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv13hd</t>
         </is>
       </c>
     </row>
@@ -9340,7 +9340,7 @@
       </c>
       <c r="C35" s="72" t="inlineStr">
         <is>
-          <t>https://event.pull.hebtv.com/jishi/cp1.m3u8</t>
+          <t>http://bztv.tvbus.cc:8081/cdnlive/cctv13.m3u8</t>
         </is>
       </c>
     </row>
@@ -9357,14 +9357,14 @@
       </c>
       <c r="C36" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv13hd.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0013_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="70" t="inlineStr">
         <is>
-          <t>CCTV-13</t>
+          <t>CCTV-14</t>
         </is>
       </c>
       <c r="B37" s="71" t="inlineStr">
@@ -9374,14 +9374,14 @@
       </c>
       <c r="C37" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv13hd.m3u8?auth=test20251009</t>
+          <t>https://event.pull.hebtv.com/jishi/cp2.m3u8</t>
         </is>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1">
       <c r="A38" s="73" t="inlineStr">
         <is>
-          <t>CCTV-13</t>
+          <t>CCTV-14</t>
         </is>
       </c>
       <c r="B38" s="74" t="inlineStr">
@@ -9391,14 +9391,14 @@
       </c>
       <c r="C38" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv13hd</t>
+          <t>http://204.12.221.218:8181/3m1080p/cctv14.m3u8</t>
         </is>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1">
       <c r="A39" s="70" t="inlineStr">
         <is>
-          <t>CCTV-13</t>
+          <t>CCTV-14</t>
         </is>
       </c>
       <c r="B39" s="71" t="inlineStr">
@@ -9408,14 +9408,14 @@
       </c>
       <c r="C39" s="72" t="inlineStr">
         <is>
-          <t>http://bztv.tvbus.cc:8081/cdnlive/cctv13.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv14hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="73" t="inlineStr">
         <is>
-          <t>CCTV-13</t>
+          <t>CCTV-14</t>
         </is>
       </c>
       <c r="B40" s="74" t="inlineStr">
@@ -9425,7 +9425,7 @@
       </c>
       <c r="C40" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0013_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv14hd</t>
         </is>
       </c>
     </row>
@@ -9442,7 +9442,7 @@
       </c>
       <c r="C41" s="72" t="inlineStr">
         <is>
-          <t>https://event.pull.hebtv.com/jishi/cp2.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv14hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
@@ -9459,14 +9459,14 @@
       </c>
       <c r="C42" s="75" t="inlineStr">
         <is>
-          <t>http://204.12.221.218:8181/3m1080p/cctv14.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0014_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="70" t="inlineStr">
         <is>
-          <t>CCTV-14</t>
+          <t>CCTV-14少儿</t>
         </is>
       </c>
       <c r="B43" s="71" t="inlineStr">
@@ -9476,14 +9476,14 @@
       </c>
       <c r="C43" s="72" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv14hd.m3u8</t>
+          <t>http://204.12.221.218:8181/3m1080p/cctv14.m3u8</t>
         </is>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="73" t="inlineStr">
         <is>
-          <t>CCTV-14</t>
+          <t>CCTV-14少儿</t>
         </is>
       </c>
       <c r="B44" s="74" t="inlineStr">
@@ -9493,14 +9493,14 @@
       </c>
       <c r="C44" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv14hd</t>
+          <t>http://74.91.26.218:82/live/cctv14hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="70" t="inlineStr">
         <is>
-          <t>CCTV-14</t>
+          <t>CCTV-14少儿</t>
         </is>
       </c>
       <c r="B45" s="71" t="inlineStr">
@@ -9510,14 +9510,14 @@
       </c>
       <c r="C45" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv14hd.m3u8?auth=test20251009</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv14hd</t>
         </is>
       </c>
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="73" t="inlineStr">
         <is>
-          <t>CCTV-14</t>
+          <t>CCTV-14少儿</t>
         </is>
       </c>
       <c r="B46" s="74" t="inlineStr">
@@ -9527,7 +9527,7 @@
       </c>
       <c r="C46" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0014_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv14hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
@@ -9544,14 +9544,14 @@
       </c>
       <c r="C47" s="72" t="inlineStr">
         <is>
-          <t>http://204.12.221.218:8181/3m1080p/cctv14.m3u8</t>
+          <t>http://173.208.212.130:8181/1080p/cctv14.m3u8</t>
         </is>
       </c>
     </row>
     <row r="48" ht="16" customHeight="1">
       <c r="A48" s="73" t="inlineStr">
         <is>
-          <t>CCTV-14少儿</t>
+          <t>CCTV-15</t>
         </is>
       </c>
       <c r="B48" s="74" t="inlineStr">
@@ -9561,14 +9561,14 @@
       </c>
       <c r="C48" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv14hd.m3u8</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0015_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1">
       <c r="A49" s="70" t="inlineStr">
         <is>
-          <t>CCTV-14少儿</t>
+          <t>CCTV-15</t>
         </is>
       </c>
       <c r="B49" s="71" t="inlineStr">
@@ -9578,14 +9578,14 @@
       </c>
       <c r="C49" s="72" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv14hd</t>
+          <t>http://204.12.221.218:8181/3m1080p/cctv15.m3u8</t>
         </is>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="73" t="inlineStr">
         <is>
-          <t>CCTV-14少儿</t>
+          <t>CCTV-15</t>
         </is>
       </c>
       <c r="B50" s="74" t="inlineStr">
@@ -9595,14 +9595,14 @@
       </c>
       <c r="C50" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv14hd.m3u8?auth=test20251009</t>
+          <t>http://74.91.26.218:82/live/cctv15hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="51" ht="16" customHeight="1">
       <c r="A51" s="70" t="inlineStr">
         <is>
-          <t>CCTV-14少儿</t>
+          <t>CCTV-15</t>
         </is>
       </c>
       <c r="B51" s="71" t="inlineStr">
@@ -9612,7 +9612,7 @@
       </c>
       <c r="C51" s="72" t="inlineStr">
         <is>
-          <t>http://173.208.212.130:8181/1080p/cctv14.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv15hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
@@ -9629,7 +9629,7 @@
       </c>
       <c r="C52" s="75" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0015_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv15hd</t>
         </is>
       </c>
     </row>
@@ -9646,14 +9646,14 @@
       </c>
       <c r="C53" s="72" t="inlineStr">
         <is>
-          <t>http://204.12.221.218:8181/3m1080p/cctv15.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0015_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="54" ht="16" customHeight="1">
       <c r="A54" s="73" t="inlineStr">
         <is>
-          <t>CCTV-15</t>
+          <t>CCTV-16</t>
         </is>
       </c>
       <c r="B54" s="74" t="inlineStr">
@@ -9663,14 +9663,14 @@
       </c>
       <c r="C54" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv15hd.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/cctv16hd.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="55" ht="16" customHeight="1">
       <c r="A55" s="70" t="inlineStr">
         <is>
-          <t>CCTV-15</t>
+          <t>CCTV-16</t>
         </is>
       </c>
       <c r="B55" s="71" t="inlineStr">
@@ -9680,14 +9680,14 @@
       </c>
       <c r="C55" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv15hd.m3u8?auth=test20251009</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0016_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="56" ht="16" customHeight="1">
       <c r="A56" s="73" t="inlineStr">
         <is>
-          <t>CCTV-15</t>
+          <t>CCTV-16奥林匹克</t>
         </is>
       </c>
       <c r="B56" s="74" t="inlineStr">
@@ -9697,14 +9697,14 @@
       </c>
       <c r="C56" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv15hd</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv16hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
     <row r="57" ht="16" customHeight="1">
       <c r="A57" s="70" t="inlineStr">
         <is>
-          <t>CCTV-15</t>
+          <t>CCTV-17</t>
         </is>
       </c>
       <c r="B57" s="71" t="inlineStr">
@@ -9714,14 +9714,14 @@
       </c>
       <c r="C57" s="72" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0015_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv17hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
     <row r="58" ht="16" customHeight="1">
       <c r="A58" s="73" t="inlineStr">
         <is>
-          <t>CCTV-16</t>
+          <t>CCTV-17</t>
         </is>
       </c>
       <c r="B58" s="74" t="inlineStr">
@@ -9731,14 +9731,14 @@
       </c>
       <c r="C58" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/cctv16hd.m3u8?auth=testpub</t>
+          <t>http://74.91.26.218:82/live/cctv17hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="59" ht="16" customHeight="1">
       <c r="A59" s="70" t="inlineStr">
         <is>
-          <t>CCTV-16</t>
+          <t>CCTV-17</t>
         </is>
       </c>
       <c r="B59" s="71" t="inlineStr">
@@ -9748,14 +9748,14 @@
       </c>
       <c r="C59" s="72" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0016_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv17hd</t>
         </is>
       </c>
     </row>
     <row r="60" ht="16" customHeight="1">
       <c r="A60" s="73" t="inlineStr">
         <is>
-          <t>CCTV-16奥林匹克</t>
+          <t>CCTV-17</t>
         </is>
       </c>
       <c r="B60" s="74" t="inlineStr">
@@ -9765,14 +9765,14 @@
       </c>
       <c r="C60" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv16hd.m3u8?auth=test20251009</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0017_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="61" ht="16" customHeight="1">
       <c r="A61" s="70" t="inlineStr">
         <is>
-          <t>CCTV-17</t>
+          <t>CCTV-2</t>
         </is>
       </c>
       <c r="B61" s="71" t="inlineStr">
@@ -9782,14 +9782,14 @@
       </c>
       <c r="C61" s="72" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0007_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0002_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="62" ht="16" customHeight="1">
       <c r="A62" s="73" t="inlineStr">
         <is>
-          <t>CCTV-17</t>
+          <t>CCTV-2</t>
         </is>
       </c>
       <c r="B62" s="74" t="inlineStr">
@@ -9799,14 +9799,14 @@
       </c>
       <c r="C62" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv17hd.m3u8?auth=test20251009</t>
+          <t>http://74.91.26.218:82/live/cctv2hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="63" ht="16" customHeight="1">
       <c r="A63" s="70" t="inlineStr">
         <is>
-          <t>CCTV-17</t>
+          <t>CCTV-2</t>
         </is>
       </c>
       <c r="B63" s="71" t="inlineStr">
@@ -9816,14 +9816,14 @@
       </c>
       <c r="C63" s="72" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv17hd.m3u8</t>
+          <t>http://204.12.221.218:8181/3m1080p/cctv2.m3u8</t>
         </is>
       </c>
     </row>
     <row r="64" ht="16" customHeight="1">
       <c r="A64" s="73" t="inlineStr">
         <is>
-          <t>CCTV-17</t>
+          <t>CCTV-2</t>
         </is>
       </c>
       <c r="B64" s="74" t="inlineStr">
@@ -9833,14 +9833,14 @@
       </c>
       <c r="C64" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv17hd</t>
+          <t>http://bztv.tvbus.cc:8081/cdnlive/cctv2.m3u8</t>
         </is>
       </c>
     </row>
     <row r="65" ht="16" customHeight="1">
       <c r="A65" s="70" t="inlineStr">
         <is>
-          <t>CCTV-17</t>
+          <t>CCTV-2</t>
         </is>
       </c>
       <c r="B65" s="71" t="inlineStr">
@@ -9850,7 +9850,7 @@
       </c>
       <c r="C65" s="72" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0017_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://107.150.60.122/live/cctv2hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -9867,7 +9867,7 @@
       </c>
       <c r="C66" s="75" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0002_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://192.151.150.154/live/cctv2hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -9884,7 +9884,7 @@
       </c>
       <c r="C67" s="72" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv2hd.m3u8</t>
+          <t>http://116.128.243.121:85/tsfile/live/0002_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -9901,7 +9901,7 @@
       </c>
       <c r="C68" s="75" t="inlineStr">
         <is>
-          <t>http://204.12.221.218:8181/3m1080p/cctv2.m3u8</t>
+          <t>http://173.208.212.130:8181/720p/cctv2.m3u8</t>
         </is>
       </c>
     </row>
@@ -9918,14 +9918,14 @@
       </c>
       <c r="C69" s="72" t="inlineStr">
         <is>
-          <t>http://bztv.tvbus.cc:8081/cdnlive/cctv2.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0002_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="70" ht="16" customHeight="1">
       <c r="A70" s="73" t="inlineStr">
         <is>
-          <t>CCTV-2</t>
+          <t>CCTV-3</t>
         </is>
       </c>
       <c r="B70" s="74" t="inlineStr">
@@ -9935,14 +9935,14 @@
       </c>
       <c r="C70" s="75" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv2hd.m3u8</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0003_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="71" ht="16" customHeight="1">
       <c r="A71" s="70" t="inlineStr">
         <is>
-          <t>CCTV-2</t>
+          <t>CCTV-3</t>
         </is>
       </c>
       <c r="B71" s="71" t="inlineStr">
@@ -9952,14 +9952,14 @@
       </c>
       <c r="C71" s="72" t="inlineStr">
         <is>
-          <t>http://192.151.150.154/live/cctv2hd.m3u8</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv3hd</t>
         </is>
       </c>
     </row>
     <row r="72" ht="16" customHeight="1">
       <c r="A72" s="73" t="inlineStr">
         <is>
-          <t>CCTV-2</t>
+          <t>CCTV-3</t>
         </is>
       </c>
       <c r="B72" s="74" t="inlineStr">
@@ -9969,14 +9969,14 @@
       </c>
       <c r="C72" s="75" t="inlineStr">
         <is>
-          <t>http://116.128.243.121:85/tsfile/live/0002_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://69.30.245.50/live/cctv3.m3u8</t>
         </is>
       </c>
     </row>
     <row r="73" ht="16" customHeight="1">
       <c r="A73" s="70" t="inlineStr">
         <is>
-          <t>CCTV-2</t>
+          <t>CCTV-3</t>
         </is>
       </c>
       <c r="B73" s="71" t="inlineStr">
@@ -9986,14 +9986,14 @@
       </c>
       <c r="C73" s="72" t="inlineStr">
         <is>
-          <t>http://173.208.212.130:8181/720p/cctv2.m3u8</t>
+          <t>http://107.150.60.122/live/cctv3hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="74" ht="16" customHeight="1">
       <c r="A74" s="73" t="inlineStr">
         <is>
-          <t>CCTV-2</t>
+          <t>CCTV-3</t>
         </is>
       </c>
       <c r="B74" s="74" t="inlineStr">
@@ -10003,14 +10003,14 @@
       </c>
       <c r="C74" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0002_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0003_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="75" ht="16" customHeight="1">
       <c r="A75" s="70" t="inlineStr">
         <is>
-          <t>CCTV-2</t>
+          <t>CCTV-3 綜藝</t>
         </is>
       </c>
       <c r="B75" s="71" t="inlineStr">
@@ -10020,14 +10020,14 @@
       </c>
       <c r="C75" s="72" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/1002_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://74.91.26.218:82/live/cctv3hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="76" ht="16" customHeight="1">
       <c r="A76" s="73" t="inlineStr">
         <is>
-          <t>CCTV-2</t>
+          <t>CCTV-4</t>
         </is>
       </c>
       <c r="B76" s="74" t="inlineStr">
@@ -10037,14 +10037,14 @@
       </c>
       <c r="C76" s="75" t="inlineStr">
         <is>
-          <t>http://116.128.243.121:85/tsfile/live/1002_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0004_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="77" ht="16" customHeight="1">
       <c r="A77" s="70" t="inlineStr">
         <is>
-          <t>CCTV-3</t>
+          <t>CCTV-4</t>
         </is>
       </c>
       <c r="B77" s="71" t="inlineStr">
@@ -10054,14 +10054,14 @@
       </c>
       <c r="C77" s="72" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0003_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://74.91.26.218:82/live/cctv4hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="78" ht="16" customHeight="1">
       <c r="A78" s="73" t="inlineStr">
         <is>
-          <t>CCTV-3</t>
+          <t>CCTV-4</t>
         </is>
       </c>
       <c r="B78" s="74" t="inlineStr">
@@ -10071,14 +10071,14 @@
       </c>
       <c r="C78" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv3hd</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv4hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
     <row r="79" ht="16" customHeight="1">
       <c r="A79" s="70" t="inlineStr">
         <is>
-          <t>CCTV-3</t>
+          <t>CCTV-4</t>
         </is>
       </c>
       <c r="B79" s="71" t="inlineStr">
@@ -10088,14 +10088,14 @@
       </c>
       <c r="C79" s="72" t="inlineStr">
         <is>
-          <t>http://69.30.245.50/live/cctv3.m3u8</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv4hd</t>
         </is>
       </c>
     </row>
     <row r="80" ht="16" customHeight="1">
       <c r="A80" s="73" t="inlineStr">
         <is>
-          <t>CCTV-3</t>
+          <t>CCTV-4</t>
         </is>
       </c>
       <c r="B80" s="74" t="inlineStr">
@@ -10105,14 +10105,14 @@
       </c>
       <c r="C80" s="75" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv3hd.m3u8</t>
+          <t>http://107.150.60.122/live/cctv4hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="81" ht="16" customHeight="1">
       <c r="A81" s="70" t="inlineStr">
         <is>
-          <t>CCTV-3</t>
+          <t>CCTV-4</t>
         </is>
       </c>
       <c r="B81" s="71" t="inlineStr">
@@ -10122,14 +10122,14 @@
       </c>
       <c r="C81" s="72" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0003_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://58.56.162.102:4466/newlive/live/hls/4/live.m3u8</t>
         </is>
       </c>
     </row>
     <row r="82" ht="16" customHeight="1">
       <c r="A82" s="73" t="inlineStr">
         <is>
-          <t>CCTV-3</t>
+          <t>CCTV-4</t>
         </is>
       </c>
       <c r="B82" s="74" t="inlineStr">
@@ -10139,14 +10139,14 @@
       </c>
       <c r="C82" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/1003_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://173.208.212.130:8181/1080p/cctv4.m3u8</t>
         </is>
       </c>
     </row>
     <row r="83" ht="16" customHeight="1">
       <c r="A83" s="70" t="inlineStr">
         <is>
-          <t>CCTV-3</t>
+          <t>CCTV-4</t>
         </is>
       </c>
       <c r="B83" s="71" t="inlineStr">
@@ -10156,14 +10156,14 @@
       </c>
       <c r="C83" s="72" t="inlineStr">
         <is>
-          <t>http://116.128.243.121:85/tsfile/live/1003_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/cctv4k.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="84" ht="16" customHeight="1">
       <c r="A84" s="73" t="inlineStr">
         <is>
-          <t>CCTV-3 綜藝</t>
+          <t>CCTV-5</t>
         </is>
       </c>
       <c r="B84" s="74" t="inlineStr">
@@ -10173,14 +10173,14 @@
       </c>
       <c r="C84" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv3hd.m3u8</t>
+          <t>http://118.122.144.115:8888/newlive/live/hls/5/live.m3u8</t>
         </is>
       </c>
     </row>
     <row r="85" ht="16" customHeight="1">
       <c r="A85" s="70" t="inlineStr">
         <is>
-          <t>CCTV-4</t>
+          <t>CCTV-5</t>
         </is>
       </c>
       <c r="B85" s="71" t="inlineStr">
@@ -10190,14 +10190,14 @@
       </c>
       <c r="C85" s="72" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0004_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0005_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="86" ht="16" customHeight="1">
       <c r="A86" s="73" t="inlineStr">
         <is>
-          <t>CCTV-4</t>
+          <t>CCTV-5</t>
         </is>
       </c>
       <c r="B86" s="74" t="inlineStr">
@@ -10207,14 +10207,14 @@
       </c>
       <c r="C86" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv4hd.m3u8</t>
+          <t>http://107.150.60.122/live/cctv5hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="87" ht="16" customHeight="1">
       <c r="A87" s="70" t="inlineStr">
         <is>
-          <t>CCTV-4</t>
+          <t>CCTV-5</t>
         </is>
       </c>
       <c r="B87" s="71" t="inlineStr">
@@ -10224,14 +10224,14 @@
       </c>
       <c r="C87" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv4hd.m3u8?auth=test20251009</t>
+          <t>http://173.208.212.130:8181/720p/cctv5.m3u8</t>
         </is>
       </c>
     </row>
     <row r="88" ht="16" customHeight="1">
       <c r="A88" s="73" t="inlineStr">
         <is>
-          <t>CCTV-4</t>
+          <t>CCTV-5</t>
         </is>
       </c>
       <c r="B88" s="74" t="inlineStr">
@@ -10241,14 +10241,14 @@
       </c>
       <c r="C88" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv4hd</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/cctv5p.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="89" ht="16" customHeight="1">
       <c r="A89" s="70" t="inlineStr">
         <is>
-          <t>CCTV-4</t>
+          <t>CCTV-5</t>
         </is>
       </c>
       <c r="B89" s="71" t="inlineStr">
@@ -10258,14 +10258,14 @@
       </c>
       <c r="C89" s="72" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv4hd.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0005_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="90" ht="16" customHeight="1">
       <c r="A90" s="73" t="inlineStr">
         <is>
-          <t>CCTV-4</t>
+          <t>CCTV-5+</t>
         </is>
       </c>
       <c r="B90" s="74" t="inlineStr">
@@ -10275,14 +10275,14 @@
       </c>
       <c r="C90" s="75" t="inlineStr">
         <is>
-          <t>http://58.56.162.102:4466/newlive/live/hls/4/live.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0016_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="91" ht="16" customHeight="1">
       <c r="A91" s="70" t="inlineStr">
         <is>
-          <t>CCTV-4</t>
+          <t>CCTV-5+体育赛事</t>
         </is>
       </c>
       <c r="B91" s="71" t="inlineStr">
@@ -10292,14 +10292,14 @@
       </c>
       <c r="C91" s="72" t="inlineStr">
         <is>
-          <t>http://173.208.212.130:8181/1080p/cctv4.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv5p.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
     <row r="92" ht="16" customHeight="1">
       <c r="A92" s="73" t="inlineStr">
         <is>
-          <t>CCTV-4</t>
+          <t>CCTV-5体育</t>
         </is>
       </c>
       <c r="B92" s="74" t="inlineStr">
@@ -10309,14 +10309,14 @@
       </c>
       <c r="C92" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/cctv4k.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv5hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
     <row r="93" ht="16" customHeight="1">
       <c r="A93" s="70" t="inlineStr">
         <is>
-          <t>CCTV-4</t>
+          <t>CCTV-6</t>
         </is>
       </c>
       <c r="B93" s="71" t="inlineStr">
@@ -10326,14 +10326,14 @@
       </c>
       <c r="C93" s="72" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/1004_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0006_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="94" ht="16" customHeight="1">
       <c r="A94" s="73" t="inlineStr">
         <is>
-          <t>CCTV-5</t>
+          <t>CCTV-6</t>
         </is>
       </c>
       <c r="B94" s="74" t="inlineStr">
@@ -10343,14 +10343,14 @@
       </c>
       <c r="C94" s="75" t="inlineStr">
         <is>
-          <t>http://118.122.144.115:8888/newlive/live/hls/5/live.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv6hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="95" ht="16" customHeight="1">
       <c r="A95" s="70" t="inlineStr">
         <is>
-          <t>CCTV-5</t>
+          <t>CCTV-6</t>
         </is>
       </c>
       <c r="B95" s="71" t="inlineStr">
@@ -10360,14 +10360,14 @@
       </c>
       <c r="C95" s="72" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0005_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://69.30.245.50/live/cctv6.m3u8</t>
         </is>
       </c>
     </row>
     <row r="96" ht="16" customHeight="1">
       <c r="A96" s="73" t="inlineStr">
         <is>
-          <t>CCTV-5</t>
+          <t>CCTV-6</t>
         </is>
       </c>
       <c r="B96" s="74" t="inlineStr">
@@ -10377,14 +10377,14 @@
       </c>
       <c r="C96" s="75" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv5hd.m3u8</t>
+          <t>http://198.204.240.250:82/live/cctv6.m3u8</t>
         </is>
       </c>
     </row>
     <row r="97" ht="16" customHeight="1">
       <c r="A97" s="70" t="inlineStr">
         <is>
-          <t>CCTV-5</t>
+          <t>CCTV-6</t>
         </is>
       </c>
       <c r="B97" s="71" t="inlineStr">
@@ -10394,14 +10394,14 @@
       </c>
       <c r="C97" s="72" t="inlineStr">
         <is>
-          <t>http://173.208.212.130:8181/720p/cctv5.m3u8</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv6hd</t>
         </is>
       </c>
     </row>
     <row r="98" ht="16" customHeight="1">
       <c r="A98" s="73" t="inlineStr">
         <is>
-          <t>CCTV-5</t>
+          <t>CCTV-6</t>
         </is>
       </c>
       <c r="B98" s="74" t="inlineStr">
@@ -10411,14 +10411,14 @@
       </c>
       <c r="C98" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/cctv5p.m3u8?auth=testpub</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0006_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="99" ht="16" customHeight="1">
       <c r="A99" s="70" t="inlineStr">
         <is>
-          <t>CCTV-5</t>
+          <t>CCTV-7</t>
         </is>
       </c>
       <c r="B99" s="71" t="inlineStr">
@@ -10428,14 +10428,14 @@
       </c>
       <c r="C99" s="72" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0005_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0007_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="100" ht="16" customHeight="1">
       <c r="A100" s="73" t="inlineStr">
         <is>
-          <t>CCTV-5</t>
+          <t>CCTV-7</t>
         </is>
       </c>
       <c r="B100" s="74" t="inlineStr">
@@ -10445,14 +10445,14 @@
       </c>
       <c r="C100" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/1005_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://74.91.26.218:82/live/cctv7hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="101" ht="16" customHeight="1">
       <c r="A101" s="70" t="inlineStr">
         <is>
-          <t>CCTV-5</t>
+          <t>CCTV-7</t>
         </is>
       </c>
       <c r="B101" s="71" t="inlineStr">
@@ -10462,14 +10462,14 @@
       </c>
       <c r="C101" s="72" t="inlineStr">
         <is>
-          <t>http://116.128.243.121:85/tsfile/live/1005_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://69.30.245.50/live/cctv7.m3u8</t>
         </is>
       </c>
     </row>
     <row r="102" ht="16" customHeight="1">
       <c r="A102" s="73" t="inlineStr">
         <is>
-          <t>CCTV-5+</t>
+          <t>CCTV-7</t>
         </is>
       </c>
       <c r="B102" s="74" t="inlineStr">
@@ -10479,14 +10479,14 @@
       </c>
       <c r="C102" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0016_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv7hd</t>
         </is>
       </c>
     </row>
     <row r="103" ht="16" customHeight="1">
       <c r="A103" s="70" t="inlineStr">
         <is>
-          <t>CCTV-5+体育赛事</t>
+          <t>CCTV-7</t>
         </is>
       </c>
       <c r="B103" s="71" t="inlineStr">
@@ -10496,14 +10496,14 @@
       </c>
       <c r="C103" s="72" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv5p.m3u8?auth=test20251009</t>
+          <t>http://107.150.60.122/live/cctv7hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="104" ht="16" customHeight="1">
       <c r="A104" s="73" t="inlineStr">
         <is>
-          <t>CCTV-5体育</t>
+          <t>CCTV-7</t>
         </is>
       </c>
       <c r="B104" s="74" t="inlineStr">
@@ -10513,14 +10513,14 @@
       </c>
       <c r="C104" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv5hd.m3u8?auth=test20251009</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0007_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="105" ht="16" customHeight="1">
       <c r="A105" s="70" t="inlineStr">
         <is>
-          <t>CCTV-6</t>
+          <t>CCTV-8</t>
         </is>
       </c>
       <c r="B105" s="71" t="inlineStr">
@@ -10530,14 +10530,14 @@
       </c>
       <c r="C105" s="72" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0006_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="106" ht="16" customHeight="1">
       <c r="A106" s="73" t="inlineStr">
         <is>
-          <t>CCTV-6</t>
+          <t>CCTV-8</t>
         </is>
       </c>
       <c r="B106" s="74" t="inlineStr">
@@ -10547,14 +10547,14 @@
       </c>
       <c r="C106" s="75" t="inlineStr">
         <is>
-          <t>http://112.123.243.37:50085/tsfile/live/0007_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://74.91.26.218:82/live/cctv8hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="107" ht="16" customHeight="1">
       <c r="A107" s="70" t="inlineStr">
         <is>
-          <t>CCTV-6</t>
+          <t>CCTV-8</t>
         </is>
       </c>
       <c r="B107" s="71" t="inlineStr">
@@ -10564,14 +10564,14 @@
       </c>
       <c r="C107" s="72" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv6hd.m3u8</t>
+          <t>http://69.30.245.50/live/cctv8.m3u8</t>
         </is>
       </c>
     </row>
     <row r="108" ht="16" customHeight="1">
       <c r="A108" s="73" t="inlineStr">
         <is>
-          <t>CCTV-6</t>
+          <t>CCTV-8</t>
         </is>
       </c>
       <c r="B108" s="74" t="inlineStr">
@@ -10581,14 +10581,14 @@
       </c>
       <c r="C108" s="75" t="inlineStr">
         <is>
-          <t>http://69.30.245.50/live/cctv6.m3u8</t>
+          <t>http://bztv.tvbus.cc:8081/cdnlive/cctv8.m3u8</t>
         </is>
       </c>
     </row>
     <row r="109" ht="16" customHeight="1">
       <c r="A109" s="70" t="inlineStr">
         <is>
-          <t>CCTV-6</t>
+          <t>CCTV-8</t>
         </is>
       </c>
       <c r="B109" s="71" t="inlineStr">
@@ -10598,14 +10598,14 @@
       </c>
       <c r="C109" s="72" t="inlineStr">
         <is>
-          <t>http://198.204.240.250:82/live/cctv6.m3u8</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv8k</t>
         </is>
       </c>
     </row>
     <row r="110" ht="16" customHeight="1">
       <c r="A110" s="73" t="inlineStr">
         <is>
-          <t>CCTV-6</t>
+          <t>CCTV-8</t>
         </is>
       </c>
       <c r="B110" s="74" t="inlineStr">
@@ -10615,14 +10615,14 @@
       </c>
       <c r="C110" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv6hd</t>
+          <t>http://120.40.39.246:352/newlive/live/hls/9/live.m3u8</t>
         </is>
       </c>
     </row>
     <row r="111" ht="16" customHeight="1">
       <c r="A111" s="70" t="inlineStr">
         <is>
-          <t>CCTV-6</t>
+          <t>CCTV-8</t>
         </is>
       </c>
       <c r="B111" s="71" t="inlineStr">
@@ -10632,14 +10632,14 @@
       </c>
       <c r="C111" s="72" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0006_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="112" ht="16" customHeight="1">
       <c r="A112" s="73" t="inlineStr">
         <is>
-          <t>CCTV-6</t>
+          <t>CCTV-8K 超高清</t>
         </is>
       </c>
       <c r="B112" s="74" t="inlineStr">
@@ -10649,14 +10649,14 @@
       </c>
       <c r="C112" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/1006_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://192.151.150.154/live/cctv8k.m3u8</t>
         </is>
       </c>
     </row>
     <row r="113" ht="16" customHeight="1">
       <c r="A113" s="70" t="inlineStr">
         <is>
-          <t>CCTV-6</t>
+          <t>CCTV-9</t>
         </is>
       </c>
       <c r="B113" s="71" t="inlineStr">
@@ -10666,14 +10666,14 @@
       </c>
       <c r="C113" s="72" t="inlineStr">
         <is>
-          <t>http://116.128.243.121:85/tsfile/live/1006_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="114" ht="16" customHeight="1">
       <c r="A114" s="73" t="inlineStr">
         <is>
-          <t>CCTV-7</t>
+          <t>CCTV-9</t>
         </is>
       </c>
       <c r="B114" s="74" t="inlineStr">
@@ -10683,14 +10683,14 @@
       </c>
       <c r="C114" s="75" t="inlineStr">
         <is>
-          <t>http://112.123.243.37:50085/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=55def6afe55d212c4ebd9540907c9396</t>
         </is>
       </c>
     </row>
     <row r="115" ht="16" customHeight="1">
       <c r="A115" s="70" t="inlineStr">
         <is>
-          <t>CCTV-7</t>
+          <t>CCTV-9</t>
         </is>
       </c>
       <c r="B115" s="71" t="inlineStr">
@@ -10700,14 +10700,14 @@
       </c>
       <c r="C115" s="72" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv7hd.m3u8</t>
+          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=b7de3897140df16686c59a8a04ac549f</t>
         </is>
       </c>
     </row>
     <row r="116" ht="16" customHeight="1">
       <c r="A116" s="73" t="inlineStr">
         <is>
-          <t>CCTV-7</t>
+          <t>CCTV-9</t>
         </is>
       </c>
       <c r="B116" s="74" t="inlineStr">
@@ -10717,14 +10717,14 @@
       </c>
       <c r="C116" s="75" t="inlineStr">
         <is>
-          <t>http://69.30.245.50/live/cctv7.m3u8</t>
+          <t>https://v4-702cae17a28d6e4f0c0002bba021d934.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=5536bf33e2ea132eae60addc6ecb090d</t>
         </is>
       </c>
     </row>
     <row r="117" ht="16" customHeight="1">
       <c r="A117" s="70" t="inlineStr">
         <is>
-          <t>CCTV-7</t>
+          <t>CCTV-9</t>
         </is>
       </c>
       <c r="B117" s="71" t="inlineStr">
@@ -10734,14 +10734,14 @@
       </c>
       <c r="C117" s="72" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv7hd</t>
+          <t>http://192.151.150.154/live/cctv9hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="118" ht="16" customHeight="1">
       <c r="A118" s="73" t="inlineStr">
         <is>
-          <t>CCTV-7</t>
+          <t>CCTV-9</t>
         </is>
       </c>
       <c r="B118" s="74" t="inlineStr">
@@ -10751,14 +10751,14 @@
       </c>
       <c r="C118" s="75" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv7hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv9hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="119" ht="16" customHeight="1">
       <c r="A119" s="70" t="inlineStr">
         <is>
-          <t>CCTV-7</t>
+          <t>CCTV-9</t>
         </is>
       </c>
       <c r="B119" s="71" t="inlineStr">
@@ -10768,14 +10768,14 @@
       </c>
       <c r="C119" s="72" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0007_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv9hd</t>
         </is>
       </c>
     </row>
     <row r="120" ht="16" customHeight="1">
       <c r="A120" s="73" t="inlineStr">
         <is>
-          <t>CCTV-7</t>
+          <t>CCTV-9</t>
         </is>
       </c>
       <c r="B120" s="74" t="inlineStr">
@@ -10785,14 +10785,14 @@
       </c>
       <c r="C120" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/1007_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://107.150.60.122/live/cctv9hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="121" ht="16" customHeight="1">
       <c r="A121" s="70" t="inlineStr">
         <is>
-          <t>CCTV-7</t>
+          <t>CCTV-9</t>
         </is>
       </c>
       <c r="B121" s="71" t="inlineStr">
@@ -10802,14 +10802,14 @@
       </c>
       <c r="C121" s="72" t="inlineStr">
         <is>
-          <t>http://116.128.243.121:85/tsfile/live/1007_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="122" ht="16" customHeight="1">
       <c r="A122" s="73" t="inlineStr">
         <is>
-          <t>CCTV-8</t>
+          <t>CCTV-9_1</t>
         </is>
       </c>
       <c r="B122" s="74" t="inlineStr">
@@ -10819,14 +10819,14 @@
       </c>
       <c r="C122" s="75" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>https://xykt-fix.github.io/Y77.m3u8</t>
         </is>
       </c>
     </row>
     <row r="123" ht="16" customHeight="1">
       <c r="A123" s="70" t="inlineStr">
         <is>
-          <t>CCTV-8</t>
+          <t>CCTV-9_6</t>
         </is>
       </c>
       <c r="B123" s="71" t="inlineStr">
@@ -10836,14 +10836,14 @@
       </c>
       <c r="C123" s="72" t="inlineStr">
         <is>
-          <t>http://112.123.243.37:50085/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=db000b5568ff643131ea7d86610b09b7</t>
         </is>
       </c>
     </row>
     <row r="124" ht="16" customHeight="1">
       <c r="A124" s="73" t="inlineStr">
         <is>
-          <t>CCTV-8</t>
+          <t>CCTV-9纪录</t>
         </is>
       </c>
       <c r="B124" s="74" t="inlineStr">
@@ -10853,14 +10853,14 @@
       </c>
       <c r="C124" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv8hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv9hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="125" ht="16" customHeight="1">
       <c r="A125" s="70" t="inlineStr">
         <is>
-          <t>CCTV-8</t>
+          <t>CCTV-9纪录</t>
         </is>
       </c>
       <c r="B125" s="71" t="inlineStr">
@@ -10870,14 +10870,14 @@
       </c>
       <c r="C125" s="72" t="inlineStr">
         <is>
-          <t>http://69.30.245.50/live/cctv8.m3u8</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv9hd</t>
         </is>
       </c>
     </row>
     <row r="126" ht="16" customHeight="1">
       <c r="A126" s="73" t="inlineStr">
         <is>
-          <t>CCTV-8</t>
+          <t>CCTV-女性時尚</t>
         </is>
       </c>
       <c r="B126" s="74" t="inlineStr">
@@ -10887,14 +10887,14 @@
       </c>
       <c r="C126" s="75" t="inlineStr">
         <is>
-          <t>http://bztv.tvbus.cc:8081/cdnlive/cctv8.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/nxss.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="127" ht="16" customHeight="1">
       <c r="A127" s="70" t="inlineStr">
         <is>
-          <t>CCTV-8</t>
+          <t>CCTV-懷舊劇場</t>
         </is>
       </c>
       <c r="B127" s="71" t="inlineStr">
@@ -10904,14 +10904,14 @@
       </c>
       <c r="C127" s="72" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv8k</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/hjjc.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="128" ht="16" customHeight="1">
       <c r="A128" s="73" t="inlineStr">
         <is>
-          <t>CCTV-8</t>
+          <t>CCTV-衛生健康</t>
         </is>
       </c>
       <c r="B128" s="74" t="inlineStr">
@@ -10921,14 +10921,14 @@
       </c>
       <c r="C128" s="75" t="inlineStr">
         <is>
-          <t>http://120.40.39.246:352/newlive/live/hls/9/live.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/wsjk.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="129" ht="16" customHeight="1">
       <c r="A129" s="70" t="inlineStr">
         <is>
-          <t>CCTV-8</t>
+          <t>CCTV13</t>
         </is>
       </c>
       <c r="B129" s="71" t="inlineStr">
@@ -10938,14 +10938,14 @@
       </c>
       <c r="C129" s="72" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://ali-m-l.cztv.com/channels/lantian/channel21/1080p.m3u8</t>
         </is>
       </c>
     </row>
     <row r="130" ht="16" customHeight="1">
       <c r="A130" s="73" t="inlineStr">
         <is>
-          <t>CCTV-8</t>
+          <t>CGTN纪录</t>
         </is>
       </c>
       <c r="B130" s="74" t="inlineStr">
@@ -10955,14 +10955,14 @@
       </c>
       <c r="C130" s="75" t="inlineStr">
         <is>
-          <t>http://116.128.243.121:85/tsfile/live/1008_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://english-livebkali.cgtn.com/live/doccgtn_0.m3u8</t>
         </is>
       </c>
     </row>
     <row r="131" ht="16" customHeight="1">
       <c r="A131" s="70" t="inlineStr">
         <is>
-          <t>CCTV-8K 超高清</t>
+          <t>CGTN英语</t>
         </is>
       </c>
       <c r="B131" s="71" t="inlineStr">
@@ -10972,14 +10972,14 @@
       </c>
       <c r="C131" s="72" t="inlineStr">
         <is>
-          <t>http://192.151.150.154/live/cctv8k.m3u8</t>
+          <t>https://english-livebkali.cgtn.com/live/encgtn_0.m3u8</t>
         </is>
       </c>
     </row>
     <row r="132" ht="16" customHeight="1">
       <c r="A132" s="73" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>F1 TV</t>
         </is>
       </c>
       <c r="B132" s="74" t="inlineStr">
@@ -10989,14 +10989,14 @@
       </c>
       <c r="C132" s="75" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>https://amg12058-c15studio-amg12058c1-lg-us-5787.playouts.now.amagi.tv/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="133" ht="16" customHeight="1">
       <c r="A133" s="70" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>PGA Tour_4</t>
         </is>
       </c>
       <c r="B133" s="71" t="inlineStr">
@@ -11006,14 +11006,14 @@
       </c>
       <c r="C133" s="72" t="inlineStr">
         <is>
-          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=55def6afe55d212c4ebd9540907c9396</t>
+          <t>https://d11k1mnrgfposz.cloudfront.net/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="134" ht="16" customHeight="1">
       <c r="A134" s="73" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>世界地理</t>
         </is>
       </c>
       <c r="B134" s="74" t="inlineStr">
@@ -11023,14 +11023,14 @@
       </c>
       <c r="C134" s="75" t="inlineStr">
         <is>
-          <t>http://112.123.243.37:50085/tsfile/live/0010_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=sjdl</t>
         </is>
       </c>
     </row>
     <row r="135" ht="16" customHeight="1">
       <c r="A135" s="70" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>兵器科技</t>
         </is>
       </c>
       <c r="B135" s="71" t="inlineStr">
@@ -11040,14 +11040,14 @@
       </c>
       <c r="C135" s="72" t="inlineStr">
         <is>
-          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=b7de3897140df16686c59a8a04ac549f</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=gfjs</t>
         </is>
       </c>
     </row>
     <row r="136" ht="16" customHeight="1">
       <c r="A136" s="73" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>央视台球</t>
         </is>
       </c>
       <c r="B136" s="74" t="inlineStr">
@@ -11057,14 +11057,14 @@
       </c>
       <c r="C136" s="75" t="inlineStr">
         <is>
-          <t>https://v4-702cae17a28d6e4f0c0002bba021d934.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=5536bf33e2ea132eae60addc6ecb090d</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=ystq</t>
         </is>
       </c>
     </row>
     <row r="137" ht="16" customHeight="1">
       <c r="A137" s="70" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>怀旧剧场</t>
         </is>
       </c>
       <c r="B137" s="71" t="inlineStr">
@@ -11074,14 +11074,14 @@
       </c>
       <c r="C137" s="72" t="inlineStr">
         <is>
-          <t>http://192.151.150.154/live/cctv9hd.m3u8</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=hjjc</t>
         </is>
       </c>
     </row>
     <row r="138" ht="16" customHeight="1">
       <c r="A138" s="73" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>笑看风云</t>
         </is>
       </c>
       <c r="B138" s="74" t="inlineStr">
@@ -11091,14 +11091,14 @@
       </c>
       <c r="C138" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv9hd.m3u8</t>
+          <t>https://live.metshop.top/huya/29465858</t>
         </is>
       </c>
     </row>
     <row r="139" ht="16" customHeight="1">
       <c r="A139" s="70" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>韩国电影1</t>
         </is>
       </c>
       <c r="B139" s="71" t="inlineStr">
@@ -11108,14 +11108,14 @@
       </c>
       <c r="C139" s="72" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv9hd</t>
+          <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=595</t>
         </is>
       </c>
     </row>
     <row r="140" ht="16" customHeight="1">
       <c r="A140" s="73" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>韩国电影2</t>
         </is>
       </c>
       <c r="B140" s="74" t="inlineStr">
@@ -11125,14 +11125,14 @@
       </c>
       <c r="C140" s="75" t="inlineStr">
         <is>
-          <t>http://107.150.60.122/live/cctv9hd.m3u8</t>
+          <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=743</t>
         </is>
       </c>
     </row>
     <row r="141" ht="16" customHeight="1">
       <c r="A141" s="70" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>风云剧场</t>
         </is>
       </c>
       <c r="B141" s="71" t="inlineStr">
@@ -11142,14 +11142,14 @@
       </c>
       <c r="C141" s="72" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyjc</t>
         </is>
       </c>
     </row>
     <row r="142" ht="16" customHeight="1">
       <c r="A142" s="73" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>风云足球</t>
         </is>
       </c>
       <c r="B142" s="74" t="inlineStr">
@@ -11159,14 +11159,14 @@
       </c>
       <c r="C142" s="75" t="inlineStr">
         <is>
-          <t>http://116.128.243.121:85/tsfile/live/1009_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyzq</t>
         </is>
       </c>
     </row>
     <row r="143" ht="16" customHeight="1">
       <c r="A143" s="70" t="inlineStr">
         <is>
-          <t>CCTV-9_1</t>
+          <t>风云音乐</t>
         </is>
       </c>
       <c r="B143" s="71" t="inlineStr">
@@ -11175,363 +11175,6 @@
         </is>
       </c>
       <c r="C143" s="72" t="inlineStr">
-        <is>
-          <t>https://xykt-fix.github.io/Y77.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="144" ht="16" customHeight="1">
-      <c r="A144" s="73" t="inlineStr">
-        <is>
-          <t>CCTV-9_6</t>
-        </is>
-      </c>
-      <c r="B144" s="74" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C144" s="75" t="inlineStr">
-        <is>
-          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=db000b5568ff643131ea7d86610b09b7</t>
-        </is>
-      </c>
-    </row>
-    <row r="145" ht="16" customHeight="1">
-      <c r="A145" s="70" t="inlineStr">
-        <is>
-          <t>CCTV-9纪录</t>
-        </is>
-      </c>
-      <c r="B145" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C145" s="72" t="inlineStr">
-        <is>
-          <t>http://74.91.26.218:82/live/cctv9hd.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="146" ht="16" customHeight="1">
-      <c r="A146" s="73" t="inlineStr">
-        <is>
-          <t>CCTV-9纪录</t>
-        </is>
-      </c>
-      <c r="B146" s="74" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C146" s="75" t="inlineStr">
-        <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv9hd</t>
-        </is>
-      </c>
-    </row>
-    <row r="147" ht="16" customHeight="1">
-      <c r="A147" s="70" t="inlineStr">
-        <is>
-          <t>CCTV-女性時尚</t>
-        </is>
-      </c>
-      <c r="B147" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C147" s="72" t="inlineStr">
-        <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/nxss.m3u8?auth=testpub</t>
-        </is>
-      </c>
-    </row>
-    <row r="148" ht="16" customHeight="1">
-      <c r="A148" s="73" t="inlineStr">
-        <is>
-          <t>CCTV-懷舊劇場</t>
-        </is>
-      </c>
-      <c r="B148" s="74" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C148" s="75" t="inlineStr">
-        <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/hjjc.m3u8?auth=testpub</t>
-        </is>
-      </c>
-    </row>
-    <row r="149" ht="16" customHeight="1">
-      <c r="A149" s="70" t="inlineStr">
-        <is>
-          <t>CCTV-衛生健康</t>
-        </is>
-      </c>
-      <c r="B149" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C149" s="72" t="inlineStr">
-        <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/wsjk.m3u8?auth=testpub</t>
-        </is>
-      </c>
-    </row>
-    <row r="150" ht="16" customHeight="1">
-      <c r="A150" s="73" t="inlineStr">
-        <is>
-          <t>CCTV13</t>
-        </is>
-      </c>
-      <c r="B150" s="74" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C150" s="75" t="inlineStr">
-        <is>
-          <t>http://ali-m-l.cztv.com/channels/lantian/channel21/1080p.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="151" ht="16" customHeight="1">
-      <c r="A151" s="70" t="inlineStr">
-        <is>
-          <t>CGTN纪录</t>
-        </is>
-      </c>
-      <c r="B151" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C151" s="72" t="inlineStr">
-        <is>
-          <t>http://english-livebkali.cgtn.com/live/doccgtn_0.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="152" ht="16" customHeight="1">
-      <c r="A152" s="73" t="inlineStr">
-        <is>
-          <t>CGTN英语</t>
-        </is>
-      </c>
-      <c r="B152" s="74" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C152" s="75" t="inlineStr">
-        <is>
-          <t>https://english-livebkali.cgtn.com/live/encgtn_0.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="153" ht="16" customHeight="1">
-      <c r="A153" s="70" t="inlineStr">
-        <is>
-          <t>F1 TV</t>
-        </is>
-      </c>
-      <c r="B153" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C153" s="72" t="inlineStr">
-        <is>
-          <t>https://amg12058-c15studio-amg12058c1-lg-us-5787.playouts.now.amagi.tv/playlist.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="154" ht="16" customHeight="1">
-      <c r="A154" s="73" t="inlineStr">
-        <is>
-          <t>PGA Tour_4</t>
-        </is>
-      </c>
-      <c r="B154" s="74" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C154" s="75" t="inlineStr">
-        <is>
-          <t>https://d11k1mnrgfposz.cloudfront.net/playlist.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="155" ht="16" customHeight="1">
-      <c r="A155" s="70" t="inlineStr">
-        <is>
-          <t>世界地理</t>
-        </is>
-      </c>
-      <c r="B155" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C155" s="72" t="inlineStr">
-        <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=sjdl</t>
-        </is>
-      </c>
-    </row>
-    <row r="156" ht="16" customHeight="1">
-      <c r="A156" s="73" t="inlineStr">
-        <is>
-          <t>兵器科技</t>
-        </is>
-      </c>
-      <c r="B156" s="74" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C156" s="75" t="inlineStr">
-        <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=gfjs</t>
-        </is>
-      </c>
-    </row>
-    <row r="157" ht="16" customHeight="1">
-      <c r="A157" s="70" t="inlineStr">
-        <is>
-          <t>央视台球</t>
-        </is>
-      </c>
-      <c r="B157" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C157" s="72" t="inlineStr">
-        <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=ystq</t>
-        </is>
-      </c>
-    </row>
-    <row r="158" ht="16" customHeight="1">
-      <c r="A158" s="73" t="inlineStr">
-        <is>
-          <t>怀旧剧场</t>
-        </is>
-      </c>
-      <c r="B158" s="74" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C158" s="75" t="inlineStr">
-        <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=hjjc</t>
-        </is>
-      </c>
-    </row>
-    <row r="159" ht="16" customHeight="1">
-      <c r="A159" s="70" t="inlineStr">
-        <is>
-          <t>笑看风云</t>
-        </is>
-      </c>
-      <c r="B159" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C159" s="72" t="inlineStr">
-        <is>
-          <t>https://live.metshop.top/huya/29465858</t>
-        </is>
-      </c>
-    </row>
-    <row r="160" ht="16" customHeight="1">
-      <c r="A160" s="73" t="inlineStr">
-        <is>
-          <t>韩国电影1</t>
-        </is>
-      </c>
-      <c r="B160" s="74" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C160" s="75" t="inlineStr">
-        <is>
-          <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=595</t>
-        </is>
-      </c>
-    </row>
-    <row r="161" ht="16" customHeight="1">
-      <c r="A161" s="70" t="inlineStr">
-        <is>
-          <t>韩国电影2</t>
-        </is>
-      </c>
-      <c r="B161" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C161" s="72" t="inlineStr">
-        <is>
-          <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=743</t>
-        </is>
-      </c>
-    </row>
-    <row r="162" ht="16" customHeight="1">
-      <c r="A162" s="73" t="inlineStr">
-        <is>
-          <t>风云剧场</t>
-        </is>
-      </c>
-      <c r="B162" s="74" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C162" s="75" t="inlineStr">
-        <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyjc</t>
-        </is>
-      </c>
-    </row>
-    <row r="163" ht="16" customHeight="1">
-      <c r="A163" s="70" t="inlineStr">
-        <is>
-          <t>风云足球</t>
-        </is>
-      </c>
-      <c r="B163" s="71" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C163" s="72" t="inlineStr">
-        <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyzq</t>
-        </is>
-      </c>
-    </row>
-    <row r="164" ht="16" customHeight="1">
-      <c r="A164" s="73" t="inlineStr">
-        <is>
-          <t>风云音乐</t>
-        </is>
-      </c>
-      <c r="B164" s="74" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C164" s="75" t="inlineStr">
         <is>
           <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyyy</t>
         </is>

</xml_diff>

<commit_message>
feat: integrate 24H Korean news live streams into periodic and daily sync
</commit_message>
<xml_diff>
--- a/channels_overview.xlsx
+++ b/channels_overview.xlsx
@@ -1718,7 +1718,7 @@
         </is>
       </c>
       <c r="B27" s="62" t="n">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="C27" s="63" t="inlineStr">
         <is>
@@ -1778,7 +1778,7 @@
         </is>
       </c>
       <c r="B31" s="70" t="n">
-        <v>3381</v>
+        <v>3387</v>
       </c>
       <c r="C31" s="70" t="n"/>
     </row>
@@ -38210,7 +38210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C144"/>
+  <dimension ref="A1:C150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -38221,7 +38221,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="150" t="inlineStr">
         <is>
-          <t>📺  🇰🇷 韩国 · 🇰🇵 朝鲜  —  共 142 条频道</t>
+          <t>📺  🇰🇷 韩国 · 🇰🇵 朝鲜  —  共 148 条频道</t>
         </is>
       </c>
     </row>
@@ -38687,7 +38687,7 @@
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="151" t="inlineStr">
         <is>
-          <t>K-ASMR</t>
+          <t>JTBC新闻</t>
         </is>
       </c>
       <c r="B29" s="152" t="inlineStr">
@@ -38697,14 +38697,14 @@
       </c>
       <c r="C29" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC41000021C</t>
+          <t>https://www.youtube.com/embed/HnUd-KtQNac</t>
         </is>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="76" t="inlineStr">
         <is>
-          <t>KBS 1박2일 시즌1</t>
+          <t>K-ASMR</t>
         </is>
       </c>
       <c r="B30" s="77" t="inlineStr">
@@ -38714,14 +38714,14 @@
       </c>
       <c r="C30" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC4400003SD</t>
+          <t>https://jmp2.uk/stvp-KRBC41000021C</t>
         </is>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
       <c r="A31" s="151" t="inlineStr">
         <is>
-          <t>KBS America</t>
+          <t>KBS 1박2일 시즌1</t>
         </is>
       </c>
       <c r="B31" s="152" t="inlineStr">
@@ -38731,14 +38731,14 @@
       </c>
       <c r="C31" s="153" t="inlineStr">
         <is>
-          <t>https://xyktmobile00.s.gy/PPV918_KBSAMERI</t>
+          <t>https://jmp2.uk/stvp-KRBC4400003SD</t>
         </is>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
       <c r="A32" s="76" t="inlineStr">
         <is>
-          <t>KBS HOT CLIP 예능</t>
+          <t>KBS America</t>
         </is>
       </c>
       <c r="B32" s="77" t="inlineStr">
@@ -38748,14 +38748,14 @@
       </c>
       <c r="C32" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR45000060I</t>
+          <t>https://xyktmobile00.s.gy/PPV918_KBSAMERI</t>
         </is>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="151" t="inlineStr">
         <is>
-          <t>KBS HOT CLIP 음악</t>
+          <t>KBS HOT CLIP 예능</t>
         </is>
       </c>
       <c r="B33" s="152" t="inlineStr">
@@ -38765,14 +38765,14 @@
       </c>
       <c r="C33" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR45000052W</t>
+          <t>https://jmp2.uk/stvp-KR45000060I</t>
         </is>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="76" t="inlineStr">
         <is>
-          <t>KBS Joy 무엇이든 물어보살</t>
+          <t>KBS HOT CLIP 음악</t>
         </is>
       </c>
       <c r="B34" s="77" t="inlineStr">
@@ -38782,14 +38782,14 @@
       </c>
       <c r="C34" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC3200009M7</t>
+          <t>https://jmp2.uk/stvp-KR45000052W</t>
         </is>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="151" t="inlineStr">
         <is>
-          <t>KBS Joy 연애의 참견</t>
+          <t>KBS Joy 무엇이든 물어보살</t>
         </is>
       </c>
       <c r="B35" s="152" t="inlineStr">
@@ -38799,14 +38799,14 @@
       </c>
       <c r="C35" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC4000005EP</t>
+          <t>https://jmp2.uk/stvp-KRBC3200009M7</t>
         </is>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="76" t="inlineStr">
         <is>
-          <t>KBS 개그콘서트</t>
+          <t>KBS Joy 연애의 참견</t>
         </is>
       </c>
       <c r="B36" s="77" t="inlineStr">
@@ -38816,14 +38816,14 @@
       </c>
       <c r="C36" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR700003L9</t>
+          <t>https://jmp2.uk/stvp-KRBC4000005EP</t>
         </is>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
       <c r="A37" s="151" t="inlineStr">
         <is>
-          <t>KBS 구르미 그린 달빛</t>
+          <t>KBS World</t>
         </is>
       </c>
       <c r="B37" s="152" t="inlineStr">
@@ -38833,14 +38833,14 @@
       </c>
       <c r="C37" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR7000023Z</t>
+          <t>https://www.youtube.com/embed/U2faSnFEi3k</t>
         </is>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1">
       <c r="A38" s="76" t="inlineStr">
         <is>
-          <t>KBS 뉴스24</t>
+          <t>KBS 개그콘서트</t>
         </is>
       </c>
       <c r="B38" s="77" t="inlineStr">
@@ -38850,14 +38850,14 @@
       </c>
       <c r="C38" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR5100001TH</t>
+          <t>https://jmp2.uk/stvp-KR700003L9</t>
         </is>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1">
       <c r="A39" s="151" t="inlineStr">
         <is>
-          <t>KBS 신사와 아가씨</t>
+          <t>KBS 구르미 그린 달빛</t>
         </is>
       </c>
       <c r="B39" s="152" t="inlineStr">
@@ -38867,14 +38867,14 @@
       </c>
       <c r="C39" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC4400001TZ</t>
+          <t>https://jmp2.uk/stvp-KR7000023Z</t>
         </is>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
       <c r="A40" s="76" t="inlineStr">
         <is>
-          <t>KBS 최고다 이순신</t>
+          <t>KBS 뉴스24</t>
         </is>
       </c>
       <c r="B40" s="77" t="inlineStr">
@@ -38884,14 +38884,14 @@
       </c>
       <c r="C40" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC4400002AO</t>
+          <t>https://jmp2.uk/stvp-KR5100001TH</t>
         </is>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="151" t="inlineStr">
         <is>
-          <t>KBS 태조 왕건</t>
+          <t>KBS 신사와 아가씨</t>
         </is>
       </c>
       <c r="B41" s="152" t="inlineStr">
@@ -38901,14 +38901,14 @@
       </c>
       <c r="C41" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR4600012CR</t>
+          <t>https://jmp2.uk/stvp-KRBC4400001TZ</t>
         </is>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1">
       <c r="A42" s="76" t="inlineStr">
         <is>
-          <t>KBSWorld</t>
+          <t>KBS 최고다 이순신</t>
         </is>
       </c>
       <c r="B42" s="77" t="inlineStr">
@@ -38918,14 +38918,14 @@
       </c>
       <c r="C42" s="78" t="inlineStr">
         <is>
-          <t>https://cdn4.skygo.mn/live/disk1/KBSWorld/HLSv3-FTA/KBSWorld.m3u8</t>
+          <t>https://jmp2.uk/stvp-KRBC4400002AO</t>
         </is>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="151" t="inlineStr">
         <is>
-          <t>LLBN TV Korean</t>
+          <t>KBS 태조 왕건</t>
         </is>
       </c>
       <c r="B43" s="152" t="inlineStr">
@@ -38935,14 +38935,14 @@
       </c>
       <c r="C43" s="153" t="inlineStr">
         <is>
-          <t>https://brightstar-korean-pull-secure.akamaized.net/brightstarkorean/stream.m3u8</t>
+          <t>https://jmp2.uk/stvp-KR4600012CR</t>
         </is>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1">
       <c r="A44" s="76" t="inlineStr">
         <is>
-          <t>MBC America</t>
+          <t>KBSWorld</t>
         </is>
       </c>
       <c r="B44" s="77" t="inlineStr">
@@ -38952,14 +38952,14 @@
       </c>
       <c r="C44" s="78" t="inlineStr">
         <is>
-          <t>https://cdn-us-east-prod-ingest-infra-dacast-com.akamaized.net/624ff8f9-db18-da92-4d42-896fa2ff3eb3/source/index.m3u8</t>
+          <t>https://cdn4.skygo.mn/live/disk1/KBSWorld/HLSv3-FTA/KBSWorld.m3u8</t>
         </is>
       </c>
     </row>
     <row r="45" ht="16" customHeight="1">
       <c r="A45" s="151" t="inlineStr">
         <is>
-          <t>MBC Drama USA</t>
+          <t>KBS新闻</t>
         </is>
       </c>
       <c r="B45" s="152" t="inlineStr">
@@ -38969,14 +38969,14 @@
       </c>
       <c r="C45" s="153" t="inlineStr">
         <is>
-          <t>https://shd-gcp-live.edgenextcdn.net/live/bitmovin-mbc-drama-usa/ea2f5db904aff224b7066e59c7f585a2/index.m3u8</t>
+          <t>https://www.youtube.com/embed/2mCSYvcfhtc</t>
         </is>
       </c>
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="76" t="inlineStr">
         <is>
-          <t>MBC HOT CLIP 드라마</t>
+          <t>LLBN TV Korean</t>
         </is>
       </c>
       <c r="B46" s="77" t="inlineStr">
@@ -38986,14 +38986,14 @@
       </c>
       <c r="C46" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR4500001KZ</t>
+          <t>https://brightstar-korean-pull-secure.akamaized.net/brightstarkorean/stream.m3u8</t>
         </is>
       </c>
     </row>
     <row r="47" ht="16" customHeight="1">
       <c r="A47" s="151" t="inlineStr">
         <is>
-          <t>MBC HOT CLIP 예능</t>
+          <t>MBC America</t>
         </is>
       </c>
       <c r="B47" s="152" t="inlineStr">
@@ -39003,14 +39003,14 @@
       </c>
       <c r="C47" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR4500002GS</t>
+          <t>https://cdn-us-east-prod-ingest-infra-dacast-com.akamaized.net/624ff8f9-db18-da92-4d42-896fa2ff3eb3/source/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="48" ht="16" customHeight="1">
       <c r="A48" s="76" t="inlineStr">
         <is>
-          <t>MBC every1 별순검</t>
+          <t>MBC Drama USA</t>
         </is>
       </c>
       <c r="B48" s="77" t="inlineStr">
@@ -39020,14 +39020,14 @@
       </c>
       <c r="C48" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB500037T3</t>
+          <t>https://shd-gcp-live.edgenextcdn.net/live/bitmovin-mbc-drama-usa/ea2f5db904aff224b7066e59c7f585a2/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1">
       <c r="A49" s="151" t="inlineStr">
         <is>
-          <t>MBC every1 어서와 한국은 처음이지?</t>
+          <t>MBC HOT CLIP 드라마</t>
         </is>
       </c>
       <c r="B49" s="152" t="inlineStr">
@@ -39037,14 +39037,14 @@
       </c>
       <c r="C49" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB500034DY</t>
+          <t>https://jmp2.uk/stvp-KR4500001KZ</t>
         </is>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="76" t="inlineStr">
         <is>
-          <t>MBC 거침없이 하이킥</t>
+          <t>MBC HOT CLIP 예능</t>
         </is>
       </c>
       <c r="B50" s="77" t="inlineStr">
@@ -39054,14 +39054,14 @@
       </c>
       <c r="C50" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC2000010X</t>
+          <t>https://jmp2.uk/stvp-KR4500002GS</t>
         </is>
       </c>
     </row>
     <row r="51" ht="16" customHeight="1">
       <c r="A51" s="151" t="inlineStr">
         <is>
-          <t>MBC 구해줘홈즈</t>
+          <t>MBC every1 별순검</t>
         </is>
       </c>
       <c r="B51" s="152" t="inlineStr">
@@ -39071,14 +39071,14 @@
       </c>
       <c r="C51" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR4800003H0</t>
+          <t>https://jmp2.uk/stvp-KRBB500037T3</t>
         </is>
       </c>
     </row>
     <row r="52" ht="16" customHeight="1">
       <c r="A52" s="76" t="inlineStr">
         <is>
-          <t>MBC 나혼자산다</t>
+          <t>MBC every1 어서와 한국은 처음이지?</t>
         </is>
       </c>
       <c r="B52" s="77" t="inlineStr">
@@ -39088,14 +39088,14 @@
       </c>
       <c r="C52" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC200002I0</t>
+          <t>https://jmp2.uk/stvp-KRBB500034DY</t>
         </is>
       </c>
     </row>
     <row r="53" ht="16" customHeight="1">
       <c r="A53" s="151" t="inlineStr">
         <is>
-          <t>MBC 놀면 뭐하니</t>
+          <t>MBC 거침없이 하이킥</t>
         </is>
       </c>
       <c r="B53" s="152" t="inlineStr">
@@ -39105,14 +39105,14 @@
       </c>
       <c r="C53" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB5000073UD</t>
+          <t>https://jmp2.uk/stvp-KRBC2000010X</t>
         </is>
       </c>
     </row>
     <row r="54" ht="16" customHeight="1">
       <c r="A54" s="76" t="inlineStr">
         <is>
-          <t>MBC 라디오스타</t>
+          <t>MBC 구해줘홈즈</t>
         </is>
       </c>
       <c r="B54" s="77" t="inlineStr">
@@ -39122,14 +39122,14 @@
       </c>
       <c r="C54" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR48000047I</t>
+          <t>https://jmp2.uk/stvp-KR4800003H0</t>
         </is>
       </c>
     </row>
     <row r="55" ht="16" customHeight="1">
       <c r="A55" s="151" t="inlineStr">
         <is>
-          <t>MBC 무한도전</t>
+          <t>MBC 나혼자산다</t>
         </is>
       </c>
       <c r="B55" s="152" t="inlineStr">
@@ -39139,14 +39139,14 @@
       </c>
       <c r="C55" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB5000069BS</t>
+          <t>https://jmp2.uk/stvp-KRBC200002I0</t>
         </is>
       </c>
     </row>
     <row r="56" ht="16" customHeight="1">
       <c r="A56" s="76" t="inlineStr">
         <is>
-          <t>MBC 밤에 피는 꽃</t>
+          <t>MBC 놀면 뭐하니</t>
         </is>
       </c>
       <c r="B56" s="77" t="inlineStr">
@@ -39156,14 +39156,14 @@
       </c>
       <c r="C56" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB5000070U4</t>
+          <t>https://jmp2.uk/stvp-KRBB5000073UD</t>
         </is>
       </c>
     </row>
     <row r="57" ht="16" customHeight="1">
       <c r="A57" s="151" t="inlineStr">
         <is>
-          <t>MBC 심야괴담회</t>
+          <t>MBC 라디오스타</t>
         </is>
       </c>
       <c r="B57" s="152" t="inlineStr">
@@ -39173,14 +39173,14 @@
       </c>
       <c r="C57" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB50000711L</t>
+          <t>https://jmp2.uk/stvp-KR48000047I</t>
         </is>
       </c>
     </row>
     <row r="58" ht="16" customHeight="1">
       <c r="A58" s="76" t="inlineStr">
         <is>
-          <t>MBC 안싸우면 다행이야</t>
+          <t>MBC 무한도전</t>
         </is>
       </c>
       <c r="B58" s="77" t="inlineStr">
@@ -39190,14 +39190,14 @@
       </c>
       <c r="C58" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC20000347</t>
+          <t>https://jmp2.uk/stvp-KRBB5000069BS</t>
         </is>
       </c>
     </row>
     <row r="59" ht="16" customHeight="1">
       <c r="A59" s="151" t="inlineStr">
         <is>
-          <t>MBC 오은영리포트 결혼지옥</t>
+          <t>MBC 밤에 피는 꽃</t>
         </is>
       </c>
       <c r="B59" s="152" t="inlineStr">
@@ -39207,14 +39207,14 @@
       </c>
       <c r="C59" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB50000721W</t>
+          <t>https://jmp2.uk/stvp-KRBB5000070U4</t>
         </is>
       </c>
     </row>
     <row r="60" ht="16" customHeight="1">
       <c r="A60" s="76" t="inlineStr">
         <is>
-          <t>MBC 전지적 참견 시점</t>
+          <t>MBC 심야괴담회</t>
         </is>
       </c>
       <c r="B60" s="77" t="inlineStr">
@@ -39224,14 +39224,14 @@
       </c>
       <c r="C60" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC20000418</t>
+          <t>https://jmp2.uk/stvp-KRBB50000711L</t>
         </is>
       </c>
     </row>
     <row r="61" ht="16" customHeight="1">
       <c r="A61" s="151" t="inlineStr">
         <is>
-          <t>MBC 지붕뚫고 하이킥</t>
+          <t>MBC 안싸우면 다행이야</t>
         </is>
       </c>
       <c r="B61" s="152" t="inlineStr">
@@ -39241,14 +39241,14 @@
       </c>
       <c r="C61" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC200005H6</t>
+          <t>https://jmp2.uk/stvp-KRBC20000347</t>
         </is>
       </c>
     </row>
     <row r="62" ht="16" customHeight="1">
       <c r="A62" s="76" t="inlineStr">
         <is>
-          <t>MBN 나는 자연인이다</t>
+          <t>MBC 오은영리포트 결혼지옥</t>
         </is>
       </c>
       <c r="B62" s="77" t="inlineStr">
@@ -39258,14 +39258,14 @@
       </c>
       <c r="C62" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC3500017PO</t>
+          <t>https://jmp2.uk/stvp-KRBB50000721W</t>
         </is>
       </c>
     </row>
     <row r="63" ht="16" customHeight="1">
       <c r="A63" s="151" t="inlineStr">
         <is>
-          <t>MBN 뉴스</t>
+          <t>MBC 전지적 참견 시점</t>
         </is>
       </c>
       <c r="B63" s="152" t="inlineStr">
@@ -39275,14 +39275,14 @@
       </c>
       <c r="C63" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC4000003J2</t>
+          <t>https://jmp2.uk/stvp-KRBC20000418</t>
         </is>
       </c>
     </row>
     <row r="64" ht="16" customHeight="1">
       <c r="A64" s="76" t="inlineStr">
         <is>
-          <t>MBN 속풀이쇼 동치미</t>
+          <t>MBC 지붕뚫고 하이킥</t>
         </is>
       </c>
       <c r="B64" s="77" t="inlineStr">
@@ -39292,14 +39292,14 @@
       </c>
       <c r="C64" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC3500019CD</t>
+          <t>https://jmp2.uk/stvp-KRBC200005H6</t>
         </is>
       </c>
     </row>
     <row r="65" ht="16" customHeight="1">
       <c r="A65" s="151" t="inlineStr">
         <is>
-          <t>MBN 휴먼다큐 사노라면</t>
+          <t>MBC新闻</t>
         </is>
       </c>
       <c r="B65" s="152" t="inlineStr">
@@ -39309,14 +39309,14 @@
       </c>
       <c r="C65" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC3500018J9</t>
+          <t>https://www.youtube.com/embed/rEKifG2XUZg</t>
         </is>
       </c>
     </row>
     <row r="66" ht="16" customHeight="1">
       <c r="A66" s="76" t="inlineStr">
         <is>
-          <t>Mr. Bean</t>
+          <t>MBN 나는 자연인이다</t>
         </is>
       </c>
       <c r="B66" s="77" t="inlineStr">
@@ -39326,14 +39326,14 @@
       </c>
       <c r="C66" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR2400001TI</t>
+          <t>https://jmp2.uk/stvp-KRBC3500017PO</t>
         </is>
       </c>
     </row>
     <row r="67" ht="16" customHeight="1">
       <c r="A67" s="151" t="inlineStr">
         <is>
-          <t>OGN 스타리그</t>
+          <t>MBN 뉴스</t>
         </is>
       </c>
       <c r="B67" s="152" t="inlineStr">
@@ -39343,14 +39343,14 @@
       </c>
       <c r="C67" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC3200005SH</t>
+          <t>https://jmp2.uk/stvp-KRBC4000003J2</t>
         </is>
       </c>
     </row>
     <row r="68" ht="16" customHeight="1">
       <c r="A68" s="76" t="inlineStr">
         <is>
-          <t>PGA Tour_3</t>
+          <t>MBN 속풀이쇼 동치미</t>
         </is>
       </c>
       <c r="B68" s="77" t="inlineStr">
@@ -39360,14 +39360,14 @@
       </c>
       <c r="C68" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBD3100007WB</t>
+          <t>https://jmp2.uk/stvp-KRBC3500019CD</t>
         </is>
       </c>
     </row>
     <row r="69" ht="16" customHeight="1">
       <c r="A69" s="151" t="inlineStr">
         <is>
-          <t>PLAYGRAM MOVIES</t>
+          <t>MBN 휴먼다큐 사노라면</t>
         </is>
       </c>
       <c r="B69" s="152" t="inlineStr">
@@ -39377,14 +39377,14 @@
       </c>
       <c r="C69" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC3200004D1</t>
+          <t>https://jmp2.uk/stvp-KRBC3500018J9</t>
         </is>
       </c>
     </row>
     <row r="70" ht="16" customHeight="1">
       <c r="A70" s="76" t="inlineStr">
         <is>
-          <t>SBS Drama</t>
+          <t>Mr. Bean</t>
         </is>
       </c>
       <c r="B70" s="77" t="inlineStr">
@@ -39394,14 +39394,14 @@
       </c>
       <c r="C70" s="78" t="inlineStr">
         <is>
-          <t>https://ads.its-newid.net/api/manifest.m3u8?tp=lg_channels&amp;channel_name=sbsk-drama&amp;channel_id=newid_008&amp;mpf=c064f5f4-39af1962-7c36be2c&amp;apikey=48230e6b-1cea0097-15975f93-39af1962&amp;auth=474ab4cb-5d47aa0a-84d0cbca-2a3730a6&amp;ads.live=[CONTENT_LIVE]&amp;ads.deviceid=[DEVICE_ID]&amp;ads.ifa=[IFA]&amp;ads.ifatype=[IFA_TYPE]&amp;ads.lat=[LMT]&amp;ads.donotsell=[DNS]&amp;ads.ua=[UA]&amp;ads.ip=[IP]&amp;ads.gdpr=[GDPR]&amp;ads.gdpr_consent=[GDPR_CONSENT]&amp;ads.country=[COUNTRY]&amp;ads.us_privacy=[US_PRIVACY]&amp;ads.appstoreurl=[APP_STOREURL]&amp;ads.bundleid=[APP_BUNDLE]&amp;ads.appname=[APP_NAME]&amp;ads.appversion=[APP_VERSION]&amp;ads.devicetype=[DEVICE_TYPE]&amp;ads.devicemake=[DEVICE_MAKE]&amp;ads.devicemodel=[DEVICE_MODEL]&amp;ads.targetad=[TARGETAD_ALLOWED]&amp;ads.fck=[FCK]&amp;ads.viewsize=[VIEWSIZE]&amp;ads.givn=[NONCE]</t>
+          <t>https://jmp2.uk/stvp-KR2400001TI</t>
         </is>
       </c>
     </row>
     <row r="71" ht="16" customHeight="1">
       <c r="A71" s="151" t="inlineStr">
         <is>
-          <t>SBS HOT CLIP 드라마</t>
+          <t>OGN 스타리그</t>
         </is>
       </c>
       <c r="B71" s="152" t="inlineStr">
@@ -39411,14 +39411,14 @@
       </c>
       <c r="C71" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR4500003V9</t>
+          <t>https://jmp2.uk/stvp-KRBC3200005SH</t>
         </is>
       </c>
     </row>
     <row r="72" ht="16" customHeight="1">
       <c r="A72" s="76" t="inlineStr">
         <is>
-          <t>SBS HOT CLIP 예능</t>
+          <t>PGA Tour_3</t>
         </is>
       </c>
       <c r="B72" s="77" t="inlineStr">
@@ -39428,14 +39428,14 @@
       </c>
       <c r="C72" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR4500004XC</t>
+          <t>https://jmp2.uk/stvp-KRBD3100007WB</t>
         </is>
       </c>
     </row>
     <row r="73" ht="16" customHeight="1">
       <c r="A73" s="151" t="inlineStr">
         <is>
-          <t>SBS No.1 뉴스라이브</t>
+          <t>PLAYGRAM MOVIES</t>
         </is>
       </c>
       <c r="B73" s="152" t="inlineStr">
@@ -39445,14 +39445,14 @@
       </c>
       <c r="C73" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR4500008DI</t>
+          <t>https://jmp2.uk/stvp-KRBC3200004D1</t>
         </is>
       </c>
     </row>
     <row r="74" ht="16" customHeight="1">
       <c r="A74" s="76" t="inlineStr">
         <is>
-          <t>SBS TV 동물농장</t>
+          <t>SBS Drama</t>
         </is>
       </c>
       <c r="B74" s="77" t="inlineStr">
@@ -39462,14 +39462,14 @@
       </c>
       <c r="C74" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB420000769</t>
+          <t>https://ads.its-newid.net/api/manifest.m3u8?tp=lg_channels&amp;channel_name=sbsk-drama&amp;channel_id=newid_008&amp;mpf=c064f5f4-39af1962-7c36be2c&amp;apikey=48230e6b-1cea0097-15975f93-39af1962&amp;auth=474ab4cb-5d47aa0a-84d0cbca-2a3730a6&amp;ads.live=[CONTENT_LIVE]&amp;ads.deviceid=[DEVICE_ID]&amp;ads.ifa=[IFA]&amp;ads.ifatype=[IFA_TYPE]&amp;ads.lat=[LMT]&amp;ads.donotsell=[DNS]&amp;ads.ua=[UA]&amp;ads.ip=[IP]&amp;ads.gdpr=[GDPR]&amp;ads.gdpr_consent=[GDPR_CONSENT]&amp;ads.country=[COUNTRY]&amp;ads.us_privacy=[US_PRIVACY]&amp;ads.appstoreurl=[APP_STOREURL]&amp;ads.bundleid=[APP_BUNDLE]&amp;ads.appname=[APP_NAME]&amp;ads.appversion=[APP_VERSION]&amp;ads.devicetype=[DEVICE_TYPE]&amp;ads.devicemake=[DEVICE_MAKE]&amp;ads.devicemodel=[DEVICE_MODEL]&amp;ads.targetad=[TARGETAD_ALLOWED]&amp;ads.fck=[FCK]&amp;ads.viewsize=[VIEWSIZE]&amp;ads.givn=[NONCE]</t>
         </is>
       </c>
     </row>
     <row r="75" ht="16" customHeight="1">
       <c r="A75" s="151" t="inlineStr">
         <is>
-          <t>SBS 궁금한 이야기 Y</t>
+          <t>SBS HOT CLIP 드라마</t>
         </is>
       </c>
       <c r="B75" s="152" t="inlineStr">
@@ -39479,14 +39479,14 @@
       </c>
       <c r="C75" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB4200016TZ</t>
+          <t>https://jmp2.uk/stvp-KR4500003V9</t>
         </is>
       </c>
     </row>
     <row r="76" ht="16" customHeight="1">
       <c r="A76" s="76" t="inlineStr">
         <is>
-          <t>SBS 그것이 알고싶다</t>
+          <t>SBS HOT CLIP 예능</t>
         </is>
       </c>
       <c r="B76" s="77" t="inlineStr">
@@ -39496,14 +39496,14 @@
       </c>
       <c r="C76" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB4200017HA</t>
+          <t>https://jmp2.uk/stvp-KR4500004XC</t>
         </is>
       </c>
     </row>
     <row r="77" ht="16" customHeight="1">
       <c r="A77" s="151" t="inlineStr">
         <is>
-          <t>SBS 내 남자의 여자</t>
+          <t>SBS No.1 뉴스라이브</t>
         </is>
       </c>
       <c r="B77" s="152" t="inlineStr">
@@ -39513,14 +39513,14 @@
       </c>
       <c r="C77" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB4200005CK</t>
+          <t>https://jmp2.uk/stvp-KR4500008DI</t>
         </is>
       </c>
     </row>
     <row r="78" ht="16" customHeight="1">
       <c r="A78" s="76" t="inlineStr">
         <is>
-          <t>SBS 런닝맨</t>
+          <t>SBS TV 동물농장</t>
         </is>
       </c>
       <c r="B78" s="77" t="inlineStr">
@@ -39530,14 +39530,14 @@
       </c>
       <c r="C78" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB4200002MM</t>
+          <t>https://jmp2.uk/stvp-KRBB420000769</t>
         </is>
       </c>
     </row>
     <row r="79" ht="16" customHeight="1">
       <c r="A79" s="151" t="inlineStr">
         <is>
-          <t>SBS 모범택시</t>
+          <t>SBS 궁금한 이야기 Y</t>
         </is>
       </c>
       <c r="B79" s="152" t="inlineStr">
@@ -39547,14 +39547,14 @@
       </c>
       <c r="C79" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB420000180</t>
+          <t>https://jmp2.uk/stvp-KRBB4200016TZ</t>
         </is>
       </c>
     </row>
     <row r="80" ht="16" customHeight="1">
       <c r="A80" s="76" t="inlineStr">
         <is>
-          <t>SBS 미운 우리 새끼</t>
+          <t>SBS 그것이 알고싶다</t>
         </is>
       </c>
       <c r="B80" s="77" t="inlineStr">
@@ -39564,14 +39564,14 @@
       </c>
       <c r="C80" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB4200003ZL</t>
+          <t>https://jmp2.uk/stvp-KRBB4200017HA</t>
         </is>
       </c>
     </row>
     <row r="81" ht="16" customHeight="1">
       <c r="A81" s="151" t="inlineStr">
         <is>
-          <t>SBS 백종원의 골목식당</t>
+          <t>SBS 내 남자의 여자</t>
         </is>
       </c>
       <c r="B81" s="152" t="inlineStr">
@@ -39581,14 +39581,14 @@
       </c>
       <c r="C81" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB4200011RB</t>
+          <t>https://jmp2.uk/stvp-KRBB4200005CK</t>
         </is>
       </c>
     </row>
     <row r="82" ht="16" customHeight="1">
       <c r="A82" s="76" t="inlineStr">
         <is>
-          <t>SBS 불타는 청춘</t>
+          <t>SBS 런닝맨</t>
         </is>
       </c>
       <c r="B82" s="77" t="inlineStr">
@@ -39598,14 +39598,14 @@
       </c>
       <c r="C82" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB42000100V</t>
+          <t>https://jmp2.uk/stvp-KRBB4200002MM</t>
         </is>
       </c>
     </row>
     <row r="83" ht="16" customHeight="1">
       <c r="A83" s="151" t="inlineStr">
         <is>
-          <t>SBS 생활의 달인</t>
+          <t>SBS 모범택시</t>
         </is>
       </c>
       <c r="B83" s="152" t="inlineStr">
@@ -39615,14 +39615,14 @@
       </c>
       <c r="C83" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB4200018FT</t>
+          <t>https://jmp2.uk/stvp-KRBB420000180</t>
         </is>
       </c>
     </row>
     <row r="84" ht="16" customHeight="1">
       <c r="A84" s="76" t="inlineStr">
         <is>
-          <t>SBS 순간포착 세상에 이런일이</t>
+          <t>SBS 미운 우리 새끼</t>
         </is>
       </c>
       <c r="B84" s="77" t="inlineStr">
@@ -39632,14 +39632,14 @@
       </c>
       <c r="C84" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB4200013L5</t>
+          <t>https://jmp2.uk/stvp-KRBB4200003ZL</t>
         </is>
       </c>
     </row>
     <row r="85" ht="16" customHeight="1">
       <c r="A85" s="151" t="inlineStr">
         <is>
-          <t>SBS 순풍산부인과</t>
+          <t>SBS 백종원의 골목식당</t>
         </is>
       </c>
       <c r="B85" s="152" t="inlineStr">
@@ -39649,14 +39649,14 @@
       </c>
       <c r="C85" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB4200004RA</t>
+          <t>https://jmp2.uk/stvp-KRBB4200011RB</t>
         </is>
       </c>
     </row>
     <row r="86" ht="16" customHeight="1">
       <c r="A86" s="76" t="inlineStr">
         <is>
-          <t>SBS 신발 벗고 돌싱포맨</t>
+          <t>SBS 불타는 청춘</t>
         </is>
       </c>
       <c r="B86" s="77" t="inlineStr">
@@ -39666,14 +39666,14 @@
       </c>
       <c r="C86" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB4200008PR</t>
+          <t>https://jmp2.uk/stvp-KRBB42000100V</t>
         </is>
       </c>
     </row>
     <row r="87" ht="16" customHeight="1">
       <c r="A87" s="151" t="inlineStr">
         <is>
-          <t>SBS 야인시대</t>
+          <t>SBS 생활의 달인</t>
         </is>
       </c>
       <c r="B87" s="152" t="inlineStr">
@@ -39683,14 +39683,14 @@
       </c>
       <c r="C87" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB42000061Z</t>
+          <t>https://jmp2.uk/stvp-KRBB4200018FT</t>
         </is>
       </c>
     </row>
     <row r="88" ht="16" customHeight="1">
       <c r="A88" s="76" t="inlineStr">
         <is>
-          <t>SBS 올인</t>
+          <t>SBS 순간포착 세상에 이런일이</t>
         </is>
       </c>
       <c r="B88" s="77" t="inlineStr">
@@ -39700,14 +39700,14 @@
       </c>
       <c r="C88" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB420001572</t>
+          <t>https://jmp2.uk/stvp-KRBB4200013L5</t>
         </is>
       </c>
     </row>
     <row r="89" ht="16" customHeight="1">
       <c r="A89" s="151" t="inlineStr">
         <is>
-          <t>SBS 정글의 법칙</t>
+          <t>SBS 순풍산부인과</t>
         </is>
       </c>
       <c r="B89" s="152" t="inlineStr">
@@ -39717,14 +39717,14 @@
       </c>
       <c r="C89" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB4200012PV</t>
+          <t>https://jmp2.uk/stvp-KRBB4200004RA</t>
         </is>
       </c>
     </row>
     <row r="90" ht="16" customHeight="1">
       <c r="A90" s="76" t="inlineStr">
         <is>
-          <t>SBS 패밀리가 떴다</t>
+          <t>SBS 신발 벗고 돌싱포맨</t>
         </is>
       </c>
       <c r="B90" s="77" t="inlineStr">
@@ -39734,14 +39734,14 @@
       </c>
       <c r="C90" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB4200014MY</t>
+          <t>https://jmp2.uk/stvp-KRBB4200008PR</t>
         </is>
       </c>
     </row>
     <row r="91" ht="16" customHeight="1">
       <c r="A91" s="151" t="inlineStr">
         <is>
-          <t>SMTOWN_8</t>
+          <t>SBS 야인시대</t>
         </is>
       </c>
       <c r="B91" s="152" t="inlineStr">
@@ -39751,14 +39751,14 @@
       </c>
       <c r="C91" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR10000027H</t>
+          <t>https://jmp2.uk/stvp-KRBB42000061Z</t>
         </is>
       </c>
     </row>
     <row r="92" ht="16" customHeight="1">
       <c r="A92" s="76" t="inlineStr">
         <is>
-          <t>TBS_Korea_1</t>
+          <t>SBS 올인</t>
         </is>
       </c>
       <c r="B92" s="77" t="inlineStr">
@@ -39768,14 +39768,14 @@
       </c>
       <c r="C92" s="78" t="inlineStr">
         <is>
-          <t>https://cdntv.tbs.seoul.kr/tbs/tbs_tv_web.smil/playlist.m3u8</t>
+          <t>https://jmp2.uk/stvp-KRBB420001572</t>
         </is>
       </c>
     </row>
     <row r="93" ht="16" customHeight="1">
       <c r="A93" s="151" t="inlineStr">
         <is>
-          <t>TV CHOSUN 식객 허영만의 백반기행</t>
+          <t>SBS 정글의 법칙</t>
         </is>
       </c>
       <c r="B93" s="152" t="inlineStr">
@@ -39785,14 +39785,14 @@
       </c>
       <c r="C93" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC3200008M6</t>
+          <t>https://jmp2.uk/stvp-KRBB4200012PV</t>
         </is>
       </c>
     </row>
     <row r="94" ht="16" customHeight="1">
       <c r="A94" s="76" t="inlineStr">
         <is>
-          <t>YTN</t>
+          <t>SBS 패밀리가 떴다</t>
         </is>
       </c>
       <c r="B94" s="77" t="inlineStr">
@@ -39802,14 +39802,14 @@
       </c>
       <c r="C94" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBD2400001XD</t>
+          <t>https://jmp2.uk/stvp-KRBB4200014MY</t>
         </is>
       </c>
     </row>
     <row r="95" ht="16" customHeight="1">
       <c r="A95" s="151" t="inlineStr">
         <is>
-          <t>arirangKorea</t>
+          <t>SBS新闻</t>
         </is>
       </c>
       <c r="B95" s="152" t="inlineStr">
@@ -39819,14 +39819,14 @@
       </c>
       <c r="C95" s="153" t="inlineStr">
         <is>
-          <t>https://amdlive-ch01-ctnd-com.akamaized.net/arirang_1ch/smil:arirang_1ch.smil/playlist.m3u8</t>
+          <t>https://www.youtube.com/embed/7R0p3-LOn8Q</t>
         </is>
       </c>
     </row>
     <row r="96" ht="16" customHeight="1">
       <c r="A96" s="76" t="inlineStr">
         <is>
-          <t>arirangKorea_1</t>
+          <t>SMTOWN_8</t>
         </is>
       </c>
       <c r="B96" s="77" t="inlineStr">
@@ -39836,14 +39836,14 @@
       </c>
       <c r="C96" s="78" t="inlineStr">
         <is>
-          <t>https://amdlive-ch01-ctnd-com.akamaized.net/arirang_1ch/smil:arirang_1ch.smil/chunklist_b2256000_sleng.m3u8</t>
+          <t>https://jmp2.uk/stvp-KR10000027H</t>
         </is>
       </c>
     </row>
     <row r="97" ht="16" customHeight="1">
       <c r="A97" s="151" t="inlineStr">
         <is>
-          <t>ch.핑크퐁</t>
+          <t>TBS_Korea_1</t>
         </is>
       </c>
       <c r="B97" s="152" t="inlineStr">
@@ -39853,14 +39853,14 @@
       </c>
       <c r="C97" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC32000126M</t>
+          <t>https://cdntv.tbs.seoul.kr/tbs/tbs_tv_web.smil/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="98" ht="16" customHeight="1">
       <c r="A98" s="76" t="inlineStr">
         <is>
-          <t>essential; by Bugs</t>
+          <t>TV CHOSUN 식객 허영만의 백반기행</t>
         </is>
       </c>
       <c r="B98" s="77" t="inlineStr">
@@ -39870,14 +39870,14 @@
       </c>
       <c r="C98" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR410000247</t>
+          <t>https://jmp2.uk/stvp-KRBC3200008M6</t>
         </is>
       </c>
     </row>
     <row r="99" ht="16" customHeight="1">
       <c r="A99" s="151" t="inlineStr">
         <is>
-          <t>iHQ 돈쭐내러 왔습니다</t>
+          <t>YTN</t>
         </is>
       </c>
       <c r="B99" s="152" t="inlineStr">
@@ -39887,14 +39887,14 @@
       </c>
       <c r="C99" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC4000002ME</t>
+          <t>https://jmp2.uk/stvp-KRBD2400001XD</t>
         </is>
       </c>
     </row>
     <row r="100" ht="16" customHeight="1">
       <c r="A100" s="76" t="inlineStr">
         <is>
-          <t>tvN Asia</t>
+          <t>YTN新闻</t>
         </is>
       </c>
       <c r="B100" s="77" t="inlineStr">
@@ -39904,14 +39904,14 @@
       </c>
       <c r="C100" s="78" t="inlineStr">
         <is>
-          <t>http://58.8.186.128:10005/bysid/2518</t>
+          <t>https://www.youtube.com/embed/6QZ_qc75ihU</t>
         </is>
       </c>
     </row>
     <row r="101" ht="16" customHeight="1">
       <c r="A101" s="151" t="inlineStr">
         <is>
-          <t>tvN 삼시세끼 고창편</t>
+          <t>arirangKorea</t>
         </is>
       </c>
       <c r="B101" s="152" t="inlineStr">
@@ -39921,14 +39921,14 @@
       </c>
       <c r="C101" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC3200030BO</t>
+          <t>https://amdlive-ch01-ctnd-com.akamaized.net/arirang_1ch/smil:arirang_1ch.smil/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="102" ht="16" customHeight="1">
       <c r="A102" s="76" t="inlineStr">
         <is>
-          <t>tvN_Korea</t>
+          <t>arirangKorea_1</t>
         </is>
       </c>
       <c r="B102" s="77" t="inlineStr">
@@ -39938,14 +39938,14 @@
       </c>
       <c r="C102" s="78" t="inlineStr">
         <is>
-          <t>https://d21dxaer0ypwk1.cloudfront.net/v1/master/3722c60a815c199d9c0ef36c5b73da68a62b09d1/cc-a6m2cy2rylsvo-ssai-prd/54ac8e25_eb5a_4f10_ba20_ffb254f0a16c/hls/playlist.m3u8</t>
+          <t>https://amdlive-ch01-ctnd-com.akamaized.net/arirang_1ch/smil:arirang_1ch.smil/chunklist_b2256000_sleng.m3u8</t>
         </is>
       </c>
     </row>
     <row r="103" ht="16" customHeight="1">
       <c r="A103" s="151" t="inlineStr">
         <is>
-          <t>体育电视台</t>
+          <t>ch.핑크퐁</t>
         </is>
       </c>
       <c r="B103" s="152" t="inlineStr">
@@ -39955,14 +39955,14 @@
       </c>
       <c r="C103" s="153" t="inlineStr">
         <is>
-          <t>https://live.koryocdn.org/sports/index.m3u8</t>
+          <t>https://jmp2.uk/stvp-KRBC32000126M</t>
         </is>
       </c>
     </row>
     <row r="104" ht="16" customHeight="1">
       <c r="A104" s="76" t="inlineStr">
         <is>
-          <t>朝鲜中央电视台</t>
+          <t>essential; by Bugs</t>
         </is>
       </c>
       <c r="B104" s="77" t="inlineStr">
@@ -39972,14 +39972,14 @@
       </c>
       <c r="C104" s="78" t="inlineStr">
         <is>
-          <t>https://live.koryocdn.org/kctv/index.m3u8</t>
+          <t>https://jmp2.uk/stvp-KR410000247</t>
         </is>
       </c>
     </row>
     <row r="105" ht="16" customHeight="1">
       <c r="A105" s="151" t="inlineStr">
         <is>
-          <t>龙南山电视台</t>
+          <t>iHQ 돈쭐내러 왔습니다</t>
         </is>
       </c>
       <c r="B105" s="152" t="inlineStr">
@@ -39989,14 +39989,14 @@
       </c>
       <c r="C105" s="153" t="inlineStr">
         <is>
-          <t>https://live.koryocdn.org/ryongnamsan/index.m3u8</t>
+          <t>https://jmp2.uk/stvp-KRBC4000002ME</t>
         </is>
       </c>
     </row>
     <row r="106" ht="16" customHeight="1">
       <c r="A106" s="76" t="inlineStr">
         <is>
-          <t>고독한 미식가</t>
+          <t>tvN Asia</t>
         </is>
       </c>
       <c r="B106" s="77" t="inlineStr">
@@ -40006,14 +40006,14 @@
       </c>
       <c r="C106" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC3500014ZH</t>
+          <t>http://58.8.186.128:10005/bysid/2518</t>
         </is>
       </c>
     </row>
     <row r="107" ht="16" customHeight="1">
       <c r="A107" s="151" t="inlineStr">
         <is>
-          <t>구필수는 없다</t>
+          <t>tvN 삼시세끼 고창편</t>
         </is>
       </c>
       <c r="B107" s="152" t="inlineStr">
@@ -40023,14 +40023,14 @@
       </c>
       <c r="C107" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR2000004DJ</t>
+          <t>https://jmp2.uk/stvp-KRBC3200030BO</t>
         </is>
       </c>
     </row>
     <row r="108" ht="16" customHeight="1">
       <c r="A108" s="76" t="inlineStr">
         <is>
-          <t>글로벌 뉴스 by LeadStory</t>
+          <t>tvN_Korea</t>
         </is>
       </c>
       <c r="B108" s="77" t="inlineStr">
@@ -40040,14 +40040,14 @@
       </c>
       <c r="C108" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBD3100006X4</t>
+          <t>https://d21dxaer0ypwk1.cloudfront.net/v1/master/3722c60a815c199d9c0ef36c5b73da68a62b09d1/cc-a6m2cy2rylsvo-ssai-prd/54ac8e25_eb5a_4f10_ba20_ffb254f0a16c/hls/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="109" ht="16" customHeight="1">
       <c r="A109" s="151" t="inlineStr">
         <is>
-          <t>나는 솔로</t>
+          <t>体育电视台</t>
         </is>
       </c>
       <c r="B109" s="152" t="inlineStr">
@@ -40057,14 +40057,14 @@
       </c>
       <c r="C109" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB4200009C3</t>
+          <t>https://live.koryocdn.org/sports/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="110" ht="16" customHeight="1">
       <c r="A110" s="76" t="inlineStr">
         <is>
-          <t>나미브</t>
+          <t>朝鲜中央电视台</t>
         </is>
       </c>
       <c r="B110" s="77" t="inlineStr">
@@ -40074,14 +40074,14 @@
       </c>
       <c r="C110" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR2000011GA</t>
+          <t>https://live.koryocdn.org/kctv/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="111" ht="16" customHeight="1">
       <c r="A111" s="151" t="inlineStr">
         <is>
-          <t>나의 해리에게</t>
+          <t>龙南山电视台</t>
         </is>
       </c>
       <c r="B111" s="152" t="inlineStr">
@@ -40091,14 +40091,14 @@
       </c>
       <c r="C111" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR2000010K7</t>
+          <t>https://live.koryocdn.org/ryongnamsan/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="112" ht="16" customHeight="1">
       <c r="A112" s="76" t="inlineStr">
         <is>
-          <t>낮에 뜨는 달</t>
+          <t>고독한 미식가</t>
         </is>
       </c>
       <c r="B112" s="77" t="inlineStr">
@@ -40108,14 +40108,14 @@
       </c>
       <c r="C112" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR2000009EC</t>
+          <t>https://jmp2.uk/stvp-KRBC3500014ZH</t>
         </is>
       </c>
     </row>
     <row r="113" ht="16" customHeight="1">
       <c r="A113" s="151" t="inlineStr">
         <is>
-          <t>라이딩 인생</t>
+          <t>구필수는 없다</t>
         </is>
       </c>
       <c r="B113" s="152" t="inlineStr">
@@ -40125,14 +40125,14 @@
       </c>
       <c r="C113" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR2000003T6</t>
+          <t>https://jmp2.uk/stvp-KR2000004DJ</t>
         </is>
       </c>
     </row>
     <row r="114" ht="16" customHeight="1">
       <c r="A114" s="76" t="inlineStr">
         <is>
-          <t>로보카폴리 TV</t>
+          <t>글로벌 뉴스 by LeadStory</t>
         </is>
       </c>
       <c r="B114" s="77" t="inlineStr">
@@ -40142,14 +40142,14 @@
       </c>
       <c r="C114" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC3500013VH</t>
+          <t>https://jmp2.uk/stvp-KRBD3100006X4</t>
         </is>
       </c>
     </row>
     <row r="115" ht="16" customHeight="1">
       <c r="A115" s="151" t="inlineStr">
         <is>
-          <t>맛있는 녀석들</t>
+          <t>나는 솔로</t>
         </is>
       </c>
       <c r="B115" s="152" t="inlineStr">
@@ -40159,14 +40159,14 @@
       </c>
       <c r="C115" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC3200007D1</t>
+          <t>https://jmp2.uk/stvp-KRBB4200009C3</t>
         </is>
       </c>
     </row>
     <row r="116" ht="16" customHeight="1">
       <c r="A116" s="76" t="inlineStr">
         <is>
-          <t>바오패밀리</t>
+          <t>나미브</t>
         </is>
       </c>
       <c r="B116" s="77" t="inlineStr">
@@ -40176,14 +40176,14 @@
       </c>
       <c r="C116" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR2900001RN</t>
+          <t>https://jmp2.uk/stvp-KR2000011GA</t>
         </is>
       </c>
     </row>
     <row r="117" ht="16" customHeight="1">
       <c r="A117" s="151" t="inlineStr">
         <is>
-          <t>베베핀</t>
+          <t>나의 해리에게</t>
         </is>
       </c>
       <c r="B117" s="152" t="inlineStr">
@@ -40193,14 +40193,14 @@
       </c>
       <c r="C117" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC3500020AF</t>
+          <t>https://jmp2.uk/stvp-KR2000010K7</t>
         </is>
       </c>
     </row>
     <row r="118" ht="16" customHeight="1">
       <c r="A118" s="76" t="inlineStr">
         <is>
-          <t>비보티비</t>
+          <t>낮에 뜨는 달</t>
         </is>
       </c>
       <c r="B118" s="77" t="inlineStr">
@@ -40210,14 +40210,14 @@
       </c>
       <c r="C118" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR1800002Q7</t>
+          <t>https://jmp2.uk/stvp-KR2000009EC</t>
         </is>
       </c>
     </row>
     <row r="119" ht="16" customHeight="1">
       <c r="A119" s="151" t="inlineStr">
         <is>
-          <t>빠니보틀</t>
+          <t>라이딩 인생</t>
         </is>
       </c>
       <c r="B119" s="152" t="inlineStr">
@@ -40227,14 +40227,14 @@
       </c>
       <c r="C119" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR140000508</t>
+          <t>https://jmp2.uk/stvp-KR2000003T6</t>
         </is>
       </c>
     </row>
     <row r="120" ht="16" customHeight="1">
       <c r="A120" s="76" t="inlineStr">
         <is>
-          <t>뽀요TV</t>
+          <t>로보카폴리 TV</t>
         </is>
       </c>
       <c r="B120" s="77" t="inlineStr">
@@ -40244,14 +40244,14 @@
       </c>
       <c r="C120" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR900001U5</t>
+          <t>https://jmp2.uk/stvp-KRBC3500013VH</t>
         </is>
       </c>
     </row>
     <row r="121" ht="16" customHeight="1">
       <c r="A121" s="151" t="inlineStr">
         <is>
-          <t>살롱드립</t>
+          <t>맛있는 녀석들</t>
         </is>
       </c>
       <c r="B121" s="152" t="inlineStr">
@@ -40261,14 +40261,14 @@
       </c>
       <c r="C121" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR4100001LW</t>
+          <t>https://jmp2.uk/stvp-KRBC3200007D1</t>
         </is>
       </c>
     </row>
     <row r="122" ht="16" customHeight="1">
       <c r="A122" s="76" t="inlineStr">
         <is>
-          <t>서울경제TV</t>
+          <t>바오패밀리</t>
         </is>
       </c>
       <c r="B122" s="77" t="inlineStr">
@@ -40278,14 +40278,14 @@
       </c>
       <c r="C122" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR7000044K</t>
+          <t>https://jmp2.uk/stvp-KR2900001RN</t>
         </is>
       </c>
     </row>
     <row r="123" ht="16" customHeight="1">
       <c r="A123" s="151" t="inlineStr">
         <is>
-          <t>스크린골프존</t>
+          <t>베베핀</t>
         </is>
       </c>
       <c r="B123" s="152" t="inlineStr">
@@ -40295,14 +40295,14 @@
       </c>
       <c r="C123" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR44000010Y</t>
+          <t>https://jmp2.uk/stvp-KRBC3500020AF</t>
         </is>
       </c>
     </row>
     <row r="124" ht="16" customHeight="1">
       <c r="A124" s="76" t="inlineStr">
         <is>
-          <t>신병 1 2 몰아보기</t>
+          <t>비보티비</t>
         </is>
       </c>
       <c r="B124" s="77" t="inlineStr">
@@ -40312,14 +40312,14 @@
       </c>
       <c r="C124" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR1200002QR</t>
+          <t>https://jmp2.uk/stvp-KR1800002Q7</t>
         </is>
       </c>
     </row>
     <row r="125" ht="16" customHeight="1">
       <c r="A125" s="151" t="inlineStr">
         <is>
-          <t>신병 3</t>
+          <t>빠니보틀</t>
         </is>
       </c>
       <c r="B125" s="152" t="inlineStr">
@@ -40329,14 +40329,14 @@
       </c>
       <c r="C125" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR2000007LI</t>
+          <t>https://jmp2.uk/stvp-KR140000508</t>
         </is>
       </c>
     </row>
     <row r="126" ht="16" customHeight="1">
       <c r="A126" s="76" t="inlineStr">
         <is>
-          <t>씨네21+</t>
+          <t>뽀요TV</t>
         </is>
       </c>
       <c r="B126" s="77" t="inlineStr">
@@ -40346,14 +40346,14 @@
       </c>
       <c r="C126" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBD26000011V</t>
+          <t>https://jmp2.uk/stvp-KR900001U5</t>
         </is>
       </c>
     </row>
     <row r="127" ht="16" customHeight="1">
       <c r="A127" s="151" t="inlineStr">
         <is>
-          <t>야한 사진관</t>
+          <t>살롱드립</t>
         </is>
       </c>
       <c r="B127" s="152" t="inlineStr">
@@ -40363,14 +40363,14 @@
       </c>
       <c r="C127" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR2000008LX</t>
+          <t>https://jmp2.uk/stvp-KR4100001LW</t>
         </is>
       </c>
     </row>
     <row r="128" ht="16" customHeight="1">
       <c r="A128" s="76" t="inlineStr">
         <is>
-          <t>요가소년</t>
+          <t>서울경제TV</t>
         </is>
       </c>
       <c r="B128" s="77" t="inlineStr">
@@ -40380,14 +40380,14 @@
       </c>
       <c r="C128" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR39000030H</t>
+          <t>https://jmp2.uk/stvp-KR7000044K</t>
         </is>
       </c>
     </row>
     <row r="129" ht="16" customHeight="1">
       <c r="A129" s="151" t="inlineStr">
         <is>
-          <t>용감한 형사들</t>
+          <t>스크린골프존</t>
         </is>
       </c>
       <c r="B129" s="152" t="inlineStr">
@@ -40397,14 +40397,14 @@
       </c>
       <c r="C129" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC3500015BN</t>
+          <t>https://jmp2.uk/stvp-KR44000010Y</t>
         </is>
       </c>
     </row>
     <row r="130" ht="16" customHeight="1">
       <c r="A130" s="76" t="inlineStr">
         <is>
-          <t>우리의식탁</t>
+          <t>신병 1 2 몰아보기</t>
         </is>
       </c>
       <c r="B130" s="77" t="inlineStr">
@@ -40414,14 +40414,14 @@
       </c>
       <c r="C130" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBD2200001QD</t>
+          <t>https://jmp2.uk/stvp-KR1200002QR</t>
         </is>
       </c>
     </row>
     <row r="131" ht="16" customHeight="1">
       <c r="A131" s="151" t="inlineStr">
         <is>
-          <t>유병재</t>
+          <t>신병 3</t>
         </is>
       </c>
       <c r="B131" s="152" t="inlineStr">
@@ -40431,14 +40431,14 @@
       </c>
       <c r="C131" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR1400009B8</t>
+          <t>https://jmp2.uk/stvp-KR2000007LI</t>
         </is>
       </c>
     </row>
     <row r="132" ht="16" customHeight="1">
       <c r="A132" s="76" t="inlineStr">
         <is>
-          <t>지구마불 세계여행</t>
+          <t>씨네21+</t>
         </is>
       </c>
       <c r="B132" s="77" t="inlineStr">
@@ -40448,14 +40448,14 @@
       </c>
       <c r="C132" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR400049VH</t>
+          <t>https://jmp2.uk/stvp-KRBD26000011V</t>
         </is>
       </c>
     </row>
     <row r="133" ht="16" customHeight="1">
       <c r="A133" s="151" t="inlineStr">
         <is>
-          <t>쯔양</t>
+          <t>야한 사진관</t>
         </is>
       </c>
       <c r="B133" s="152" t="inlineStr">
@@ -40465,14 +40465,14 @@
       </c>
       <c r="C133" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR5000002QW</t>
+          <t>https://jmp2.uk/stvp-KR2000008LX</t>
         </is>
       </c>
     </row>
     <row r="134" ht="16" customHeight="1">
       <c r="A134" s="76" t="inlineStr">
         <is>
-          <t>채널A 나만 믿고 따라와 도시어부</t>
+          <t>요가소년</t>
         </is>
       </c>
       <c r="B134" s="77" t="inlineStr">
@@ -40482,14 +40482,14 @@
       </c>
       <c r="C134" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC4100001LY</t>
+          <t>https://jmp2.uk/stvp-KR39000030H</t>
         </is>
       </c>
     </row>
     <row r="135" ht="16" customHeight="1">
       <c r="A135" s="151" t="inlineStr">
         <is>
-          <t>채널A 이제 만나러 갑니다</t>
+          <t>용감한 형사들</t>
         </is>
       </c>
       <c r="B135" s="152" t="inlineStr">
@@ -40499,14 +40499,14 @@
       </c>
       <c r="C135" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC4100005N5</t>
+          <t>https://jmp2.uk/stvp-KRBC3500015BN</t>
         </is>
       </c>
     </row>
     <row r="136" ht="16" customHeight="1">
       <c r="A136" s="76" t="inlineStr">
         <is>
-          <t>초록뱀미디어 K-STAR 골프</t>
+          <t>우리의식탁</t>
         </is>
       </c>
       <c r="B136" s="77" t="inlineStr">
@@ -40516,14 +40516,14 @@
       </c>
       <c r="C136" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB5000364M</t>
+          <t>https://jmp2.uk/stvp-KRBD2200001QD</t>
         </is>
       </c>
     </row>
     <row r="137" ht="16" customHeight="1">
       <c r="A137" s="151" t="inlineStr">
         <is>
-          <t>코코비TV</t>
+          <t>유병재</t>
         </is>
       </c>
       <c r="B137" s="152" t="inlineStr">
@@ -40533,14 +40533,14 @@
       </c>
       <c r="C137" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBB500035VF</t>
+          <t>https://jmp2.uk/stvp-KR1400009B8</t>
         </is>
       </c>
     </row>
     <row r="138" ht="16" customHeight="1">
       <c r="A138" s="76" t="inlineStr">
         <is>
-          <t>투니버스 명탐정 코난 (자막)</t>
+          <t>지구마불 세계여행</t>
         </is>
       </c>
       <c r="B138" s="77" t="inlineStr">
@@ -40550,14 +40550,14 @@
       </c>
       <c r="C138" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC32000200B</t>
+          <t>https://jmp2.uk/stvp-KR400049VH</t>
         </is>
       </c>
     </row>
     <row r="139" ht="16" customHeight="1">
       <c r="A139" s="151" t="inlineStr">
         <is>
-          <t>투니버스 짱구는 못말려</t>
+          <t>쯔양</t>
         </is>
       </c>
       <c r="B139" s="152" t="inlineStr">
@@ -40567,14 +40567,14 @@
       </c>
       <c r="C139" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR10000017U</t>
+          <t>https://jmp2.uk/stvp-KR5000002QW</t>
         </is>
       </c>
     </row>
     <row r="140" ht="16" customHeight="1">
       <c r="A140" s="76" t="inlineStr">
         <is>
-          <t>투니버스 흔한남매의 안흔한일기</t>
+          <t>채널A 나만 믿고 따라와 도시어부</t>
         </is>
       </c>
       <c r="B140" s="77" t="inlineStr">
@@ -40584,14 +40584,14 @@
       </c>
       <c r="C140" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRBC3200017JQ</t>
+          <t>https://jmp2.uk/stvp-KRBC4100001LY</t>
         </is>
       </c>
     </row>
     <row r="141" ht="16" customHeight="1">
       <c r="A141" s="151" t="inlineStr">
         <is>
-          <t>할명수</t>
+          <t>채널A 이제 만나러 갑니다</t>
         </is>
       </c>
       <c r="B141" s="152" t="inlineStr">
@@ -40601,14 +40601,14 @@
       </c>
       <c r="C141" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR480000234</t>
+          <t>https://jmp2.uk/stvp-KRBC4100005N5</t>
         </is>
       </c>
     </row>
     <row r="142" ht="16" customHeight="1">
       <c r="A142" s="76" t="inlineStr">
         <is>
-          <t>행복배틀</t>
+          <t>초록뱀미디어 K-STAR 골프</t>
         </is>
       </c>
       <c r="B142" s="77" t="inlineStr">
@@ -40618,14 +40618,14 @@
       </c>
       <c r="C142" s="78" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KR200000503</t>
+          <t>https://jmp2.uk/stvp-KRBB5000364M</t>
         </is>
       </c>
     </row>
     <row r="143" ht="16" customHeight="1">
       <c r="A143" s="151" t="inlineStr">
         <is>
-          <t>현대홈쇼핑+Shop</t>
+          <t>코코비TV</t>
         </is>
       </c>
       <c r="B143" s="152" t="inlineStr">
@@ -40635,22 +40635,124 @@
       </c>
       <c r="C143" s="153" t="inlineStr">
         <is>
-          <t>https://jmp2.uk/stvp-KRAH4602000A</t>
+          <t>https://jmp2.uk/stvp-KRBB500035VF</t>
         </is>
       </c>
     </row>
     <row r="144" ht="16" customHeight="1">
       <c r="A144" s="76" t="inlineStr">
         <is>
+          <t>투니버스 명탐정 코난 (자막)</t>
+        </is>
+      </c>
+      <c r="B144" s="77" t="inlineStr">
+        <is>
+          <t>韩国/朝鲜</t>
+        </is>
+      </c>
+      <c r="C144" s="78" t="inlineStr">
+        <is>
+          <t>https://jmp2.uk/stvp-KRBC32000200B</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="16" customHeight="1">
+      <c r="A145" s="151" t="inlineStr">
+        <is>
+          <t>투니버스 짱구는 못말려</t>
+        </is>
+      </c>
+      <c r="B145" s="152" t="inlineStr">
+        <is>
+          <t>韩国/朝鲜</t>
+        </is>
+      </c>
+      <c r="C145" s="153" t="inlineStr">
+        <is>
+          <t>https://jmp2.uk/stvp-KR10000017U</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="16" customHeight="1">
+      <c r="A146" s="76" t="inlineStr">
+        <is>
+          <t>투니버스 흔한남매의 안흔한일기</t>
+        </is>
+      </c>
+      <c r="B146" s="77" t="inlineStr">
+        <is>
+          <t>韩国/朝鲜</t>
+        </is>
+      </c>
+      <c r="C146" s="78" t="inlineStr">
+        <is>
+          <t>https://jmp2.uk/stvp-KRBC3200017JQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="16" customHeight="1">
+      <c r="A147" s="151" t="inlineStr">
+        <is>
+          <t>할명수</t>
+        </is>
+      </c>
+      <c r="B147" s="152" t="inlineStr">
+        <is>
+          <t>韩国/朝鲜</t>
+        </is>
+      </c>
+      <c r="C147" s="153" t="inlineStr">
+        <is>
+          <t>https://jmp2.uk/stvp-KR480000234</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="16" customHeight="1">
+      <c r="A148" s="76" t="inlineStr">
+        <is>
+          <t>행복배틀</t>
+        </is>
+      </c>
+      <c r="B148" s="77" t="inlineStr">
+        <is>
+          <t>韩国/朝鲜</t>
+        </is>
+      </c>
+      <c r="C148" s="78" t="inlineStr">
+        <is>
+          <t>https://jmp2.uk/stvp-KR200000503</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="16" customHeight="1">
+      <c r="A149" s="151" t="inlineStr">
+        <is>
+          <t>현대홈쇼핑+Shop</t>
+        </is>
+      </c>
+      <c r="B149" s="152" t="inlineStr">
+        <is>
+          <t>韩国/朝鲜</t>
+        </is>
+      </c>
+      <c r="C149" s="153" t="inlineStr">
+        <is>
+          <t>https://jmp2.uk/stvp-KRAH4602000A</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="16" customHeight="1">
+      <c r="A150" s="76" t="inlineStr">
+        <is>
           <t>힙으뜸</t>
         </is>
       </c>
-      <c r="B144" s="77" t="inlineStr">
+      <c r="B150" s="77" t="inlineStr">
         <is>
           <t>韩国/朝鲜</t>
         </is>
       </c>
-      <c r="C144" s="78" t="inlineStr">
+      <c r="C150" s="78" t="inlineStr">
         <is>
           <t>https://jmp2.uk/stvp-KR260000274</t>
         </is>

</xml_diff>

<commit_message>
fix: remove fake 2023 loop and test cards for CCTV-13/14, promote genuine 1080P live stream to Line 1
</commit_message>
<xml_diff>
--- a/channels_overview.xlsx
+++ b/channels_overview.xlsx
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
@@ -1778,7 +1778,7 @@
         </is>
       </c>
       <c r="B31" s="70" t="n">
-        <v>3531</v>
+        <v>3528</v>
       </c>
       <c r="C31" s="70" t="n"/>
     </row>
@@ -13527,7 +13527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C104"/>
+  <dimension ref="A1:C101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -13538,7 +13538,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="71" t="inlineStr">
         <is>
-          <t>📺  📡 中国大陆 · 央视  —  共 102 条频道</t>
+          <t>📺  📡 中国大陆 · 央视  —  共 99 条频道</t>
         </is>
       </c>
     </row>
@@ -13963,14 +13963,14 @@
       </c>
       <c r="C26" s="78" t="inlineStr">
         <is>
-          <t>https://event.pull.hebtv.com/jishi/cp1.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0013_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="73" t="inlineStr">
         <is>
-          <t>CCTV-13</t>
+          <t>CCTV-13 新聞</t>
         </is>
       </c>
       <c r="B27" s="74" t="inlineStr">
@@ -13980,14 +13980,14 @@
       </c>
       <c r="C27" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0013_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv13hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="76" t="inlineStr">
         <is>
-          <t>CCTV-13 新聞</t>
+          <t>CCTV-14</t>
         </is>
       </c>
       <c r="B28" s="77" t="inlineStr">
@@ -13997,7 +13997,7 @@
       </c>
       <c r="C28" s="78" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv13hd.m3u8?auth=test20251009</t>
+          <t>http://74.91.26.218:82/live/cctv14hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -14014,7 +14014,7 @@
       </c>
       <c r="C29" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv14hd.m3u8</t>
+          <t>http://69.197.146.138:82/live/cctv14.m3u8</t>
         </is>
       </c>
     </row>
@@ -14031,7 +14031,7 @@
       </c>
       <c r="C30" s="78" t="inlineStr">
         <is>
-          <t>http://69.197.146.138:82/live/cctv14.m3u8</t>
+          <t>http://63.141.224.162:82/live/cctv14md.m3u8</t>
         </is>
       </c>
     </row>
@@ -14048,7 +14048,7 @@
       </c>
       <c r="C31" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.224.162:82/live/cctv14md.m3u8</t>
+          <t>http://124.228.160.112:9901/tsfile/live/0014_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -14065,14 +14065,14 @@
       </c>
       <c r="C32" s="78" t="inlineStr">
         <is>
-          <t>http://124.228.160.112:9901/tsfile/live/0014_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0014_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
       <c r="A33" s="73" t="inlineStr">
         <is>
-          <t>CCTV-14</t>
+          <t>CCTV-14少儿</t>
         </is>
       </c>
       <c r="B33" s="74" t="inlineStr">
@@ -14082,14 +14082,14 @@
       </c>
       <c r="C33" s="75" t="inlineStr">
         <is>
-          <t>https://event.pull.hebtv.com/jishi/cp2.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv14hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="A34" s="76" t="inlineStr">
         <is>
-          <t>CCTV-14</t>
+          <t>CCTV-14少儿</t>
         </is>
       </c>
       <c r="B34" s="77" t="inlineStr">
@@ -14099,14 +14099,14 @@
       </c>
       <c r="C34" s="78" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0014_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv14hd</t>
         </is>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="A35" s="73" t="inlineStr">
         <is>
-          <t>CCTV-14少儿</t>
+          <t>CCTV-15</t>
         </is>
       </c>
       <c r="B35" s="74" t="inlineStr">
@@ -14116,14 +14116,14 @@
       </c>
       <c r="C35" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv14hd.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv15hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="A36" s="76" t="inlineStr">
         <is>
-          <t>CCTV-14少儿</t>
+          <t>CCTV-15</t>
         </is>
       </c>
       <c r="B36" s="77" t="inlineStr">
@@ -14133,7 +14133,7 @@
       </c>
       <c r="C36" s="78" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv14hd</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv15hd</t>
         </is>
       </c>
     </row>
@@ -14150,7 +14150,7 @@
       </c>
       <c r="C37" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv15hd.m3u8</t>
+          <t>http://69.197.146.138:82/live/cctv15.m3u8</t>
         </is>
       </c>
     </row>
@@ -14167,7 +14167,7 @@
       </c>
       <c r="C38" s="78" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv15hd</t>
+          <t>http://63.141.224.162:82/live/cctv15md.m3u8</t>
         </is>
       </c>
     </row>
@@ -14184,7 +14184,7 @@
       </c>
       <c r="C39" s="75" t="inlineStr">
         <is>
-          <t>http://69.197.146.138:82/live/cctv15.m3u8</t>
+          <t>http://124.228.160.112:9901/tsfile/live/0015_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -14201,14 +14201,14 @@
       </c>
       <c r="C40" s="78" t="inlineStr">
         <is>
-          <t>http://63.141.224.162:82/live/cctv15md.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0015_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1">
       <c r="A41" s="73" t="inlineStr">
         <is>
-          <t>CCTV-15</t>
+          <t>CCTV-15 音樂</t>
         </is>
       </c>
       <c r="B41" s="74" t="inlineStr">
@@ -14218,14 +14218,14 @@
       </c>
       <c r="C41" s="75" t="inlineStr">
         <is>
-          <t>http://124.228.160.112:9901/tsfile/live/0015_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv15hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1">
       <c r="A42" s="76" t="inlineStr">
         <is>
-          <t>CCTV-15</t>
+          <t>CCTV-16</t>
         </is>
       </c>
       <c r="B42" s="77" t="inlineStr">
@@ -14235,14 +14235,14 @@
       </c>
       <c r="C42" s="78" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0015_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://69.197.146.138:82/live/cctv16.m3u8</t>
         </is>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1">
       <c r="A43" s="73" t="inlineStr">
         <is>
-          <t>CCTV-15 音樂</t>
+          <t>CCTV-16</t>
         </is>
       </c>
       <c r="B43" s="74" t="inlineStr">
@@ -14252,7 +14252,7 @@
       </c>
       <c r="C43" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv15hd.m3u8?auth=test20251009</t>
+          <t>http://113.57.140.161:10081/newlive/live/hls/17/live.m3u8</t>
         </is>
       </c>
     </row>
@@ -14269,7 +14269,7 @@
       </c>
       <c r="C44" s="78" t="inlineStr">
         <is>
-          <t>http://69.197.146.138:82/live/cctv16.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv16hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
@@ -14286,14 +14286,14 @@
       </c>
       <c r="C45" s="75" t="inlineStr">
         <is>
-          <t>http://113.57.140.161:10081/newlive/live/hls/17/live.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0016_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="46" ht="16" customHeight="1">
       <c r="A46" s="76" t="inlineStr">
         <is>
-          <t>CCTV-16</t>
+          <t>CCTV-17</t>
         </is>
       </c>
       <c r="B46" s="77" t="inlineStr">
@@ -14303,14 +14303,14 @@
       </c>
       <c r="C46" s="78" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv16hd.m3u8?auth=test20251009</t>
+          <t>http://74.91.26.218:82/live/cctv17hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="47" ht="16" customHeight="1">
       <c r="A47" s="73" t="inlineStr">
         <is>
-          <t>CCTV-16</t>
+          <t>CCTV-17</t>
         </is>
       </c>
       <c r="B47" s="74" t="inlineStr">
@@ -14320,7 +14320,7 @@
       </c>
       <c r="C47" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0016_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://69.197.146.138:82/live/cctv17.m3u8</t>
         </is>
       </c>
     </row>
@@ -14337,14 +14337,14 @@
       </c>
       <c r="C48" s="78" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv17hd.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0017_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1">
       <c r="A49" s="73" t="inlineStr">
         <is>
-          <t>CCTV-17</t>
+          <t>CCTV-17 農業農村</t>
         </is>
       </c>
       <c r="B49" s="74" t="inlineStr">
@@ -14354,14 +14354,14 @@
       </c>
       <c r="C49" s="75" t="inlineStr">
         <is>
-          <t>http://69.197.146.138:82/live/cctv17.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv17hd.m3u8?auth=test20251009</t>
         </is>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1">
       <c r="A50" s="76" t="inlineStr">
         <is>
-          <t>CCTV-17</t>
+          <t>CCTV-17 農業農村</t>
         </is>
       </c>
       <c r="B50" s="77" t="inlineStr">
@@ -14371,14 +14371,14 @@
       </c>
       <c r="C50" s="78" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0017_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv17hd</t>
         </is>
       </c>
     </row>
     <row r="51" ht="16" customHeight="1">
       <c r="A51" s="73" t="inlineStr">
         <is>
-          <t>CCTV-17 農業農村</t>
+          <t>CCTV-2</t>
         </is>
       </c>
       <c r="B51" s="74" t="inlineStr">
@@ -14388,14 +14388,14 @@
       </c>
       <c r="C51" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqbv/cctv17hd.m3u8?auth=test20251009</t>
+          <t>http://63.141.224.162:82/live/cctv2md.m3u8</t>
         </is>
       </c>
     </row>
     <row r="52" ht="16" customHeight="1">
       <c r="A52" s="76" t="inlineStr">
         <is>
-          <t>CCTV-17 農業農村</t>
+          <t>CCTV-2</t>
         </is>
       </c>
       <c r="B52" s="77" t="inlineStr">
@@ -14405,7 +14405,7 @@
       </c>
       <c r="C52" s="78" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv17hd</t>
+          <t>http://116.128.243.121:85/tsfile/live/0002_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -14422,14 +14422,14 @@
       </c>
       <c r="C53" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.224.162:82/live/cctv2md.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0002_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="54" ht="16" customHeight="1">
       <c r="A54" s="76" t="inlineStr">
         <is>
-          <t>CCTV-2</t>
+          <t>CCTV-3</t>
         </is>
       </c>
       <c r="B54" s="77" t="inlineStr">
@@ -14439,14 +14439,14 @@
       </c>
       <c r="C54" s="78" t="inlineStr">
         <is>
-          <t>http://116.128.243.121:85/tsfile/live/0002_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://63.141.224.162:82/live/cctv3md.m3u8</t>
         </is>
       </c>
     </row>
     <row r="55" ht="16" customHeight="1">
       <c r="A55" s="73" t="inlineStr">
         <is>
-          <t>CCTV-2</t>
+          <t>CCTV-3</t>
         </is>
       </c>
       <c r="B55" s="74" t="inlineStr">
@@ -14456,14 +14456,14 @@
       </c>
       <c r="C55" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0002_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0003_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="56" ht="16" customHeight="1">
       <c r="A56" s="76" t="inlineStr">
         <is>
-          <t>CCTV-3</t>
+          <t>CCTV-4</t>
         </is>
       </c>
       <c r="B56" s="77" t="inlineStr">
@@ -14473,14 +14473,14 @@
       </c>
       <c r="C56" s="78" t="inlineStr">
         <is>
-          <t>http://63.141.224.162:82/live/cctv3md.m3u8</t>
+          <t>http://58.56.162.102:4466/newlive/live/hls/4/live.m3u8</t>
         </is>
       </c>
     </row>
     <row r="57" ht="16" customHeight="1">
       <c r="A57" s="73" t="inlineStr">
         <is>
-          <t>CCTV-3</t>
+          <t>CCTV-4</t>
         </is>
       </c>
       <c r="B57" s="74" t="inlineStr">
@@ -14490,14 +14490,14 @@
       </c>
       <c r="C57" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0003_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0004_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="58" ht="16" customHeight="1">
       <c r="A58" s="76" t="inlineStr">
         <is>
-          <t>CCTV-4</t>
+          <t>CCTV-5</t>
         </is>
       </c>
       <c r="B58" s="77" t="inlineStr">
@@ -14507,14 +14507,14 @@
       </c>
       <c r="C58" s="78" t="inlineStr">
         <is>
-          <t>http://58.56.162.102:4466/newlive/live/hls/4/live.m3u8</t>
+          <t>http://69.197.146.138:82/live/cctv5.m3u8</t>
         </is>
       </c>
     </row>
     <row r="59" ht="16" customHeight="1">
       <c r="A59" s="73" t="inlineStr">
         <is>
-          <t>CCTV-4</t>
+          <t>CCTV-5</t>
         </is>
       </c>
       <c r="B59" s="74" t="inlineStr">
@@ -14524,14 +14524,14 @@
       </c>
       <c r="C59" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0004_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0005_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="60" ht="16" customHeight="1">
       <c r="A60" s="76" t="inlineStr">
         <is>
-          <t>CCTV-5</t>
+          <t>CCTV-5+</t>
         </is>
       </c>
       <c r="B60" s="77" t="inlineStr">
@@ -14541,14 +14541,14 @@
       </c>
       <c r="C60" s="78" t="inlineStr">
         <is>
-          <t>http://69.197.146.138:82/live/cctv5.m3u8</t>
+          <t>http://69.197.146.138:82/live/cctv5p.m3u8</t>
         </is>
       </c>
     </row>
     <row r="61" ht="16" customHeight="1">
       <c r="A61" s="73" t="inlineStr">
         <is>
-          <t>CCTV-5</t>
+          <t>CCTV-5体育</t>
         </is>
       </c>
       <c r="B61" s="74" t="inlineStr">
@@ -14558,14 +14558,14 @@
       </c>
       <c r="C61" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0005_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://63.141.224.162:82/live/cctv5md.m3u8</t>
         </is>
       </c>
     </row>
     <row r="62" ht="16" customHeight="1">
       <c r="A62" s="76" t="inlineStr">
         <is>
-          <t>CCTV-5+</t>
+          <t>CCTV-6</t>
         </is>
       </c>
       <c r="B62" s="77" t="inlineStr">
@@ -14575,14 +14575,14 @@
       </c>
       <c r="C62" s="78" t="inlineStr">
         <is>
-          <t>http://69.197.146.138:82/live/cctv5p.m3u8</t>
+          <t>http://63.141.224.162:82/live/cctv6md.m3u8</t>
         </is>
       </c>
     </row>
     <row r="63" ht="16" customHeight="1">
       <c r="A63" s="73" t="inlineStr">
         <is>
-          <t>CCTV-5体育</t>
+          <t>CCTV-6</t>
         </is>
       </c>
       <c r="B63" s="74" t="inlineStr">
@@ -14592,7 +14592,7 @@
       </c>
       <c r="C63" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.224.162:82/live/cctv5md.m3u8</t>
+          <t>http://124.228.160.112:9901/tsfile/live/0006_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -14609,14 +14609,14 @@
       </c>
       <c r="C64" s="78" t="inlineStr">
         <is>
-          <t>http://63.141.224.162:82/live/cctv6md.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0006_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="65" ht="16" customHeight="1">
       <c r="A65" s="73" t="inlineStr">
         <is>
-          <t>CCTV-6</t>
+          <t>CCTV-6 電影</t>
         </is>
       </c>
       <c r="B65" s="74" t="inlineStr">
@@ -14626,14 +14626,14 @@
       </c>
       <c r="C65" s="75" t="inlineStr">
         <is>
-          <t>http://124.228.160.112:9901/tsfile/live/0006_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv6hd</t>
         </is>
       </c>
     </row>
     <row r="66" ht="16" customHeight="1">
       <c r="A66" s="76" t="inlineStr">
         <is>
-          <t>CCTV-6</t>
+          <t>CCTV-6 電影</t>
         </is>
       </c>
       <c r="B66" s="77" t="inlineStr">
@@ -14643,14 +14643,14 @@
       </c>
       <c r="C66" s="78" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0006_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://74.91.26.218:82/live/cctv6hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="67" ht="16" customHeight="1">
       <c r="A67" s="73" t="inlineStr">
         <is>
-          <t>CCTV-6 電影</t>
+          <t>CCTV-7</t>
         </is>
       </c>
       <c r="B67" s="74" t="inlineStr">
@@ -14660,14 +14660,14 @@
       </c>
       <c r="C67" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv6hd</t>
+          <t>http://124.228.160.112:9901/tsfile/live/0007_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="68" ht="16" customHeight="1">
       <c r="A68" s="76" t="inlineStr">
         <is>
-          <t>CCTV-6 電影</t>
+          <t>CCTV-7</t>
         </is>
       </c>
       <c r="B68" s="77" t="inlineStr">
@@ -14677,14 +14677,14 @@
       </c>
       <c r="C68" s="78" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv6hd.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0007_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="69" ht="16" customHeight="1">
       <c r="A69" s="73" t="inlineStr">
         <is>
-          <t>CCTV-7</t>
+          <t>CCTV-7 國防軍事</t>
         </is>
       </c>
       <c r="B69" s="74" t="inlineStr">
@@ -14694,14 +14694,14 @@
       </c>
       <c r="C69" s="75" t="inlineStr">
         <is>
-          <t>http://124.228.160.112:9901/tsfile/live/0007_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv7hd</t>
         </is>
       </c>
     </row>
     <row r="70" ht="16" customHeight="1">
       <c r="A70" s="76" t="inlineStr">
         <is>
-          <t>CCTV-7</t>
+          <t>CCTV-8</t>
         </is>
       </c>
       <c r="B70" s="77" t="inlineStr">
@@ -14711,14 +14711,14 @@
       </c>
       <c r="C70" s="78" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0007_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://124.228.160.112:9901/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="71" ht="16" customHeight="1">
       <c r="A71" s="73" t="inlineStr">
         <is>
-          <t>CCTV-7 國防軍事</t>
+          <t>CCTV-8</t>
         </is>
       </c>
       <c r="B71" s="74" t="inlineStr">
@@ -14728,7 +14728,7 @@
       </c>
       <c r="C71" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv7hd</t>
+          <t>http://63.141.224.162:82/live/cctv8md.m3u8</t>
         </is>
       </c>
     </row>
@@ -14745,7 +14745,7 @@
       </c>
       <c r="C72" s="78" t="inlineStr">
         <is>
-          <t>http://124.228.160.112:9901/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://183.10.180.81:9901/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -14762,14 +14762,14 @@
       </c>
       <c r="C73" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.224.162:82/live/cctv8md.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="74" ht="16" customHeight="1">
       <c r="A74" s="76" t="inlineStr">
         <is>
-          <t>CCTV-8</t>
+          <t>CCTV-9</t>
         </is>
       </c>
       <c r="B74" s="77" t="inlineStr">
@@ -14779,14 +14779,14 @@
       </c>
       <c r="C74" s="78" t="inlineStr">
         <is>
-          <t>http://183.10.180.81:9901/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://74.91.26.218:82/live/cctv9hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="75" ht="16" customHeight="1">
       <c r="A75" s="73" t="inlineStr">
         <is>
-          <t>CCTV-8</t>
+          <t>CCTV-9</t>
         </is>
       </c>
       <c r="B75" s="74" t="inlineStr">
@@ -14796,7 +14796,7 @@
       </c>
       <c r="C75" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://124.228.160.112:9901/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -14813,7 +14813,7 @@
       </c>
       <c r="C76" s="78" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv9hd.m3u8</t>
+          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=55def6afe55d212c4ebd9540907c9396</t>
         </is>
       </c>
     </row>
@@ -14830,7 +14830,7 @@
       </c>
       <c r="C77" s="75" t="inlineStr">
         <is>
-          <t>http://124.228.160.112:9901/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>https://v4-702cae17a28d6e4f0c0002bba021d934.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=04d0734a39c43ac7409c482c75ab83eb</t>
         </is>
       </c>
     </row>
@@ -14847,14 +14847,14 @@
       </c>
       <c r="C78" s="78" t="inlineStr">
         <is>
-          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=55def6afe55d212c4ebd9540907c9396</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="79" ht="16" customHeight="1">
       <c r="A79" s="73" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>CCTV-9 紀錄</t>
         </is>
       </c>
       <c r="B79" s="74" t="inlineStr">
@@ -14864,14 +14864,14 @@
       </c>
       <c r="C79" s="75" t="inlineStr">
         <is>
-          <t>https://v4-702cae17a28d6e4f0c0002bba021d934.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=04d0734a39c43ac7409c482c75ab83eb</t>
+          <t>https://xykt-fix.github.io/Y77.m3u8</t>
         </is>
       </c>
     </row>
     <row r="80" ht="16" customHeight="1">
       <c r="A80" s="76" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>CCTV-9_6</t>
         </is>
       </c>
       <c r="B80" s="77" t="inlineStr">
@@ -14881,14 +14881,14 @@
       </c>
       <c r="C80" s="78" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=db000b5568ff643131ea7d86610b09b7</t>
         </is>
       </c>
     </row>
     <row r="81" ht="16" customHeight="1">
       <c r="A81" s="73" t="inlineStr">
         <is>
-          <t>CCTV-9 紀錄</t>
+          <t>CCTV-9纪录</t>
         </is>
       </c>
       <c r="B81" s="74" t="inlineStr">
@@ -14898,14 +14898,14 @@
       </c>
       <c r="C81" s="75" t="inlineStr">
         <is>
-          <t>https://xykt-fix.github.io/Y77.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv9hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="82" ht="16" customHeight="1">
       <c r="A82" s="76" t="inlineStr">
         <is>
-          <t>CCTV-9_6</t>
+          <t>CCTV-9纪录</t>
         </is>
       </c>
       <c r="B82" s="77" t="inlineStr">
@@ -14915,14 +14915,14 @@
       </c>
       <c r="C82" s="78" t="inlineStr">
         <is>
-          <t>https://v4-e6b1c5baf4e240fe63adbf68dda23435.livehwc4.com/play.kankanlive.com/live/1698423397390920.m3u8?sub_m3u8=true&amp;edge_slice=true&amp;user_session_id=db000b5568ff643131ea7d86610b09b7</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv9hd</t>
         </is>
       </c>
     </row>
     <row r="83" ht="16" customHeight="1">
       <c r="A83" s="73" t="inlineStr">
         <is>
-          <t>CCTV-9纪录</t>
+          <t>CCTV-世界地理</t>
         </is>
       </c>
       <c r="B83" s="74" t="inlineStr">
@@ -14932,14 +14932,14 @@
       </c>
       <c r="C83" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv9hd.m3u8</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/sjdl.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="84" ht="16" customHeight="1">
       <c r="A84" s="76" t="inlineStr">
         <is>
-          <t>CCTV-9纪录</t>
+          <t>CCTV-央視檯球</t>
         </is>
       </c>
       <c r="B84" s="77" t="inlineStr">
@@ -14949,14 +14949,14 @@
       </c>
       <c r="C84" s="78" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv9hd</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/ystq.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="85" ht="16" customHeight="1">
       <c r="A85" s="73" t="inlineStr">
         <is>
-          <t>CCTV-世界地理</t>
+          <t>CCTV-懷舊劇場</t>
         </is>
       </c>
       <c r="B85" s="74" t="inlineStr">
@@ -14966,14 +14966,14 @@
       </c>
       <c r="C85" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/sjdl.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/hjjc.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="86" ht="16" customHeight="1">
       <c r="A86" s="76" t="inlineStr">
         <is>
-          <t>CCTV-央視檯球</t>
+          <t>CCTV-第一劇場</t>
         </is>
       </c>
       <c r="B86" s="77" t="inlineStr">
@@ -14983,14 +14983,14 @@
       </c>
       <c r="C86" s="78" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/ystq.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/dyjc.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="87" ht="16" customHeight="1">
       <c r="A87" s="73" t="inlineStr">
         <is>
-          <t>CCTV-懷舊劇場</t>
+          <t>CCTV-風雲劇場</t>
         </is>
       </c>
       <c r="B87" s="74" t="inlineStr">
@@ -15000,14 +15000,14 @@
       </c>
       <c r="C87" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/hjjc.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/fyjc.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="88" ht="16" customHeight="1">
       <c r="A88" s="76" t="inlineStr">
         <is>
-          <t>CCTV-第一劇場</t>
+          <t>CCTV-風雲足球</t>
         </is>
       </c>
       <c r="B88" s="77" t="inlineStr">
@@ -15017,14 +15017,14 @@
       </c>
       <c r="C88" s="78" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/dyjc.m3u8?auth=testpub</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/fyzq.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="89" ht="16" customHeight="1">
       <c r="A89" s="73" t="inlineStr">
         <is>
-          <t>CCTV-風雲劇場</t>
+          <t>CCTV16</t>
         </is>
       </c>
       <c r="B89" s="74" t="inlineStr">
@@ -15034,14 +15034,14 @@
       </c>
       <c r="C89" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/fyjc.m3u8?auth=testpub</t>
+          <t>http://gmxw.7766.org:808/hls/169/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="90" ht="16" customHeight="1">
       <c r="A90" s="76" t="inlineStr">
         <is>
-          <t>CCTV-風雲足球</t>
+          <t>CGTN记录</t>
         </is>
       </c>
       <c r="B90" s="77" t="inlineStr">
@@ -15051,14 +15051,14 @@
       </c>
       <c r="C90" s="78" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/fyzq.m3u8?auth=testpub</t>
+          <t>https://english-livetx.cgtn.com/hls/yypdjlctzb_hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="91" ht="16" customHeight="1">
       <c r="A91" s="73" t="inlineStr">
         <is>
-          <t>CCTV13</t>
+          <t>F1 TV</t>
         </is>
       </c>
       <c r="B91" s="74" t="inlineStr">
@@ -15068,14 +15068,14 @@
       </c>
       <c r="C91" s="75" t="inlineStr">
         <is>
-          <t>http://ali-m-l.cztv.com/channels/lantian/channel21/1080p.m3u8</t>
+          <t>https://amg12058-c15studio-amg12058c1-lg-us-5787.playouts.now.amagi.tv/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="92" ht="16" customHeight="1">
       <c r="A92" s="76" t="inlineStr">
         <is>
-          <t>CCTV16</t>
+          <t>PGA Tour_4</t>
         </is>
       </c>
       <c r="B92" s="77" t="inlineStr">
@@ -15085,14 +15085,14 @@
       </c>
       <c r="C92" s="78" t="inlineStr">
         <is>
-          <t>http://gmxw.7766.org:808/hls/169/index.m3u8</t>
+          <t>https://d11k1mnrgfposz.cloudfront.net/playlist.m3u8</t>
         </is>
       </c>
     </row>
     <row r="93" ht="16" customHeight="1">
       <c r="A93" s="73" t="inlineStr">
         <is>
-          <t>CGTN记录</t>
+          <t>世界地理</t>
         </is>
       </c>
       <c r="B93" s="74" t="inlineStr">
@@ -15102,14 +15102,14 @@
       </c>
       <c r="C93" s="75" t="inlineStr">
         <is>
-          <t>https://english-livetx.cgtn.com/hls/yypdjlctzb_hd.m3u8</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=sjdl</t>
         </is>
       </c>
     </row>
     <row r="94" ht="16" customHeight="1">
       <c r="A94" s="76" t="inlineStr">
         <is>
-          <t>F1 TV</t>
+          <t>兵器科技</t>
         </is>
       </c>
       <c r="B94" s="77" t="inlineStr">
@@ -15119,14 +15119,14 @@
       </c>
       <c r="C94" s="78" t="inlineStr">
         <is>
-          <t>https://amg12058-c15studio-amg12058c1-lg-us-5787.playouts.now.amagi.tv/playlist.m3u8</t>
+          <t>http://63.141.224.162:82/live/gfjs.m3u8</t>
         </is>
       </c>
     </row>
     <row r="95" ht="16" customHeight="1">
       <c r="A95" s="73" t="inlineStr">
         <is>
-          <t>PGA Tour_4</t>
+          <t>第一剧场</t>
         </is>
       </c>
       <c r="B95" s="74" t="inlineStr">
@@ -15136,14 +15136,14 @@
       </c>
       <c r="C95" s="75" t="inlineStr">
         <is>
-          <t>https://d11k1mnrgfposz.cloudfront.net/playlist.m3u8</t>
+          <t>http://183.10.180.81:9901/tsfile/live/1082_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="96" ht="16" customHeight="1">
       <c r="A96" s="76" t="inlineStr">
         <is>
-          <t>世界地理</t>
+          <t>韩国电影1</t>
         </is>
       </c>
       <c r="B96" s="77" t="inlineStr">
@@ -15153,14 +15153,14 @@
       </c>
       <c r="C96" s="78" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=sjdl</t>
+          <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=595</t>
         </is>
       </c>
     </row>
     <row r="97" ht="16" customHeight="1">
       <c r="A97" s="73" t="inlineStr">
         <is>
-          <t>兵器科技</t>
+          <t>韩国电影2</t>
         </is>
       </c>
       <c r="B97" s="74" t="inlineStr">
@@ -15170,14 +15170,14 @@
       </c>
       <c r="C97" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.224.162:82/live/gfjs.m3u8</t>
+          <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=743</t>
         </is>
       </c>
     </row>
     <row r="98" ht="16" customHeight="1">
       <c r="A98" s="76" t="inlineStr">
         <is>
-          <t>第一剧场</t>
+          <t>风云剧场</t>
         </is>
       </c>
       <c r="B98" s="77" t="inlineStr">
@@ -15187,14 +15187,14 @@
       </c>
       <c r="C98" s="78" t="inlineStr">
         <is>
-          <t>http://183.10.180.81:9901/tsfile/live/1082_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://183.10.180.81:9901/tsfile/live/1032_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="99" ht="16" customHeight="1">
       <c r="A99" s="73" t="inlineStr">
         <is>
-          <t>韩国电影1</t>
+          <t>风云足球</t>
         </is>
       </c>
       <c r="B99" s="74" t="inlineStr">
@@ -15204,14 +15204,14 @@
       </c>
       <c r="C99" s="75" t="inlineStr">
         <is>
-          <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=595</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyzq</t>
         </is>
       </c>
     </row>
     <row r="100" ht="16" customHeight="1">
       <c r="A100" s="76" t="inlineStr">
         <is>
-          <t>韩国电影2</t>
+          <t>风云足球</t>
         </is>
       </c>
       <c r="B100" s="77" t="inlineStr">
@@ -15221,14 +15221,14 @@
       </c>
       <c r="C100" s="78" t="inlineStr">
         <is>
-          <t>https://stream.ads.ottera.tv/playlist.m3u8?network_id=743</t>
+          <t>http://198.204.229.234:82/live/fyzq.m3u8</t>
         </is>
       </c>
     </row>
     <row r="101" ht="16" customHeight="1">
       <c r="A101" s="73" t="inlineStr">
         <is>
-          <t>风云剧场</t>
+          <t>风云音乐</t>
         </is>
       </c>
       <c r="B101" s="74" t="inlineStr">
@@ -15237,57 +15237,6 @@
         </is>
       </c>
       <c r="C101" s="75" t="inlineStr">
-        <is>
-          <t>http://183.10.180.81:9901/tsfile/live/1032_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="16" customHeight="1">
-      <c r="A102" s="76" t="inlineStr">
-        <is>
-          <t>风云足球</t>
-        </is>
-      </c>
-      <c r="B102" s="77" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C102" s="78" t="inlineStr">
-        <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyzq</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="16" customHeight="1">
-      <c r="A103" s="73" t="inlineStr">
-        <is>
-          <t>风云足球</t>
-        </is>
-      </c>
-      <c r="B103" s="74" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C103" s="75" t="inlineStr">
-        <is>
-          <t>http://198.204.229.234:82/live/fyzq.m3u8</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="16" customHeight="1">
-      <c r="A104" s="76" t="inlineStr">
-        <is>
-          <t>风云音乐</t>
-        </is>
-      </c>
-      <c r="B104" s="77" t="inlineStr">
-        <is>
-          <t>央视频道</t>
-        </is>
-      </c>
-      <c r="C104" s="78" t="inlineStr">
         <is>
           <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyyy</t>
         </is>

</xml_diff>

<commit_message>
fix: restore full channel database (3,640 channels), fix unpack bug and add safety circuit breaker
</commit_message>
<xml_diff>
--- a/channels_overview.xlsx
+++ b/channels_overview.xlsx
@@ -1358,7 +1358,7 @@
         </is>
       </c>
       <c r="B3" s="4" t="n">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
@@ -1778,7 +1778,7 @@
         </is>
       </c>
       <c r="B31" s="70" t="n">
-        <v>3637</v>
+        <v>3640</v>
       </c>
       <c r="C31" s="70" t="n"/>
     </row>
@@ -13561,7 +13561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C222"/>
+  <dimension ref="A1:C225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -13572,7 +13572,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="71" t="inlineStr">
         <is>
-          <t>📺  📡 中国大陆 · 央视  —  共 220 条频道</t>
+          <t>📺  📡 中国大陆 · 央视  —  共 223 条频道</t>
         </is>
       </c>
     </row>
@@ -15517,7 +15517,7 @@
     <row r="116" ht="16" customHeight="1">
       <c r="A116" s="76" t="inlineStr">
         <is>
-          <t>CCTV-4</t>
+          <t>CCTV-3</t>
         </is>
       </c>
       <c r="B116" s="77" t="inlineStr">
@@ -15527,7 +15527,7 @@
       </c>
       <c r="C116" s="78" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv4hd.m3u8</t>
+          <t>http://63.141.230.178/live/cctv3hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -15544,7 +15544,7 @@
       </c>
       <c r="C117" s="75" t="inlineStr">
         <is>
-          <t>https://dash2.antik.sk/live/test_cctv_tizen/playlist.m3u8</t>
+          <t>http://74.91.26.218:82/live/cctv4hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -15561,7 +15561,7 @@
       </c>
       <c r="C118" s="78" t="inlineStr">
         <is>
-          <t>http://58.56.162.102:4466/newlive/live/hls/4/live.m3u8</t>
+          <t>https://dash2.antik.sk/live/test_cctv_tizen/playlist.m3u8</t>
         </is>
       </c>
     </row>
@@ -15578,7 +15578,7 @@
       </c>
       <c r="C119" s="75" t="inlineStr">
         <is>
-          <t>http://hlszymgsplive.miguvideo.com:8080/wd_r2/cctv/cctv4hd/1500/index.m3u8?msisdn=96a6b6df9271086a17b458ab0d603209&amp;mdspid=&amp;spid=699004&amp;netType=0&amp;sid=5500346947&amp;pid=2028597139&amp;timestamp=20261003215026&amp;Channel_ID=0116_2600034600-99000-201600010010028&amp;ProgramID=631780421&amp;ParentNodeID=-99&amp;assertID=5500346947&amp;client_ip=39.103.188.159&amp;SecurityKey=20261003215026&amp;promotionId=&amp;mvid=5101064235&amp;mcid=500020&amp;playurlVersion=WX-A1-9.9.2-SNAPSHOT&amp;userid=&amp;jmhm=&amp;videocodec=h264&amp;appCode=miguvideo_android&amp;bean=mgspad&amp;tid=android&amp;conFee=0&amp;encrypt=a88ac09fd122652c2a27e41a9c719bee&amp;sv=10004&amp;ct=android</t>
+          <t>http://58.56.162.102:4466/newlive/live/hls/4/live.m3u8</t>
         </is>
       </c>
     </row>
@@ -15595,7 +15595,7 @@
       </c>
       <c r="C120" s="78" t="inlineStr">
         <is>
-          <t>https://php.jdshipin.com:2096/TVOD/iptv.php?id=cctv4</t>
+          <t>http://hlszymgsplive.miguvideo.com:8080/wd_r2/cctv/cctv4hd/1500/index.m3u8?msisdn=96a6b6df9271086a17b458ab0d603209&amp;mdspid=&amp;spid=699004&amp;netType=0&amp;sid=5500346947&amp;pid=2028597139&amp;timestamp=20261003215026&amp;Channel_ID=0116_2600034600-99000-201600010010028&amp;ProgramID=631780421&amp;ParentNodeID=-99&amp;assertID=5500346947&amp;client_ip=39.103.188.159&amp;SecurityKey=20261003215026&amp;promotionId=&amp;mvid=5101064235&amp;mcid=500020&amp;playurlVersion=WX-A1-9.9.2-SNAPSHOT&amp;userid=&amp;jmhm=&amp;videocodec=h264&amp;appCode=miguvideo_android&amp;bean=mgspad&amp;tid=android&amp;conFee=0&amp;encrypt=a88ac09fd122652c2a27e41a9c719bee&amp;sv=10004&amp;ct=android</t>
         </is>
       </c>
     </row>
@@ -15612,14 +15612,14 @@
       </c>
       <c r="C121" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0004_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>https://php.jdshipin.com:2096/TVOD/iptv.php?id=cctv4</t>
         </is>
       </c>
     </row>
     <row r="122" ht="16" customHeight="1">
       <c r="A122" s="76" t="inlineStr">
         <is>
-          <t>CCTV-5</t>
+          <t>CCTV-4</t>
         </is>
       </c>
       <c r="B122" s="77" t="inlineStr">
@@ -15629,7 +15629,7 @@
       </c>
       <c r="C122" s="78" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0005_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0004_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -15646,14 +15646,14 @@
       </c>
       <c r="C123" s="75" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0005_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0005_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="124" ht="16" customHeight="1">
       <c r="A124" s="76" t="inlineStr">
         <is>
-          <t>CCTV-5+体育赛事</t>
+          <t>CCTV-5</t>
         </is>
       </c>
       <c r="B124" s="77" t="inlineStr">
@@ -15663,7 +15663,7 @@
       </c>
       <c r="C124" s="78" t="inlineStr">
         <is>
-          <t>http://69.197.146.138:82/live/cctv5p.m3u8</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0005_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -15680,7 +15680,7 @@
       </c>
       <c r="C125" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.250.98:82/live/cctv5pmd.m3u8?jsbt=1791048687&amp;jsbk=38b776aaeaf35470605e78a3ded10b40</t>
+          <t>http://69.197.146.138:82/live/cctv5p.m3u8</t>
         </is>
       </c>
     </row>
@@ -15697,7 +15697,7 @@
       </c>
       <c r="C126" s="78" t="inlineStr">
         <is>
-          <t>http://192.187.98.98:82/live/cctv5pmd.m3u8?jsbt=1791045398&amp;jsbk=e93cf39b12fb7f6d99efe3f957d20cc2</t>
+          <t>http://63.141.250.98:82/live/cctv5pmd.m3u8?jsbt=1791048687&amp;jsbk=38b776aaeaf35470605e78a3ded10b40</t>
         </is>
       </c>
     </row>
@@ -15714,7 +15714,7 @@
       </c>
       <c r="C127" s="75" t="inlineStr">
         <is>
-          <t>http://192.187.98.98:82/live/cctv5pmd.m3u8?jsbt=1791044153&amp;jsbk=0e7e136134d815b33b5cefe12b6a9ef6</t>
+          <t>http://192.187.98.98:82/live/cctv5pmd.m3u8?jsbt=1791045398&amp;jsbk=e93cf39b12fb7f6d99efe3f957d20cc2</t>
         </is>
       </c>
     </row>
@@ -15731,7 +15731,7 @@
       </c>
       <c r="C128" s="78" t="inlineStr">
         <is>
-          <t>http://69.30.211.138:82/live/cctv5pmd.m3u8?jsbt=1791034563&amp;jsbk=dc03ad54b0f23a58c184b0c0c22f33c9</t>
+          <t>http://192.187.98.98:82/live/cctv5pmd.m3u8?jsbt=1791044153&amp;jsbk=0e7e136134d815b33b5cefe12b6a9ef6</t>
         </is>
       </c>
     </row>
@@ -15748,7 +15748,7 @@
       </c>
       <c r="C129" s="75" t="inlineStr">
         <is>
-          <t>http://69.30.211.138:82/live/cctv5pmd.m3u8?jsbt=1791032960&amp;jsbk=897e54a0840138796fec96258d124f01</t>
+          <t>http://69.30.211.138:82/live/cctv5pmd.m3u8?jsbt=1791034563&amp;jsbk=dc03ad54b0f23a58c184b0c0c22f33c9</t>
         </is>
       </c>
     </row>
@@ -15765,14 +15765,14 @@
       </c>
       <c r="C130" s="78" t="inlineStr">
         <is>
-          <t>http://63.141.250.98:82/live/cctv5pmd.m3u8?jsbt=1791031317&amp;jsbk=6527cb53d1dc4e82514c9ef8a695c9c0</t>
+          <t>http://69.30.211.138:82/live/cctv5pmd.m3u8?jsbt=1791032960&amp;jsbk=897e54a0840138796fec96258d124f01</t>
         </is>
       </c>
     </row>
     <row r="131" ht="16" customHeight="1">
       <c r="A131" s="73" t="inlineStr">
         <is>
-          <t>CCTV-5体育</t>
+          <t>CCTV-5+体育赛事</t>
         </is>
       </c>
       <c r="B131" s="74" t="inlineStr">
@@ -15782,7 +15782,7 @@
       </c>
       <c r="C131" s="75" t="inlineStr">
         <is>
-          <t>http://69.197.146.138:82/live/cctv5.m3u8</t>
+          <t>http://63.141.250.98:82/live/cctv5pmd.m3u8?jsbt=1791031317&amp;jsbk=6527cb53d1dc4e82514c9ef8a695c9c0</t>
         </is>
       </c>
     </row>
@@ -15799,7 +15799,7 @@
       </c>
       <c r="C132" s="78" t="inlineStr">
         <is>
-          <t>http://63.141.224.162:82/live/cctv5md.m3u8</t>
+          <t>http://69.197.146.138:82/live/cctv5.m3u8</t>
         </is>
       </c>
     </row>
@@ -15816,14 +15816,14 @@
       </c>
       <c r="C133" s="75" t="inlineStr">
         <is>
-          <t>http://112.123.243.37:50085/tsfile/live/0005_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
+          <t>http://63.141.224.162:82/live/cctv5md.m3u8</t>
         </is>
       </c>
     </row>
     <row r="134" ht="16" customHeight="1">
       <c r="A134" s="76" t="inlineStr">
         <is>
-          <t>CCTV-6</t>
+          <t>CCTV-5体育</t>
         </is>
       </c>
       <c r="B134" s="77" t="inlineStr">
@@ -15833,7 +15833,7 @@
       </c>
       <c r="C134" s="78" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv6hd.m3u8</t>
+          <t>http://112.123.243.37:50085/tsfile/live/0005_1.m3u8?key=txiptv&amp;playlive=0&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -15850,7 +15850,7 @@
       </c>
       <c r="C135" s="75" t="inlineStr">
         <is>
-          <t>http://69.197.135.170:82/live/cctv6.m3u8?jsbt=1791048688&amp;jsbk=62cf991c021e2e8098a4e507c7cf157a&amp;from=zbdq5</t>
+          <t>http://74.91.26.218:82/live/cctv6hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -15867,7 +15867,7 @@
       </c>
       <c r="C136" s="78" t="inlineStr">
         <is>
-          <t>http://63.141.224.162:82/live/cctv6md.m3u8</t>
+          <t>http://69.197.135.170:82/live/cctv6.m3u8?jsbt=1791048688&amp;jsbk=62cf991c021e2e8098a4e507c7cf157a&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -15884,7 +15884,7 @@
       </c>
       <c r="C137" s="75" t="inlineStr">
         <is>
-          <t>http://hlszymgsplive.miguvideo.com:8080/wd_r2/2018/ocn/cctv6hd/2000/index.m3u8?msisdn=183854cd024b42f7f5c537c37ea90a58&amp;mdspid=&amp;spid=699004&amp;netType=0&amp;sid=5500212872&amp;pid=2028597139&amp;timestamp=20261003215028&amp;Channel_ID=0116_2600034600-99000-201600010010028&amp;ProgramID=624878396&amp;ParentNodeID=-99&amp;assertID=5500212872&amp;client_ip=39.103.182.111&amp;SecurityKey=20261003215028&amp;promotionId=&amp;mvid=5100001694&amp;mcid=500020&amp;playurlVersion=WX-A1-9.9.2-SNAPSHOT&amp;userid=&amp;jmhm=&amp;videocodec=h264&amp;appCode=miguvideo_android&amp;bean=mgspad&amp;tid=android&amp;conFee=0&amp;encrypt=eea58c03932d965d502e2a591171ea3c&amp;sv=10004&amp;ct=android</t>
+          <t>http://63.141.224.162:82/live/cctv6md.m3u8</t>
         </is>
       </c>
     </row>
@@ -15901,7 +15901,7 @@
       </c>
       <c r="C138" s="78" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv6hd</t>
+          <t>http://hlszymgsplive.miguvideo.com:8080/wd_r2/2018/ocn/cctv6hd/2000/index.m3u8?msisdn=183854cd024b42f7f5c537c37ea90a58&amp;mdspid=&amp;spid=699004&amp;netType=0&amp;sid=5500212872&amp;pid=2028597139&amp;timestamp=20261003215028&amp;Channel_ID=0116_2600034600-99000-201600010010028&amp;ProgramID=624878396&amp;ParentNodeID=-99&amp;assertID=5500212872&amp;client_ip=39.103.182.111&amp;SecurityKey=20261003215028&amp;promotionId=&amp;mvid=5100001694&amp;mcid=500020&amp;playurlVersion=WX-A1-9.9.2-SNAPSHOT&amp;userid=&amp;jmhm=&amp;videocodec=h264&amp;appCode=miguvideo_android&amp;bean=mgspad&amp;tid=android&amp;conFee=0&amp;encrypt=eea58c03932d965d502e2a591171ea3c&amp;sv=10004&amp;ct=android</t>
         </is>
       </c>
     </row>
@@ -15918,7 +15918,7 @@
       </c>
       <c r="C139" s="75" t="inlineStr">
         <is>
-          <t>https://php.jdshipin.com:2096/TVOD/iptv.php?id=cctv6</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv6hd</t>
         </is>
       </c>
     </row>
@@ -15935,7 +15935,7 @@
       </c>
       <c r="C140" s="78" t="inlineStr">
         <is>
-          <t>http://208.110.86.66:82/live/cctv6md.m3u8?jsbt=1791045398&amp;jsbk=86a298cfe60f6ca4eba16e76ee74355a&amp;from=zbdq5</t>
+          <t>https://php.jdshipin.com:2096/TVOD/iptv.php?id=cctv6</t>
         </is>
       </c>
     </row>
@@ -15952,7 +15952,7 @@
       </c>
       <c r="C141" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.226.98:82/live/cctv6md.m3u8?jsbt=1791034564&amp;jsbk=ef6e5ebcb1277670fa9650a3417b68c3&amp;from=zbdq5</t>
+          <t>http://208.110.86.66:82/live/cctv6md.m3u8?jsbt=1791045398&amp;jsbk=86a298cfe60f6ca4eba16e76ee74355a&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -15969,7 +15969,7 @@
       </c>
       <c r="C142" s="78" t="inlineStr">
         <is>
-          <t>http://208.110.86.66:82/live/cctv6md.m3u8?jsbt=1791031318&amp;jsbk=eb35d0276831f1e62b2f8c4bd852e4f4&amp;from=zbdq5</t>
+          <t>http://63.141.226.98:82/live/cctv6md.m3u8?jsbt=1791034564&amp;jsbk=ef6e5ebcb1277670fa9650a3417b68c3&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -15986,7 +15986,7 @@
       </c>
       <c r="C143" s="75" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0006_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://208.110.86.66:82/live/cctv6md.m3u8?jsbt=1791031318&amp;jsbk=eb35d0276831f1e62b2f8c4bd852e4f4&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -16003,14 +16003,14 @@
       </c>
       <c r="C144" s="78" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0006_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0006_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="145" ht="16" customHeight="1">
       <c r="A145" s="73" t="inlineStr">
         <is>
-          <t>CCTV-7</t>
+          <t>CCTV-6</t>
         </is>
       </c>
       <c r="B145" s="74" t="inlineStr">
@@ -16020,14 +16020,14 @@
       </c>
       <c r="C145" s="75" t="inlineStr">
         <is>
-          <t>http://69.197.146.146:82/live/cctv7.m3u8?jsbt=1791048688&amp;jsbk=85d32fed5be756ebb33cefebfae37aa6&amp;from=zbdq5</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0006_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="146" ht="16" customHeight="1">
       <c r="A146" s="76" t="inlineStr">
         <is>
-          <t>CCTV-7</t>
+          <t>CCTV-6</t>
         </is>
       </c>
       <c r="B146" s="77" t="inlineStr">
@@ -16037,7 +16037,7 @@
       </c>
       <c r="C146" s="78" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv7hd.m3u8</t>
+          <t>http://63.141.230.178/live/cctv6hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -16054,7 +16054,7 @@
       </c>
       <c r="C147" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv7hd</t>
+          <t>http://69.197.146.146:82/live/cctv7.m3u8?jsbt=1791048688&amp;jsbk=85d32fed5be756ebb33cefebfae37aa6&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -16071,7 +16071,7 @@
       </c>
       <c r="C148" s="78" t="inlineStr">
         <is>
-          <t>https://php.jdshipin.com:2096/TVOD/iptv.php?id=cctv7</t>
+          <t>http://74.91.26.218:82/live/cctv7hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -16088,7 +16088,7 @@
       </c>
       <c r="C149" s="75" t="inlineStr">
         <is>
-          <t>http://69.197.146.146:82/live/cctv7.m3u8?jsbt=1791045399&amp;jsbk=d90eecb551c0c222a334e749e3d36bc2&amp;from=zbdq5</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv7hd</t>
         </is>
       </c>
     </row>
@@ -16105,7 +16105,7 @@
       </c>
       <c r="C150" s="78" t="inlineStr">
         <is>
-          <t>http://69.197.146.146:82/live/cctv7.m3u8?jsbt=1791044154&amp;jsbk=3bf59475a8064a93034a7418892804e0&amp;from=zbdq5</t>
+          <t>https://php.jdshipin.com:2096/TVOD/iptv.php?id=cctv7</t>
         </is>
       </c>
     </row>
@@ -16122,7 +16122,7 @@
       </c>
       <c r="C151" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.226.98:82/live/cctv7md.m3u8?jsbt=1791034564&amp;jsbk=c802376f39d6ea564fa6491b5e6faf58&amp;from=zbdq5</t>
+          <t>http://69.197.146.146:82/live/cctv7.m3u8?jsbt=1791045399&amp;jsbk=d90eecb551c0c222a334e749e3d36bc2&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -16139,14 +16139,14 @@
       </c>
       <c r="C152" s="78" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0007_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://69.197.146.146:82/live/cctv7.m3u8?jsbt=1791044154&amp;jsbk=3bf59475a8064a93034a7418892804e0&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
     <row r="153" ht="16" customHeight="1">
       <c r="A153" s="73" t="inlineStr">
         <is>
-          <t>CCTV-8</t>
+          <t>CCTV-7</t>
         </is>
       </c>
       <c r="B153" s="74" t="inlineStr">
@@ -16156,14 +16156,14 @@
       </c>
       <c r="C153" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.224.162:82/live/cctv8md.m3u8</t>
+          <t>http://63.141.226.98:82/live/cctv7md.m3u8?jsbt=1791034564&amp;jsbk=c802376f39d6ea564fa6491b5e6faf58&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
     <row r="154" ht="16" customHeight="1">
       <c r="A154" s="76" t="inlineStr">
         <is>
-          <t>CCTV-8</t>
+          <t>CCTV-7</t>
         </is>
       </c>
       <c r="B154" s="77" t="inlineStr">
@@ -16173,7 +16173,7 @@
       </c>
       <c r="C154" s="78" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv8hd.m3u8</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0007_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -16190,7 +16190,7 @@
       </c>
       <c r="C155" s="75" t="inlineStr">
         <is>
-          <t>https://php.jdshipin.com:2096/TVOD/iptv.php?id=cctv8</t>
+          <t>http://63.141.224.162:82/live/cctv8md.m3u8</t>
         </is>
       </c>
     </row>
@@ -16207,7 +16207,7 @@
       </c>
       <c r="C156" s="78" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://74.91.26.218:82/live/cctv8hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -16224,14 +16224,14 @@
       </c>
       <c r="C157" s="75" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>https://php.jdshipin.com:2096/TVOD/iptv.php?id=cctv8</t>
         </is>
       </c>
     </row>
     <row r="158" ht="16" customHeight="1">
       <c r="A158" s="76" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>CCTV-8</t>
         </is>
       </c>
       <c r="B158" s="77" t="inlineStr">
@@ -16241,14 +16241,14 @@
       </c>
       <c r="C158" s="78" t="inlineStr">
         <is>
-          <t>http://69.197.146.146:82/live/cctv9.m3u8?jsbt=1791048687&amp;jsbk=cf73f6fd7d8f40ed454d7504449b85cf&amp;from=zbdq5</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="159" ht="16" customHeight="1">
       <c r="A159" s="73" t="inlineStr">
         <is>
-          <t>CCTV-9</t>
+          <t>CCTV-8</t>
         </is>
       </c>
       <c r="B159" s="74" t="inlineStr">
@@ -16258,7 +16258,7 @@
       </c>
       <c r="C159" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.26.218:82/live/cctv9hd.m3u8</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0008_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
@@ -16275,7 +16275,7 @@
       </c>
       <c r="C160" s="78" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv9hd</t>
+          <t>http://69.197.146.146:82/live/cctv9.m3u8?jsbt=1791048687&amp;jsbk=cf73f6fd7d8f40ed454d7504449b85cf&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -16292,7 +16292,7 @@
       </c>
       <c r="C161" s="75" t="inlineStr">
         <is>
-          <t>https://php.jdshipin.com:2096/TVOD/iptv.php?id=cctv9</t>
+          <t>http://74.91.26.218:82/live/cctv9hd.m3u8</t>
         </is>
       </c>
     </row>
@@ -16309,7 +16309,7 @@
       </c>
       <c r="C162" s="78" t="inlineStr">
         <is>
-          <t>https://xykt-fix.github.io/Y77.m3u8</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=cctv9hd</t>
         </is>
       </c>
     </row>
@@ -16326,7 +16326,7 @@
       </c>
       <c r="C163" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.250.98:82/live/cctv9md.m3u8?jsbt=1791045398&amp;jsbk=40981c992216c67c00fd323bfe8815d0&amp;from=zbdq5</t>
+          <t>https://php.jdshipin.com:2096/TVOD/iptv.php?id=cctv9</t>
         </is>
       </c>
     </row>
@@ -16343,7 +16343,7 @@
       </c>
       <c r="C164" s="78" t="inlineStr">
         <is>
-          <t>http://69.197.146.146:82/live/cctv9.m3u8?jsbt=1791044153&amp;jsbk=5543bcc0dd8f5031f445fd57cdd41b62&amp;from=zbdq5</t>
+          <t>https://xykt-fix.github.io/Y77.m3u8</t>
         </is>
       </c>
     </row>
@@ -16360,7 +16360,7 @@
       </c>
       <c r="C165" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.250.98:82/live/cctv9md.m3u8?jsbt=1791034563&amp;jsbk=9f08bfed3623e2c7da1aa361fb1c7f1b&amp;from=zbdq5</t>
+          <t>http://63.141.250.98:82/live/cctv9md.m3u8?jsbt=1791045398&amp;jsbk=40981c992216c67c00fd323bfe8815d0&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -16377,7 +16377,7 @@
       </c>
       <c r="C166" s="78" t="inlineStr">
         <is>
-          <t>http://69.197.146.146:82/live/cctv9.m3u8?jsbt=1791032961&amp;jsbk=cc6d20f93c382b92407aa1ebede930cc&amp;from=zbdq5</t>
+          <t>http://69.197.146.146:82/live/cctv9.m3u8?jsbt=1791044153&amp;jsbk=5543bcc0dd8f5031f445fd57cdd41b62&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -16394,7 +16394,7 @@
       </c>
       <c r="C167" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.250.98:82/live/cctv9md.m3u8?jsbt=1791031317&amp;jsbk=1f90f99109c2ef45dfc4c84d96693dc9&amp;from=zbdq5</t>
+          <t>http://63.141.250.98:82/live/cctv9md.m3u8?jsbt=1791034563&amp;jsbk=9f08bfed3623e2c7da1aa361fb1c7f1b&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -16411,7 +16411,7 @@
       </c>
       <c r="C168" s="78" t="inlineStr">
         <is>
-          <t>http://59.39.89.130:60901/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://69.197.146.146:82/live/cctv9.m3u8?jsbt=1791032961&amp;jsbk=cc6d20f93c382b92407aa1ebede930cc&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -16428,14 +16428,14 @@
       </c>
       <c r="C169" s="75" t="inlineStr">
         <is>
-          <t>http://222.169.85.8:9901/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
+          <t>http://63.141.250.98:82/live/cctv9md.m3u8?jsbt=1791031317&amp;jsbk=1f90f99109c2ef45dfc4c84d96693dc9&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
     <row r="170" ht="16" customHeight="1">
       <c r="A170" s="76" t="inlineStr">
         <is>
-          <t>CCTV中文国际-YT</t>
+          <t>CCTV-9</t>
         </is>
       </c>
       <c r="B170" s="77" t="inlineStr">
@@ -16445,14 +16445,14 @@
       </c>
       <c r="C170" s="78" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/embed/vNVp6bxkL1c</t>
+          <t>http://59.39.89.130:60901/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="171" ht="16" customHeight="1">
       <c r="A171" s="73" t="inlineStr">
         <is>
-          <t>世界地理</t>
+          <t>CCTV-9</t>
         </is>
       </c>
       <c r="B171" s="74" t="inlineStr">
@@ -16462,14 +16462,14 @@
       </c>
       <c r="C171" s="75" t="inlineStr">
         <is>
-          <t>http://69.30.196.146:82/live/sjdl.m3u8?jsbt=1791048688&amp;jsbk=034e7c09540d2c8f8a7db6262a3f22cd&amp;from=zbdq5</t>
+          <t>http://222.169.85.8:9901/tsfile/live/0009_1.m3u8?key=txiptv&amp;playlive=1&amp;authid=0</t>
         </is>
       </c>
     </row>
     <row r="172" ht="16" customHeight="1">
       <c r="A172" s="76" t="inlineStr">
         <is>
-          <t>世界地理</t>
+          <t>CCTV-9</t>
         </is>
       </c>
       <c r="B172" s="77" t="inlineStr">
@@ -16479,14 +16479,14 @@
       </c>
       <c r="C172" s="78" t="inlineStr">
         <is>
-          <t>http://69.30.254.58:82/live/sjdl.m3u8?jsbt=1791048688&amp;jsbk=2fd7e309d4c987fb250dfa4c0659f295</t>
+          <t>http://63.141.230.178/live/cctv9hd.m3u8</t>
         </is>
       </c>
     </row>
     <row r="173" ht="16" customHeight="1">
       <c r="A173" s="73" t="inlineStr">
         <is>
-          <t>世界地理</t>
+          <t>CCTV中文国际-YT</t>
         </is>
       </c>
       <c r="B173" s="74" t="inlineStr">
@@ -16496,7 +16496,7 @@
       </c>
       <c r="C173" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=sjdl</t>
+          <t>https://www.youtube.com/embed/vNVp6bxkL1c</t>
         </is>
       </c>
     </row>
@@ -16513,7 +16513,7 @@
       </c>
       <c r="C174" s="78" t="inlineStr">
         <is>
-          <t>http://69.30.254.58:82/live/sjdl.m3u8?jsbt=1791045399&amp;jsbk=700f89c3bcec055abaa5d4c5b71a298b&amp;from=zbdq5</t>
+          <t>http://69.30.196.146:82/live/sjdl.m3u8?jsbt=1791048688&amp;jsbk=034e7c09540d2c8f8a7db6262a3f22cd&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -16530,7 +16530,7 @@
       </c>
       <c r="C175" s="75" t="inlineStr">
         <is>
-          <t>http://69.30.196.146:82/live/sjdl.m3u8?jsbt=1791045398&amp;jsbk=74c77ac1c7119556bd69fc59f79cfeaf</t>
+          <t>http://69.30.254.58:82/live/sjdl.m3u8?jsbt=1791048688&amp;jsbk=2fd7e309d4c987fb250dfa4c0659f295</t>
         </is>
       </c>
     </row>
@@ -16547,7 +16547,7 @@
       </c>
       <c r="C176" s="78" t="inlineStr">
         <is>
-          <t>http://69.30.254.58:82/live/sjdl.m3u8?jsbt=1791044154&amp;jsbk=5a17486dc1e7bbb9b2541f0b17eb53a4</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=sjdl</t>
         </is>
       </c>
     </row>
@@ -16564,7 +16564,7 @@
       </c>
       <c r="C177" s="75" t="inlineStr">
         <is>
-          <t>http://69.30.254.58:82/live/sjdl.m3u8?jsbt=1791044154&amp;jsbk=5a17486dc1e7bbb9b2541f0b17eb53a4&amp;from=zbdq5</t>
+          <t>http://69.30.254.58:82/live/sjdl.m3u8?jsbt=1791045399&amp;jsbk=700f89c3bcec055abaa5d4c5b71a298b&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -16581,7 +16581,7 @@
       </c>
       <c r="C178" s="78" t="inlineStr">
         <is>
-          <t>http://107.150.35.234:82/live/sjdl.m3u8?jsbt=1791034563&amp;jsbk=a95102b1592e258721cdc8990c054442</t>
+          <t>http://69.30.196.146:82/live/sjdl.m3u8?jsbt=1791045398&amp;jsbk=74c77ac1c7119556bd69fc59f79cfeaf</t>
         </is>
       </c>
     </row>
@@ -16598,14 +16598,14 @@
       </c>
       <c r="C179" s="75" t="inlineStr">
         <is>
-          <t>http://107.150.35.234:82/live/sjdl.m3u8?jsbt=1791032961&amp;jsbk=60314936f68f75e736ed045c0f40b6f4</t>
+          <t>http://69.30.254.58:82/live/sjdl.m3u8?jsbt=1791044154&amp;jsbk=5a17486dc1e7bbb9b2541f0b17eb53a4</t>
         </is>
       </c>
     </row>
     <row r="180" ht="16" customHeight="1">
       <c r="A180" s="76" t="inlineStr">
         <is>
-          <t>兵器科技</t>
+          <t>世界地理</t>
         </is>
       </c>
       <c r="B180" s="77" t="inlineStr">
@@ -16615,14 +16615,14 @@
       </c>
       <c r="C180" s="78" t="inlineStr">
         <is>
-          <t>http://63.141.224.162:82/live/gfjs.m3u8</t>
+          <t>http://69.30.254.58:82/live/sjdl.m3u8?jsbt=1791044154&amp;jsbk=5a17486dc1e7bbb9b2541f0b17eb53a4&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
     <row r="181" ht="16" customHeight="1">
       <c r="A181" s="73" t="inlineStr">
         <is>
-          <t>兵器科技</t>
+          <t>世界地理</t>
         </is>
       </c>
       <c r="B181" s="74" t="inlineStr">
@@ -16632,14 +16632,14 @@
       </c>
       <c r="C181" s="75" t="inlineStr">
         <is>
-          <t>http://69.30.211.138:82/live/gfjs.m3u8?jsbt=1791034564&amp;jsbk=b38d23bf4cad174fb91dedeb62c9b8f1</t>
+          <t>http://107.150.35.234:82/live/sjdl.m3u8?jsbt=1791034563&amp;jsbk=a95102b1592e258721cdc8990c054442</t>
         </is>
       </c>
     </row>
     <row r="182" ht="16" customHeight="1">
       <c r="A182" s="76" t="inlineStr">
         <is>
-          <t>兵器科技</t>
+          <t>世界地理</t>
         </is>
       </c>
       <c r="B182" s="77" t="inlineStr">
@@ -16649,7 +16649,7 @@
       </c>
       <c r="C182" s="78" t="inlineStr">
         <is>
-          <t>http://69.30.211.138:82/live/gfjs.m3u8?jsbt=1791032962&amp;jsbk=d7fbf0355f17ee529a9479208328ab49</t>
+          <t>http://107.150.35.234:82/live/sjdl.m3u8?jsbt=1791032961&amp;jsbk=60314936f68f75e736ed045c0f40b6f4</t>
         </is>
       </c>
     </row>
@@ -16666,7 +16666,7 @@
       </c>
       <c r="C183" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=gfjs</t>
+          <t>http://63.141.224.162:82/live/gfjs.m3u8</t>
         </is>
       </c>
     </row>
@@ -16683,14 +16683,14 @@
       </c>
       <c r="C184" s="78" t="inlineStr">
         <is>
-          <t>http://69.197.181.106:82/live/gfjs.m3u8?jsbt=1791031319&amp;jsbk=1ed11a0f0ab71f6a1b3e9e4f7ea2c8bf</t>
+          <t>http://69.30.211.138:82/live/gfjs.m3u8?jsbt=1791034564&amp;jsbk=b38d23bf4cad174fb91dedeb62c9b8f1</t>
         </is>
       </c>
     </row>
     <row r="185" ht="16" customHeight="1">
       <c r="A185" s="73" t="inlineStr">
         <is>
-          <t>冤狱风云</t>
+          <t>兵器科技</t>
         </is>
       </c>
       <c r="B185" s="74" t="inlineStr">
@@ -16700,14 +16700,14 @@
       </c>
       <c r="C185" s="75" t="inlineStr">
         <is>
-          <t>https://hn.bfvvs.com/play/QbYOAKOe/index.m3u8</t>
+          <t>http://69.30.211.138:82/live/gfjs.m3u8?jsbt=1791032962&amp;jsbk=d7fbf0355f17ee529a9479208328ab49</t>
         </is>
       </c>
     </row>
     <row r="186" ht="16" customHeight="1">
       <c r="A186" s="76" t="inlineStr">
         <is>
-          <t>卫生健康</t>
+          <t>兵器科技</t>
         </is>
       </c>
       <c r="B186" s="77" t="inlineStr">
@@ -16717,14 +16717,14 @@
       </c>
       <c r="C186" s="78" t="inlineStr">
         <is>
-          <t>http://198.204.233.138:82/live/wsjk.m3u8?jsbt=1791044154&amp;jsbk=fd170280befb249baddd19c632aa8d23</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=gfjs</t>
         </is>
       </c>
     </row>
     <row r="187" ht="16" customHeight="1">
       <c r="A187" s="73" t="inlineStr">
         <is>
-          <t>卫生健康</t>
+          <t>兵器科技</t>
         </is>
       </c>
       <c r="B187" s="74" t="inlineStr">
@@ -16734,14 +16734,14 @@
       </c>
       <c r="C187" s="75" t="inlineStr">
         <is>
-          <t>http://107.150.35.234:82/live/wsjk.m3u8?jsbt=1791034563&amp;jsbk=43ed69f621eb0588a8ae68913acd5db1</t>
+          <t>http://69.197.181.106:82/live/gfjs.m3u8?jsbt=1791031319&amp;jsbk=1ed11a0f0ab71f6a1b3e9e4f7ea2c8bf</t>
         </is>
       </c>
     </row>
     <row r="188" ht="16" customHeight="1">
       <c r="A188" s="76" t="inlineStr">
         <is>
-          <t>卫生健康</t>
+          <t>冤狱风云</t>
         </is>
       </c>
       <c r="B188" s="77" t="inlineStr">
@@ -16751,14 +16751,14 @@
       </c>
       <c r="C188" s="78" t="inlineStr">
         <is>
-          <t>http://107.150.35.234:82/live/wsjk.m3u8?jsbt=1791032961&amp;jsbk=fb2c50b3c629a3f948e4d3f2688df0fd</t>
+          <t>https://hn.bfvvs.com/play/QbYOAKOe/index.m3u8</t>
         </is>
       </c>
     </row>
     <row r="189" ht="16" customHeight="1">
       <c r="A189" s="73" t="inlineStr">
         <is>
-          <t>央视台球</t>
+          <t>卫生健康</t>
         </is>
       </c>
       <c r="B189" s="74" t="inlineStr">
@@ -16768,14 +16768,14 @@
       </c>
       <c r="C189" s="75" t="inlineStr">
         <is>
-          <t>http://199.168.97.90:82/live/ystq.m3u8?jsbt=1791048688&amp;jsbk=ec95e47f34604e34be690ba0e14483f0</t>
+          <t>http://198.204.233.138:82/live/wsjk.m3u8?jsbt=1791044154&amp;jsbk=fd170280befb249baddd19c632aa8d23</t>
         </is>
       </c>
     </row>
     <row r="190" ht="16" customHeight="1">
       <c r="A190" s="76" t="inlineStr">
         <is>
-          <t>央视台球</t>
+          <t>卫生健康</t>
         </is>
       </c>
       <c r="B190" s="77" t="inlineStr">
@@ -16785,14 +16785,14 @@
       </c>
       <c r="C190" s="78" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/ystq.m3u8?auth=testpub</t>
+          <t>http://107.150.35.234:82/live/wsjk.m3u8?jsbt=1791034563&amp;jsbk=43ed69f621eb0588a8ae68913acd5db1</t>
         </is>
       </c>
     </row>
     <row r="191" ht="16" customHeight="1">
       <c r="A191" s="73" t="inlineStr">
         <is>
-          <t>央视台球</t>
+          <t>卫生健康</t>
         </is>
       </c>
       <c r="B191" s="74" t="inlineStr">
@@ -16802,7 +16802,7 @@
       </c>
       <c r="C191" s="75" t="inlineStr">
         <is>
-          <t>http://199.168.97.90:82/live/ystq.m3u8?jsbt=1791044154&amp;jsbk=f19f45752d396fc29970def3f0719221</t>
+          <t>http://107.150.35.234:82/live/wsjk.m3u8?jsbt=1791032961&amp;jsbk=fb2c50b3c629a3f948e4d3f2688df0fd</t>
         </is>
       </c>
     </row>
@@ -16819,14 +16819,14 @@
       </c>
       <c r="C192" s="78" t="inlineStr">
         <is>
-          <t>http://199.168.97.90:82/live/ystq.m3u8?jsbt=1791031318&amp;jsbk=df41acf85277ed5ec2602b869e92943a</t>
+          <t>http://199.168.97.90:82/live/ystq.m3u8?jsbt=1791048688&amp;jsbk=ec95e47f34604e34be690ba0e14483f0</t>
         </is>
       </c>
     </row>
     <row r="193" ht="16" customHeight="1">
       <c r="A193" s="73" t="inlineStr">
         <is>
-          <t>央视精品</t>
+          <t>央视台球</t>
         </is>
       </c>
       <c r="B193" s="74" t="inlineStr">
@@ -16836,14 +16836,14 @@
       </c>
       <c r="C193" s="75" t="inlineStr">
         <is>
-          <t>http://69.30.254.58:82/live/ysjp.m3u8?jsbt=1791044154&amp;jsbk=f5a37c7e0ee5674205fb3e52ded86965</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/ystq.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="194" ht="16" customHeight="1">
       <c r="A194" s="76" t="inlineStr">
         <is>
-          <t>女性时尚</t>
+          <t>央视台球</t>
         </is>
       </c>
       <c r="B194" s="77" t="inlineStr">
@@ -16853,14 +16853,14 @@
       </c>
       <c r="C194" s="78" t="inlineStr">
         <is>
-          <t>http://69.197.181.106:82/live/nxss.m3u8?jsbt=1791031319&amp;jsbk=9c50b10bfd6f9cfb4b7d13f59aa48d02</t>
+          <t>http://199.168.97.90:82/live/ystq.m3u8?jsbt=1791044154&amp;jsbk=f19f45752d396fc29970def3f0719221</t>
         </is>
       </c>
     </row>
     <row r="195" ht="16" customHeight="1">
       <c r="A195" s="73" t="inlineStr">
         <is>
-          <t>怀旧剧场</t>
+          <t>央视台球</t>
         </is>
       </c>
       <c r="B195" s="74" t="inlineStr">
@@ -16870,14 +16870,14 @@
       </c>
       <c r="C195" s="75" t="inlineStr">
         <is>
-          <t>http://69.197.146.2:82/live/hjjc.m3u8?jsbt=1791048688&amp;jsbk=d723978b15def258f9e07c7707629f91</t>
+          <t>http://199.168.97.90:82/live/ystq.m3u8?jsbt=1791031318&amp;jsbk=df41acf85277ed5ec2602b869e92943a</t>
         </is>
       </c>
     </row>
     <row r="196" ht="16" customHeight="1">
       <c r="A196" s="76" t="inlineStr">
         <is>
-          <t>怀旧剧场</t>
+          <t>央视精品</t>
         </is>
       </c>
       <c r="B196" s="77" t="inlineStr">
@@ -16887,14 +16887,14 @@
       </c>
       <c r="C196" s="78" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/hjjc.m3u8?auth=testpub</t>
+          <t>http://69.30.254.58:82/live/ysjp.m3u8?jsbt=1791044154&amp;jsbk=f5a37c7e0ee5674205fb3e52ded86965</t>
         </is>
       </c>
     </row>
     <row r="197" ht="16" customHeight="1">
       <c r="A197" s="73" t="inlineStr">
         <is>
-          <t>怀旧剧场</t>
+          <t>女性时尚</t>
         </is>
       </c>
       <c r="B197" s="74" t="inlineStr">
@@ -16904,7 +16904,7 @@
       </c>
       <c r="C197" s="75" t="inlineStr">
         <is>
-          <t>http://69.197.146.2:82/live/hjjc.m3u8?jsbt=1791044154&amp;jsbk=2e1c72e9fbf0a5328bd040e82fc03358</t>
+          <t>http://69.197.181.106:82/live/nxss.m3u8?jsbt=1791031319&amp;jsbk=9c50b10bfd6f9cfb4b7d13f59aa48d02</t>
         </is>
       </c>
     </row>
@@ -16921,7 +16921,7 @@
       </c>
       <c r="C198" s="78" t="inlineStr">
         <is>
-          <t>http://69.30.242.162:82/live/hjjc.m3u8?jsbt=1791034564&amp;jsbk=fef4dee815770f273cd56a540beda4e2</t>
+          <t>http://69.197.146.2:82/live/hjjc.m3u8?jsbt=1791048688&amp;jsbk=d723978b15def258f9e07c7707629f91</t>
         </is>
       </c>
     </row>
@@ -16938,7 +16938,7 @@
       </c>
       <c r="C199" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.16.250:82/live/hjjc.m3u8?jsbt=1791032962&amp;jsbk=3b6c91810fa0d89b930a072363f43ab4</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/hjjc.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
@@ -16955,14 +16955,14 @@
       </c>
       <c r="C200" s="78" t="inlineStr">
         <is>
-          <t>http://74.91.16.250:82/live/hjjc.m3u8?jsbt=1791031319&amp;jsbk=4c8455468afd481130c30093621efabb</t>
+          <t>http://69.197.146.2:82/live/hjjc.m3u8?jsbt=1791044154&amp;jsbk=2e1c72e9fbf0a5328bd040e82fc03358</t>
         </is>
       </c>
     </row>
     <row r="201" ht="16" customHeight="1">
       <c r="A201" s="73" t="inlineStr">
         <is>
-          <t>电视指南</t>
+          <t>怀旧剧场</t>
         </is>
       </c>
       <c r="B201" s="74" t="inlineStr">
@@ -16972,14 +16972,14 @@
       </c>
       <c r="C201" s="75" t="inlineStr">
         <is>
-          <t>http://198.204.230.114:82/live/dszn.m3u8?jsbt=1791048689&amp;jsbk=3bc7ba3d1ed5638d3b5963ce380531fe&amp;from=zbdq5</t>
+          <t>http://69.30.242.162:82/live/hjjc.m3u8?jsbt=1791034564&amp;jsbk=fef4dee815770f273cd56a540beda4e2</t>
         </is>
       </c>
     </row>
     <row r="202" ht="16" customHeight="1">
       <c r="A202" s="76" t="inlineStr">
         <is>
-          <t>电视指南</t>
+          <t>怀旧剧场</t>
         </is>
       </c>
       <c r="B202" s="77" t="inlineStr">
@@ -16989,14 +16989,14 @@
       </c>
       <c r="C202" s="78" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=dszn</t>
+          <t>http://74.91.16.250:82/live/hjjc.m3u8?jsbt=1791032962&amp;jsbk=3b6c91810fa0d89b930a072363f43ab4</t>
         </is>
       </c>
     </row>
     <row r="203" ht="16" customHeight="1">
       <c r="A203" s="73" t="inlineStr">
         <is>
-          <t>电视指南</t>
+          <t>怀旧剧场</t>
         </is>
       </c>
       <c r="B203" s="74" t="inlineStr">
@@ -17006,14 +17006,14 @@
       </c>
       <c r="C203" s="75" t="inlineStr">
         <is>
-          <t>http://198.204.230.114:82/live/dszn.m3u8?jsbt=1791045399&amp;jsbk=6bbd0f5fbcab3b4ff0001c70bd3a58f5&amp;from=zbdq5</t>
+          <t>http://74.91.16.250:82/live/hjjc.m3u8?jsbt=1791031319&amp;jsbk=4c8455468afd481130c30093621efabb</t>
         </is>
       </c>
     </row>
     <row r="204" ht="16" customHeight="1">
       <c r="A204" s="76" t="inlineStr">
         <is>
-          <t>第一剧场</t>
+          <t>电视指南</t>
         </is>
       </c>
       <c r="B204" s="77" t="inlineStr">
@@ -17023,14 +17023,14 @@
       </c>
       <c r="C204" s="78" t="inlineStr">
         <is>
-          <t>http://107.150.55.138:82/live/dyjc.m3u8?jsbt=1791048688&amp;jsbk=6f6ffc2c74369a323b2059c5d182fa8f</t>
+          <t>http://198.204.230.114:82/live/dszn.m3u8?jsbt=1791048689&amp;jsbk=3bc7ba3d1ed5638d3b5963ce380531fe&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
     <row r="205" ht="16" customHeight="1">
       <c r="A205" s="73" t="inlineStr">
         <is>
-          <t>第一剧场</t>
+          <t>电视指南</t>
         </is>
       </c>
       <c r="B205" s="74" t="inlineStr">
@@ -17040,14 +17040,14 @@
       </c>
       <c r="C205" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/dyjc.m3u8?auth=testpub</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=dszn</t>
         </is>
       </c>
     </row>
     <row r="206" ht="16" customHeight="1">
       <c r="A206" s="76" t="inlineStr">
         <is>
-          <t>第一剧场</t>
+          <t>电视指南</t>
         </is>
       </c>
       <c r="B206" s="77" t="inlineStr">
@@ -17057,7 +17057,7 @@
       </c>
       <c r="C206" s="78" t="inlineStr">
         <is>
-          <t>http://107.150.55.138:82/live/dyjc.m3u8?jsbt=1791034563&amp;jsbk=0f40b8b543b1452f46ca14d9fd0452da</t>
+          <t>http://198.204.230.114:82/live/dszn.m3u8?jsbt=1791045399&amp;jsbk=6bbd0f5fbcab3b4ff0001c70bd3a58f5&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -17074,14 +17074,14 @@
       </c>
       <c r="C207" s="75" t="inlineStr">
         <is>
-          <t>http://107.150.55.138:82/live/dyjc.m3u8?jsbt=1791032961&amp;jsbk=914880e126dc6795a30ab6f9f8bae38c</t>
+          <t>http://107.150.55.138:82/live/dyjc.m3u8?jsbt=1791048688&amp;jsbk=6f6ffc2c74369a323b2059c5d182fa8f</t>
         </is>
       </c>
     </row>
     <row r="208" ht="16" customHeight="1">
       <c r="A208" s="76" t="inlineStr">
         <is>
-          <t>风云剧场</t>
+          <t>第一剧场</t>
         </is>
       </c>
       <c r="B208" s="77" t="inlineStr">
@@ -17091,14 +17091,14 @@
       </c>
       <c r="C208" s="78" t="inlineStr">
         <is>
-          <t>http://107.150.55.138:82/live/fyjc.m3u8?jsbt=1791048688&amp;jsbk=ebb5b48b74b073784c61dfe18759227d</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/dyjc.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="209" ht="16" customHeight="1">
       <c r="A209" s="73" t="inlineStr">
         <is>
-          <t>风云剧场</t>
+          <t>第一剧场</t>
         </is>
       </c>
       <c r="B209" s="74" t="inlineStr">
@@ -17108,14 +17108,14 @@
       </c>
       <c r="C209" s="75" t="inlineStr">
         <is>
-          <t>http://38.75.136.137:98/gslb/dsdqpub/fyjc.m3u8?auth=testpub</t>
+          <t>http://107.150.55.138:82/live/dyjc.m3u8?jsbt=1791034563&amp;jsbk=0f40b8b543b1452f46ca14d9fd0452da</t>
         </is>
       </c>
     </row>
     <row r="210" ht="16" customHeight="1">
       <c r="A210" s="76" t="inlineStr">
         <is>
-          <t>风云剧场</t>
+          <t>第一剧场</t>
         </is>
       </c>
       <c r="B210" s="77" t="inlineStr">
@@ -17125,7 +17125,7 @@
       </c>
       <c r="C210" s="78" t="inlineStr">
         <is>
-          <t>http://69.197.146.2:82/live/fyjc.m3u8?jsbt=1791044154&amp;jsbk=9fcb774df15e6a7e27a680463f115359</t>
+          <t>http://107.150.55.138:82/live/dyjc.m3u8?jsbt=1791032961&amp;jsbk=914880e126dc6795a30ab6f9f8bae38c</t>
         </is>
       </c>
     </row>
@@ -17142,7 +17142,7 @@
       </c>
       <c r="C211" s="75" t="inlineStr">
         <is>
-          <t>http://107.150.55.138:82/live/fyjc.m3u8?jsbt=1791034563&amp;jsbk=55bc8aa9c7b0023f749e422cdce62570</t>
+          <t>http://107.150.55.138:82/live/fyjc.m3u8?jsbt=1791048688&amp;jsbk=ebb5b48b74b073784c61dfe18759227d</t>
         </is>
       </c>
     </row>
@@ -17159,14 +17159,14 @@
       </c>
       <c r="C212" s="78" t="inlineStr">
         <is>
-          <t>http://107.150.55.138:82/live/fyjc.m3u8?jsbt=1791032961&amp;jsbk=544c66cc6c1f2cc391c3141606e313fc</t>
+          <t>http://38.75.136.137:98/gslb/dsdqpub/fyjc.m3u8?auth=testpub</t>
         </is>
       </c>
     </row>
     <row r="213" ht="16" customHeight="1">
       <c r="A213" s="73" t="inlineStr">
         <is>
-          <t>风云足球</t>
+          <t>风云剧场</t>
         </is>
       </c>
       <c r="B213" s="74" t="inlineStr">
@@ -17176,14 +17176,14 @@
       </c>
       <c r="C213" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyzq</t>
+          <t>http://69.197.146.2:82/live/fyjc.m3u8?jsbt=1791044154&amp;jsbk=9fcb774df15e6a7e27a680463f115359</t>
         </is>
       </c>
     </row>
     <row r="214" ht="16" customHeight="1">
       <c r="A214" s="76" t="inlineStr">
         <is>
-          <t>风云足球</t>
+          <t>风云剧场</t>
         </is>
       </c>
       <c r="B214" s="77" t="inlineStr">
@@ -17193,14 +17193,14 @@
       </c>
       <c r="C214" s="78" t="inlineStr">
         <is>
-          <t>http://69.30.242.162:82/live/fyzq.m3u8?jsbt=1791034564&amp;jsbk=d4448278c1d2c19fad6e14a5afd6ea72</t>
+          <t>http://107.150.55.138:82/live/fyjc.m3u8?jsbt=1791034563&amp;jsbk=55bc8aa9c7b0023f749e422cdce62570</t>
         </is>
       </c>
     </row>
     <row r="215" ht="16" customHeight="1">
       <c r="A215" s="73" t="inlineStr">
         <is>
-          <t>风云足球</t>
+          <t>风云剧场</t>
         </is>
       </c>
       <c r="B215" s="74" t="inlineStr">
@@ -17210,14 +17210,14 @@
       </c>
       <c r="C215" s="75" t="inlineStr">
         <is>
-          <t>http://69.30.242.162:82/live/fyzq.m3u8?jsbt=1791034563&amp;jsbk=7d364433ff3671d40e5c49781c71ba7c&amp;from=zbdq5</t>
+          <t>http://107.150.55.138:82/live/fyjc.m3u8?jsbt=1791032961&amp;jsbk=544c66cc6c1f2cc391c3141606e313fc</t>
         </is>
       </c>
     </row>
     <row r="216" ht="16" customHeight="1">
       <c r="A216" s="76" t="inlineStr">
         <is>
-          <t>风云音乐</t>
+          <t>风云足球</t>
         </is>
       </c>
       <c r="B216" s="77" t="inlineStr">
@@ -17227,14 +17227,14 @@
       </c>
       <c r="C216" s="78" t="inlineStr">
         <is>
-          <t>http://74.91.16.250:82/live/fyyy.m3u8?jsbt=1791048689&amp;jsbk=68dbb4501055f709993509ec4ec24957&amp;from=zbdq5</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyzq</t>
         </is>
       </c>
     </row>
     <row r="217" ht="16" customHeight="1">
       <c r="A217" s="73" t="inlineStr">
         <is>
-          <t>风云音乐</t>
+          <t>风云足球</t>
         </is>
       </c>
       <c r="B217" s="74" t="inlineStr">
@@ -17244,14 +17244,14 @@
       </c>
       <c r="C217" s="75" t="inlineStr">
         <is>
-          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyyy</t>
+          <t>http://69.30.242.162:82/live/fyzq.m3u8?jsbt=1791034564&amp;jsbk=d4448278c1d2c19fad6e14a5afd6ea72</t>
         </is>
       </c>
     </row>
     <row r="218" ht="16" customHeight="1">
       <c r="A218" s="76" t="inlineStr">
         <is>
-          <t>风云音乐</t>
+          <t>风云足球</t>
         </is>
       </c>
       <c r="B218" s="77" t="inlineStr">
@@ -17261,7 +17261,7 @@
       </c>
       <c r="C218" s="78" t="inlineStr">
         <is>
-          <t>http://74.91.16.250:82/live/fyyy.m3u8?jsbt=1791045399&amp;jsbk=f4cea44dd471d4d5915adaab2866dac2&amp;from=zbdq5</t>
+          <t>http://69.30.242.162:82/live/fyzq.m3u8?jsbt=1791034563&amp;jsbk=7d364433ff3671d40e5c49781c71ba7c&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -17278,7 +17278,7 @@
       </c>
       <c r="C219" s="75" t="inlineStr">
         <is>
-          <t>http://69.30.242.162:82/live/fyyy.m3u8?jsbt=1791034564&amp;jsbk=175ec4b519361417d284cbfc58f73e23</t>
+          <t>http://74.91.16.250:82/live/fyyy.m3u8?jsbt=1791048689&amp;jsbk=68dbb4501055f709993509ec4ec24957&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -17295,7 +17295,7 @@
       </c>
       <c r="C220" s="78" t="inlineStr">
         <is>
-          <t>http://69.30.242.162:82/live/fyyy.m3u8?jsbt=1791034563&amp;jsbk=e0cef423a65cc20d0d930128349ebf58&amp;from=zbdq5</t>
+          <t>http://63.141.230.178:82/gslb/zbdq5.m3u8?id=fyyy</t>
         </is>
       </c>
     </row>
@@ -17312,7 +17312,7 @@
       </c>
       <c r="C221" s="75" t="inlineStr">
         <is>
-          <t>http://74.91.16.250:82/live/fyyy.m3u8?jsbt=1791031318&amp;jsbk=5a1ee3211955d374fa596bc71df0bffb&amp;from=zbdq5</t>
+          <t>http://74.91.16.250:82/live/fyyy.m3u8?jsbt=1791045399&amp;jsbk=f4cea44dd471d4d5915adaab2866dac2&amp;from=zbdq5</t>
         </is>
       </c>
     </row>
@@ -17328,6 +17328,57 @@
         </is>
       </c>
       <c r="C222" s="78" t="inlineStr">
+        <is>
+          <t>http://69.30.242.162:82/live/fyyy.m3u8?jsbt=1791034564&amp;jsbk=175ec4b519361417d284cbfc58f73e23</t>
+        </is>
+      </c>
+    </row>
+    <row r="223" ht="16" customHeight="1">
+      <c r="A223" s="73" t="inlineStr">
+        <is>
+          <t>风云音乐</t>
+        </is>
+      </c>
+      <c r="B223" s="74" t="inlineStr">
+        <is>
+          <t>央视频道</t>
+        </is>
+      </c>
+      <c r="C223" s="75" t="inlineStr">
+        <is>
+          <t>http://69.30.242.162:82/live/fyyy.m3u8?jsbt=1791034563&amp;jsbk=e0cef423a65cc20d0d930128349ebf58&amp;from=zbdq5</t>
+        </is>
+      </c>
+    </row>
+    <row r="224" ht="16" customHeight="1">
+      <c r="A224" s="76" t="inlineStr">
+        <is>
+          <t>风云音乐</t>
+        </is>
+      </c>
+      <c r="B224" s="77" t="inlineStr">
+        <is>
+          <t>央视频道</t>
+        </is>
+      </c>
+      <c r="C224" s="78" t="inlineStr">
+        <is>
+          <t>http://74.91.16.250:82/live/fyyy.m3u8?jsbt=1791031318&amp;jsbk=5a1ee3211955d374fa596bc71df0bffb&amp;from=zbdq5</t>
+        </is>
+      </c>
+    </row>
+    <row r="225" ht="16" customHeight="1">
+      <c r="A225" s="73" t="inlineStr">
+        <is>
+          <t>风云音乐</t>
+        </is>
+      </c>
+      <c r="B225" s="74" t="inlineStr">
+        <is>
+          <t>央视频道</t>
+        </is>
+      </c>
+      <c r="C225" s="75" t="inlineStr">
         <is>
           <t>http://74.91.16.250:82/live/fyyy.m3u8?jsbt=1791031319&amp;jsbk=5c8e5e2fa98f51a39589da8a8f7937bb</t>
         </is>

</xml_diff>